<commit_message>
docs: atualiza planejamento e controle do projeto
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/INST360 - Planejamento e Controle do Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/INST360 - Planejamento e Controle do Projeto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiag\OneDrive\Documentos\GitHub\INST360\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FB21700-3B59-4ABF-B2CA-E62801300DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A967EC93-9336-4C19-87ED-FCD4293988F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -4738,7 +4738,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="308">
   <si>
     <t>Equipe</t>
   </si>
@@ -5200,14 +5200,6 @@
     <t>Plano de Contingência</t>
   </si>
   <si>
-    <t>Atrasar a entrega do sistema</t>
-  </si>
-  <si>
-    <t>1. Executar horas-extras
-2. Contratar mais pessoas
-3. Renegociar prazo final</t>
-  </si>
-  <si>
     <t>APF (Método de estimativa de tamanho de sistema)</t>
   </si>
   <si>
@@ -5696,6 +5688,69 @@
   <si>
     <t>37, 38, 39, 40, 45, 46, 47</t>
   </si>
+  <si>
+    <t>Não adoção da aplicação por parte dos envolvidos</t>
+  </si>
+  <si>
+    <t>Levantar necessidades reais dos colaboradores e da administração desde o início do projeto.</t>
+  </si>
+  <si>
+    <t>Validar protótipos e funcionalidades com os envolvidos durante as sprints</t>
+  </si>
+  <si>
+    <t>Ajustar funcionalidades, interface e fluxo da aplicação com base no feedback dos usuários</t>
+  </si>
+  <si>
+    <t>Dificuldade na definição e validação das regras de anonimato, aprovação e tratamento das postagens</t>
+  </si>
+  <si>
+    <t>Definir claramente as regras de negócio com a equipe e validar os fluxos antes da implementação</t>
+  </si>
+  <si>
+    <t>Revisar casos de uso, backlog e documentos de requisitos sempre que houver dúvida sobre o funcionamento do sistema.</t>
+  </si>
+  <si>
+    <t>Replanejar funcionalidades relacionadas ao fluxo de postagem e ajustar os casos de uso e regras de negócio.</t>
+  </si>
+  <si>
+    <t>Dificuldade no cumprimento do prazo, em razão da pouca experiência da equipe em desenvolvimento</t>
+  </si>
+  <si>
+    <t>Capacitar a equipe previamente nas tecnologias e ferramentas que serão utilizadas.</t>
+  </si>
+  <si>
+    <t>Dividir tarefas em partes menores, acompanhar o andamento semanalmente e priorizar entregas essenciais.</t>
+  </si>
+  <si>
+    <t>Reduzir escopo, redistribuir tarefas e renegociar datas internas da sprint</t>
+  </si>
+  <si>
+    <t>Solicitações inesperadas de requisitos por parte dos envolvidos</t>
+  </si>
+  <si>
+    <t>Formalizar e validar o escopo inicial com os envolvidos antes do início da construção</t>
+  </si>
+  <si>
+    <t>Registrar mudanças solicitadas e avaliar impacto antes de incluí-las no backlog.</t>
+  </si>
+  <si>
+    <t>Repriorizar backlog, mover itens para sprints futuras ou descartar alterações não essenciais.</t>
+  </si>
+  <si>
+    <t>Má gestão do tempo e da divisão de tarefas entre os integrantes da equipe.</t>
+  </si>
+  <si>
+    <t>Definir responsáveis, prazos e rotina de acompanhamento desde o início do projeto</t>
+  </si>
+  <si>
+    <t>Realizar reuniões semanais, revisar o plano de entregas e acompanhar o andamento das tarefas por sprint.</t>
+  </si>
+  <si>
+    <t>Redistribuir tarefas entre os membros e concentrar a equipe nas atividades prioritárias</t>
+  </si>
+  <si>
+    <t>11, 12, 13, 16, 17, 18, 21, 22, 29, 30, 31, 32</t>
+  </si>
 </sst>
 </file>
 
@@ -5707,9 +5762,9 @@
     <numFmt numFmtId="166" formatCode="d/m/yy"/>
     <numFmt numFmtId="167" formatCode="[$-416]0%"/>
     <numFmt numFmtId="168" formatCode="&quot; R$ &quot;#,##0.00&quot; &quot;;&quot;-R$ &quot;#,##0.00&quot; &quot;;&quot; R$ -&quot;#&quot; &quot;;@&quot; &quot;"/>
-    <numFmt numFmtId="170" formatCode="#,##0.0&quot; &quot;;&quot;-&quot;#,##0.0&quot; &quot;;&quot; -&quot;#&quot; &quot;;@&quot; &quot;"/>
-    <numFmt numFmtId="172" formatCode="#,##0.00&quot; &quot;;&quot;-&quot;#,##0.00&quot; &quot;;&quot; -&quot;#&quot; &quot;;@&quot; &quot;"/>
-    <numFmt numFmtId="173" formatCode="[$R$-416]&quot; &quot;#,##0.00;[Red]&quot;-&quot;[$R$-416]&quot; &quot;#,##0.00"/>
+    <numFmt numFmtId="169" formatCode="#,##0.0&quot; &quot;;&quot;-&quot;#,##0.0&quot; &quot;;&quot; -&quot;#&quot; &quot;;@&quot; &quot;"/>
+    <numFmt numFmtId="170" formatCode="#,##0.00&quot; &quot;;&quot;-&quot;#,##0.00&quot; &quot;;&quot; -&quot;#&quot; &quot;;@&quot; &quot;"/>
+    <numFmt numFmtId="171" formatCode="[$R$-416]&quot; &quot;#,##0.00;[Red]&quot;-&quot;[$R$-416]&quot; &quot;#,##0.00"/>
   </numFmts>
   <fonts count="43" x14ac:knownFonts="1">
     <font>
@@ -6270,7 +6325,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
@@ -6281,11 +6336,11 @@
       <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="173" fontId="8" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="168">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="10" applyProtection="1"/>
     <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6435,9 +6490,9 @@
     <xf numFmtId="164" fontId="19" fillId="0" borderId="8" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="170" fontId="23" fillId="0" borderId="8" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="169" fontId="23" fillId="0" borderId="8" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="10" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="170" fontId="23" fillId="0" borderId="8" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="169" fontId="23" fillId="0" borderId="8" xfId="10" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="10" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -6601,6 +6656,64 @@
     <xf numFmtId="164" fontId="38" fillId="3" borderId="1" xfId="16" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="12" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="13" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="39" fillId="16" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="40" fillId="16" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="3" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="5" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="15" borderId="11" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="17" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="17" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="9" xfId="17" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="9" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="10" applyFont="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="42" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="26" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
@@ -6620,46 +6733,39 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="13" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="21" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="30" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6675,6 +6781,21 @@
     <xf numFmtId="164" fontId="30" fillId="13" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="17" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6705,72 +6826,15 @@
     <xf numFmtId="164" fontId="28" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="12" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="13" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="13" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="39" fillId="16" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="40" fillId="16" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="3" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="5" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="15" borderId="11" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="17" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="17" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="9" xfId="17" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="9" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="10" applyFont="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="42" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="cf1" xfId="1" xr:uid="{2DC75580-7322-4F49-9CB7-8EEEECF7EC6C}"/>
@@ -8657,18 +8721,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="134" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="116"/>
-      <c r="C1" s="116"/>
+      <c r="B1" s="134"/>
+      <c r="C1" s="134"/>
     </row>
     <row r="2" spans="1:3" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="117" t="s">
-        <v>231</v>
-      </c>
-      <c r="B2" s="117"/>
-      <c r="C2" s="117"/>
+      <c r="A2" s="135" t="s">
+        <v>229</v>
+      </c>
+      <c r="B2" s="135"/>
+      <c r="C2" s="135"/>
     </row>
     <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -8686,10 +8750,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="C4" s="111" t="s">
         <v>222</v>
-      </c>
-      <c r="C4" s="111" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -8697,7 +8761,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -8706,10 +8770,10 @@
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C6" s="111" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -8717,10 +8781,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C7" s="111" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -8728,10 +8792,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C8" s="111" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -8739,10 +8803,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C9" s="111" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -8824,38 +8888,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="140" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="F1" s="118" t="s">
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="F1" s="141" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
+      <c r="G1" s="141"/>
+      <c r="H1" s="141"/>
+      <c r="I1" s="141"/>
+      <c r="J1" s="141"/>
+      <c r="K1" s="141"/>
+      <c r="L1" s="141"/>
     </row>
     <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="119" t="s">
+      <c r="A2" s="142" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="119"/>
-      <c r="C2" s="119"/>
-      <c r="D2" s="119"/>
-      <c r="F2" s="120" t="s">
+      <c r="B2" s="142"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="F2" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="120"/>
-      <c r="H2" s="120"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="120"/>
-      <c r="L2" s="120"/>
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
+      <c r="K2" s="143"/>
+      <c r="L2" s="143"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -8876,20 +8940,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="121" t="s">
+      <c r="H3" s="144" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="121"/>
-      <c r="J3" s="121"/>
-      <c r="K3" s="121"/>
-      <c r="L3" s="121"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="122" t="s">
+      <c r="A4" s="136" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="122"/>
-      <c r="C4" s="122"/>
+      <c r="B4" s="136"/>
+      <c r="C4" s="136"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -8931,19 +8995,19 @@
       <c r="F5" s="14">
         <v>1</v>
       </c>
-      <c r="G5" s="161" t="s">
-        <v>265</v>
-      </c>
-      <c r="H5" s="162">
+      <c r="G5" s="123" t="s">
+        <v>263</v>
+      </c>
+      <c r="H5" s="124">
         <v>8</v>
       </c>
-      <c r="I5" s="162">
+      <c r="I5" s="124">
         <v>1</v>
       </c>
-      <c r="J5" s="162">
+      <c r="J5" s="124">
         <v>10</v>
       </c>
-      <c r="K5" s="162">
+      <c r="K5" s="124">
         <v>3</v>
       </c>
       <c r="L5" s="15">
@@ -8967,19 +9031,19 @@
       <c r="F6" s="14">
         <v>2</v>
       </c>
-      <c r="G6" s="161" t="s">
-        <v>266</v>
-      </c>
-      <c r="H6" s="162">
+      <c r="G6" s="123" t="s">
+        <v>264</v>
+      </c>
+      <c r="H6" s="124">
         <v>7</v>
       </c>
-      <c r="I6" s="162">
+      <c r="I6" s="124">
         <v>1</v>
       </c>
-      <c r="J6" s="162">
+      <c r="J6" s="124">
         <v>4</v>
       </c>
-      <c r="K6" s="162">
+      <c r="K6" s="124">
         <v>3</v>
       </c>
       <c r="L6" s="15">
@@ -9003,19 +9067,19 @@
       <c r="F7" s="14">
         <v>3</v>
       </c>
-      <c r="G7" s="161" t="s">
-        <v>267</v>
-      </c>
-      <c r="H7" s="162">
+      <c r="G7" s="123" t="s">
+        <v>265</v>
+      </c>
+      <c r="H7" s="124">
         <v>9</v>
       </c>
-      <c r="I7" s="162">
+      <c r="I7" s="124">
         <v>2</v>
       </c>
-      <c r="J7" s="162">
+      <c r="J7" s="124">
         <v>8</v>
       </c>
-      <c r="K7" s="162">
+      <c r="K7" s="124">
         <v>4</v>
       </c>
       <c r="L7" s="15">
@@ -9039,19 +9103,19 @@
       <c r="F8" s="14">
         <v>4</v>
       </c>
-      <c r="G8" s="161" t="s">
-        <v>256</v>
-      </c>
-      <c r="H8" s="162">
+      <c r="G8" s="123" t="s">
+        <v>254</v>
+      </c>
+      <c r="H8" s="124">
         <v>10</v>
       </c>
-      <c r="I8" s="162">
+      <c r="I8" s="124">
         <v>2</v>
       </c>
-      <c r="J8" s="162">
+      <c r="J8" s="124">
         <v>5</v>
       </c>
-      <c r="K8" s="162">
+      <c r="K8" s="124">
         <v>5</v>
       </c>
       <c r="L8" s="15">
@@ -9075,19 +9139,19 @@
       <c r="F9" s="14">
         <v>5</v>
       </c>
-      <c r="G9" s="161" t="s">
-        <v>257</v>
-      </c>
-      <c r="H9" s="162">
+      <c r="G9" s="123" t="s">
+        <v>255</v>
+      </c>
+      <c r="H9" s="124">
         <v>10</v>
       </c>
-      <c r="I9" s="162">
+      <c r="I9" s="124">
         <v>1</v>
       </c>
-      <c r="J9" s="162">
+      <c r="J9" s="124">
         <v>4</v>
       </c>
-      <c r="K9" s="162">
+      <c r="K9" s="124">
         <v>4</v>
       </c>
       <c r="L9" s="15">
@@ -9111,19 +9175,19 @@
       <c r="F10" s="14">
         <v>6</v>
       </c>
-      <c r="G10" s="161" t="s">
-        <v>258</v>
-      </c>
-      <c r="H10" s="162">
+      <c r="G10" s="123" t="s">
+        <v>256</v>
+      </c>
+      <c r="H10" s="124">
         <v>7</v>
       </c>
-      <c r="I10" s="162">
+      <c r="I10" s="124">
         <v>2</v>
       </c>
-      <c r="J10" s="162">
+      <c r="J10" s="124">
         <v>3</v>
       </c>
-      <c r="K10" s="162">
+      <c r="K10" s="124">
         <v>3</v>
       </c>
       <c r="L10" s="15">
@@ -9132,11 +9196,11 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="122" t="s">
+      <c r="A11" s="136" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="122"/>
-      <c r="C11" s="122"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="136"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>62</v>
@@ -9144,19 +9208,19 @@
       <c r="F11" s="14">
         <v>7</v>
       </c>
-      <c r="G11" s="161" t="s">
-        <v>259</v>
-      </c>
-      <c r="H11" s="162">
+      <c r="G11" s="123" t="s">
+        <v>257</v>
+      </c>
+      <c r="H11" s="124">
         <v>9</v>
       </c>
-      <c r="I11" s="162">
+      <c r="I11" s="124">
         <v>1</v>
       </c>
-      <c r="J11" s="162">
+      <c r="J11" s="124">
         <v>8</v>
       </c>
-      <c r="K11" s="162">
+      <c r="K11" s="124">
         <v>3</v>
       </c>
       <c r="L11" s="15">
@@ -9180,19 +9244,19 @@
       <c r="F12" s="14">
         <v>8</v>
       </c>
-      <c r="G12" s="161" t="s">
-        <v>260</v>
-      </c>
-      <c r="H12" s="162">
+      <c r="G12" s="123" t="s">
+        <v>258</v>
+      </c>
+      <c r="H12" s="124">
         <v>8</v>
       </c>
-      <c r="I12" s="162">
+      <c r="I12" s="124">
         <v>1</v>
       </c>
-      <c r="J12" s="162">
+      <c r="J12" s="124">
         <v>8</v>
       </c>
-      <c r="K12" s="162">
+      <c r="K12" s="124">
         <v>3</v>
       </c>
       <c r="L12" s="15">
@@ -9216,19 +9280,19 @@
       <c r="F13" s="14">
         <v>9</v>
       </c>
-      <c r="G13" s="161" t="s">
-        <v>261</v>
-      </c>
-      <c r="H13" s="162">
+      <c r="G13" s="123" t="s">
+        <v>259</v>
+      </c>
+      <c r="H13" s="124">
         <v>9</v>
       </c>
-      <c r="I13" s="162">
+      <c r="I13" s="124">
         <v>2</v>
       </c>
-      <c r="J13" s="162">
+      <c r="J13" s="124">
         <v>7</v>
       </c>
-      <c r="K13" s="162">
+      <c r="K13" s="124">
         <v>4</v>
       </c>
       <c r="L13" s="15">
@@ -9252,19 +9316,19 @@
       <c r="F14" s="14">
         <v>10</v>
       </c>
-      <c r="G14" s="161" t="s">
-        <v>262</v>
-      </c>
-      <c r="H14" s="162">
+      <c r="G14" s="123" t="s">
+        <v>260</v>
+      </c>
+      <c r="H14" s="124">
         <v>8</v>
       </c>
-      <c r="I14" s="162">
+      <c r="I14" s="124">
         <v>2</v>
       </c>
-      <c r="J14" s="162">
+      <c r="J14" s="124">
         <v>8</v>
       </c>
-      <c r="K14" s="162">
+      <c r="K14" s="124">
         <v>4</v>
       </c>
       <c r="L14" s="15">
@@ -9279,8 +9343,8 @@
       <c r="B15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="155" t="s">
-        <v>225</v>
+      <c r="C15" s="117" t="s">
+        <v>223</v>
       </c>
       <c r="D15" s="13">
         <v>7</v>
@@ -9288,19 +9352,19 @@
       <c r="F15" s="14">
         <v>11</v>
       </c>
-      <c r="G15" s="161" t="s">
-        <v>263</v>
-      </c>
-      <c r="H15" s="162">
+      <c r="G15" s="123" t="s">
+        <v>261</v>
+      </c>
+      <c r="H15" s="124">
         <v>8</v>
       </c>
-      <c r="I15" s="162">
+      <c r="I15" s="124">
         <v>2</v>
       </c>
-      <c r="J15" s="162">
+      <c r="J15" s="124">
         <v>6</v>
       </c>
-      <c r="K15" s="162">
+      <c r="K15" s="124">
         <v>4</v>
       </c>
       <c r="L15" s="15">
@@ -9315,7 +9379,7 @@
       <c r="B16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="156" t="s">
+      <c r="C16" s="118" t="s">
         <v>35</v>
       </c>
       <c r="D16" s="13">
@@ -9324,19 +9388,19 @@
       <c r="F16" s="14">
         <v>12</v>
       </c>
-      <c r="G16" s="161" t="s">
-        <v>264</v>
-      </c>
-      <c r="H16" s="162">
+      <c r="G16" s="123" t="s">
+        <v>262</v>
+      </c>
+      <c r="H16" s="124">
         <v>6</v>
       </c>
-      <c r="I16" s="162">
+      <c r="I16" s="124">
         <v>3</v>
       </c>
-      <c r="J16" s="162">
+      <c r="J16" s="124">
         <v>4</v>
       </c>
-      <c r="K16" s="162">
+      <c r="K16" s="124">
         <v>4</v>
       </c>
       <c r="L16" s="15">
@@ -9421,12 +9485,12 @@
       <c r="L20" s="17"/>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="122" t="s">
+      <c r="A21" s="136" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="122"/>
-      <c r="C21" s="149"/>
-      <c r="D21" s="150">
+      <c r="B21" s="136"/>
+      <c r="C21" s="137"/>
+      <c r="D21" s="113">
         <f>SUM(D12:D20)</f>
         <v>92</v>
       </c>
@@ -9435,13 +9499,13 @@
       <c r="A22" s="10">
         <v>16</v>
       </c>
-      <c r="B22" s="148" t="s">
+      <c r="B22" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="153" t="s">
+      <c r="C22" s="115" t="s">
         <v>32</v>
       </c>
-      <c r="D22" s="154">
+      <c r="D22" s="116">
         <v>4</v>
       </c>
     </row>
@@ -9449,13 +9513,13 @@
       <c r="A23" s="10">
         <v>17</v>
       </c>
-      <c r="B23" s="148" t="s">
+      <c r="B23" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="153" t="s">
-        <v>232</v>
-      </c>
-      <c r="D23" s="154">
+      <c r="C23" s="115" t="s">
+        <v>230</v>
+      </c>
+      <c r="D23" s="116">
         <v>4</v>
       </c>
     </row>
@@ -9463,13 +9527,13 @@
       <c r="A24" s="10">
         <v>18</v>
       </c>
-      <c r="B24" s="148" t="s">
+      <c r="B24" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="153" t="s">
-        <v>233</v>
-      </c>
-      <c r="D24" s="154">
+      <c r="C24" s="115" t="s">
+        <v>231</v>
+      </c>
+      <c r="D24" s="116">
         <v>12</v>
       </c>
     </row>
@@ -9477,13 +9541,13 @@
       <c r="A25" s="10">
         <v>19</v>
       </c>
-      <c r="B25" s="148" t="s">
+      <c r="B25" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="153" t="s">
-        <v>234</v>
-      </c>
-      <c r="D25" s="154">
+      <c r="C25" s="115" t="s">
+        <v>232</v>
+      </c>
+      <c r="D25" s="116">
         <v>4</v>
       </c>
     </row>
@@ -9491,13 +9555,13 @@
       <c r="A26" s="10">
         <v>20</v>
       </c>
-      <c r="B26" s="148" t="s">
+      <c r="B26" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C26" s="153" t="s">
-        <v>235</v>
-      </c>
-      <c r="D26" s="154">
+      <c r="C26" s="115" t="s">
+        <v>233</v>
+      </c>
+      <c r="D26" s="116">
         <v>10</v>
       </c>
     </row>
@@ -9505,13 +9569,13 @@
       <c r="A27" s="10">
         <v>21</v>
       </c>
-      <c r="B27" s="148" t="s">
+      <c r="B27" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="153" t="s">
-        <v>236</v>
-      </c>
-      <c r="D27" s="154">
+      <c r="C27" s="115" t="s">
+        <v>234</v>
+      </c>
+      <c r="D27" s="116">
         <v>4</v>
       </c>
     </row>
@@ -9519,13 +9583,13 @@
       <c r="A28" s="10">
         <v>22</v>
       </c>
-      <c r="B28" s="148" t="s">
+      <c r="B28" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C28" s="153" t="s">
-        <v>237</v>
-      </c>
-      <c r="D28" s="154">
+      <c r="C28" s="115" t="s">
+        <v>235</v>
+      </c>
+      <c r="D28" s="116">
         <v>10</v>
       </c>
     </row>
@@ -9533,13 +9597,13 @@
       <c r="A29" s="10">
         <v>23</v>
       </c>
-      <c r="B29" s="148" t="s">
+      <c r="B29" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C29" s="153" t="s">
-        <v>238</v>
-      </c>
-      <c r="D29" s="154">
+      <c r="C29" s="115" t="s">
+        <v>236</v>
+      </c>
+      <c r="D29" s="116">
         <v>4</v>
       </c>
       <c r="H29" s="4">
@@ -9550,13 +9614,13 @@
       <c r="A30" s="10">
         <v>24</v>
       </c>
-      <c r="B30" s="148" t="s">
+      <c r="B30" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="153" t="s">
-        <v>239</v>
-      </c>
-      <c r="D30" s="154">
+      <c r="C30" s="115" t="s">
+        <v>237</v>
+      </c>
+      <c r="D30" s="116">
         <v>12</v>
       </c>
     </row>
@@ -9564,13 +9628,13 @@
       <c r="A31" s="10">
         <v>25</v>
       </c>
-      <c r="B31" s="148" t="s">
+      <c r="B31" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C31" s="153" t="s">
-        <v>240</v>
-      </c>
-      <c r="D31" s="154">
+      <c r="C31" s="115" t="s">
+        <v>238</v>
+      </c>
+      <c r="D31" s="116">
         <v>3</v>
       </c>
     </row>
@@ -9578,13 +9642,13 @@
       <c r="A32" s="10">
         <v>26</v>
       </c>
-      <c r="B32" s="148" t="s">
+      <c r="B32" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C32" s="153" t="s">
-        <v>241</v>
-      </c>
-      <c r="D32" s="154">
+      <c r="C32" s="115" t="s">
+        <v>239</v>
+      </c>
+      <c r="D32" s="116">
         <v>8</v>
       </c>
     </row>
@@ -9592,13 +9656,13 @@
       <c r="A33" s="10">
         <v>27</v>
       </c>
-      <c r="B33" s="148" t="s">
+      <c r="B33" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C33" s="153" t="s">
-        <v>242</v>
-      </c>
-      <c r="D33" s="154">
+      <c r="C33" s="115" t="s">
+        <v>240</v>
+      </c>
+      <c r="D33" s="116">
         <v>3</v>
       </c>
     </row>
@@ -9606,13 +9670,13 @@
       <c r="A34" s="10">
         <v>28</v>
       </c>
-      <c r="B34" s="148" t="s">
+      <c r="B34" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="153" t="s">
-        <v>243</v>
-      </c>
-      <c r="D34" s="154">
+      <c r="C34" s="115" t="s">
+        <v>241</v>
+      </c>
+      <c r="D34" s="116">
         <v>8</v>
       </c>
     </row>
@@ -9620,13 +9684,13 @@
       <c r="A35" s="10">
         <v>29</v>
       </c>
-      <c r="B35" s="148" t="s">
+      <c r="B35" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C35" s="153" t="s">
-        <v>244</v>
-      </c>
-      <c r="D35" s="154">
+      <c r="C35" s="115" t="s">
+        <v>242</v>
+      </c>
+      <c r="D35" s="116">
         <v>3</v>
       </c>
     </row>
@@ -9634,13 +9698,13 @@
       <c r="A36" s="10">
         <v>30</v>
       </c>
-      <c r="B36" s="148" t="s">
+      <c r="B36" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C36" s="153" t="s">
-        <v>245</v>
-      </c>
-      <c r="D36" s="154">
+      <c r="C36" s="115" t="s">
+        <v>243</v>
+      </c>
+      <c r="D36" s="116">
         <v>8</v>
       </c>
     </row>
@@ -9648,13 +9712,13 @@
       <c r="A37" s="10">
         <v>31</v>
       </c>
-      <c r="B37" s="148" t="s">
+      <c r="B37" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C37" s="153" t="s">
-        <v>246</v>
-      </c>
-      <c r="D37" s="154">
+      <c r="C37" s="115" t="s">
+        <v>244</v>
+      </c>
+      <c r="D37" s="116">
         <v>3</v>
       </c>
     </row>
@@ -9662,13 +9726,13 @@
       <c r="A38" s="10">
         <v>32</v>
       </c>
-      <c r="B38" s="148" t="s">
+      <c r="B38" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C38" s="153" t="s">
-        <v>247</v>
-      </c>
-      <c r="D38" s="154">
+      <c r="C38" s="115" t="s">
+        <v>245</v>
+      </c>
+      <c r="D38" s="116">
         <v>8</v>
       </c>
     </row>
@@ -9676,13 +9740,13 @@
       <c r="A39" s="10">
         <v>33</v>
       </c>
-      <c r="B39" s="148" t="s">
+      <c r="B39" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="153" t="s">
-        <v>248</v>
-      </c>
-      <c r="D39" s="154">
+      <c r="C39" s="115" t="s">
+        <v>246</v>
+      </c>
+      <c r="D39" s="116">
         <v>4</v>
       </c>
     </row>
@@ -9690,13 +9754,13 @@
       <c r="A40" s="10">
         <v>34</v>
       </c>
-      <c r="B40" s="148" t="s">
+      <c r="B40" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="153" t="s">
-        <v>249</v>
-      </c>
-      <c r="D40" s="154">
+      <c r="C40" s="115" t="s">
+        <v>247</v>
+      </c>
+      <c r="D40" s="116">
         <v>10</v>
       </c>
     </row>
@@ -9704,13 +9768,13 @@
       <c r="A41" s="10">
         <v>35</v>
       </c>
-      <c r="B41" s="148" t="s">
+      <c r="B41" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C41" s="153" t="s">
-        <v>250</v>
-      </c>
-      <c r="D41" s="154">
+      <c r="C41" s="115" t="s">
+        <v>248</v>
+      </c>
+      <c r="D41" s="116">
         <v>4</v>
       </c>
     </row>
@@ -9718,13 +9782,13 @@
       <c r="A42" s="10">
         <v>36</v>
       </c>
-      <c r="B42" s="148" t="s">
+      <c r="B42" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C42" s="153" t="s">
-        <v>251</v>
-      </c>
-      <c r="D42" s="154">
+      <c r="C42" s="115" t="s">
+        <v>249</v>
+      </c>
+      <c r="D42" s="116">
         <v>10</v>
       </c>
     </row>
@@ -9732,13 +9796,13 @@
       <c r="A43" s="10">
         <v>37</v>
       </c>
-      <c r="B43" s="148" t="s">
+      <c r="B43" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C43" s="153" t="s">
-        <v>252</v>
-      </c>
-      <c r="D43" s="154">
+      <c r="C43" s="115" t="s">
+        <v>250</v>
+      </c>
+      <c r="D43" s="116">
         <v>3</v>
       </c>
     </row>
@@ -9746,13 +9810,13 @@
       <c r="A44" s="10">
         <v>38</v>
       </c>
-      <c r="B44" s="148" t="s">
+      <c r="B44" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C44" s="153" t="s">
-        <v>253</v>
-      </c>
-      <c r="D44" s="154">
+      <c r="C44" s="115" t="s">
+        <v>251</v>
+      </c>
+      <c r="D44" s="116">
         <v>8</v>
       </c>
     </row>
@@ -9760,13 +9824,13 @@
       <c r="A45" s="10">
         <v>39</v>
       </c>
-      <c r="B45" s="148" t="s">
+      <c r="B45" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C45" s="153" t="s">
-        <v>254</v>
-      </c>
-      <c r="D45" s="154">
+      <c r="C45" s="115" t="s">
+        <v>252</v>
+      </c>
+      <c r="D45" s="116">
         <v>3</v>
       </c>
     </row>
@@ -9774,13 +9838,13 @@
       <c r="A46" s="10">
         <v>40</v>
       </c>
-      <c r="B46" s="148" t="s">
+      <c r="B46" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C46" s="153" t="s">
-        <v>255</v>
-      </c>
-      <c r="D46" s="154">
+      <c r="C46" s="115" t="s">
+        <v>253</v>
+      </c>
+      <c r="D46" s="116">
         <v>8</v>
       </c>
     </row>
@@ -9788,13 +9852,13 @@
       <c r="A47" s="10">
         <v>41</v>
       </c>
-      <c r="B47" s="148" t="s">
+      <c r="B47" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C47" s="153" t="s">
+      <c r="C47" s="115" t="s">
         <v>38</v>
       </c>
-      <c r="D47" s="154">
+      <c r="D47" s="116">
         <v>3</v>
       </c>
     </row>
@@ -9802,23 +9866,23 @@
       <c r="A48" s="10">
         <v>42</v>
       </c>
-      <c r="B48" s="148" t="s">
+      <c r="B48" s="112" t="s">
         <v>40</v>
       </c>
-      <c r="C48" s="153" t="s">
+      <c r="C48" s="115" t="s">
         <v>39</v>
       </c>
-      <c r="D48" s="154">
+      <c r="D48" s="116">
         <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="122" t="s">
+      <c r="A49" s="136" t="s">
         <v>41</v>
       </c>
-      <c r="B49" s="122"/>
-      <c r="C49" s="151"/>
-      <c r="D49" s="159">
+      <c r="B49" s="136"/>
+      <c r="C49" s="138"/>
+      <c r="D49" s="121">
         <f>SUM(D22:D48)</f>
         <v>164</v>
       </c>
@@ -9830,10 +9894,10 @@
       <c r="B50" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C50" s="157" t="s">
+      <c r="C50" s="119" t="s">
         <v>32</v>
       </c>
-      <c r="D50" s="160">
+      <c r="D50" s="122">
         <v>3</v>
       </c>
     </row>
@@ -9844,10 +9908,10 @@
       <c r="B51" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C51" s="158" t="s">
+      <c r="C51" s="120" t="s">
         <v>42</v>
       </c>
-      <c r="D51" s="160">
+      <c r="D51" s="122">
         <v>6</v>
       </c>
     </row>
@@ -9858,10 +9922,10 @@
       <c r="B52" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C52" s="158" t="s">
+      <c r="C52" s="120" t="s">
         <v>43</v>
       </c>
-      <c r="D52" s="160">
+      <c r="D52" s="122">
         <v>10</v>
       </c>
     </row>
@@ -9872,10 +9936,10 @@
       <c r="B53" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C53" s="158" t="s">
+      <c r="C53" s="120" t="s">
         <v>44</v>
       </c>
-      <c r="D53" s="160">
+      <c r="D53" s="122">
         <v>10</v>
       </c>
     </row>
@@ -9886,10 +9950,10 @@
       <c r="B54" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C54" s="157" t="s">
+      <c r="C54" s="119" t="s">
         <v>45</v>
       </c>
-      <c r="D54" s="160">
+      <c r="D54" s="122">
         <v>5</v>
       </c>
     </row>
@@ -9900,10 +9964,10 @@
       <c r="B55" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C55" s="157" t="s">
+      <c r="C55" s="119" t="s">
         <v>46</v>
       </c>
-      <c r="D55" s="160">
+      <c r="D55" s="122">
         <v>6</v>
       </c>
     </row>
@@ -9914,10 +9978,10 @@
       <c r="B56" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C56" s="157" t="s">
+      <c r="C56" s="119" t="s">
         <v>47</v>
       </c>
-      <c r="D56" s="160">
+      <c r="D56" s="122">
         <v>6</v>
       </c>
     </row>
@@ -9928,10 +9992,10 @@
       <c r="B57" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C57" s="157" t="s">
+      <c r="C57" s="119" t="s">
         <v>48</v>
       </c>
-      <c r="D57" s="160">
+      <c r="D57" s="122">
         <v>5</v>
       </c>
     </row>
@@ -9942,18 +10006,18 @@
       <c r="B58" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="C58" s="158" t="s">
+      <c r="C58" s="120" t="s">
         <v>38</v>
       </c>
-      <c r="D58" s="160">
+      <c r="D58" s="122">
         <v>3</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="123"/>
-      <c r="B59" s="123"/>
-      <c r="C59" s="123"/>
-      <c r="D59" s="152">
+      <c r="A59" s="139"/>
+      <c r="B59" s="139"/>
+      <c r="C59" s="139"/>
+      <c r="D59" s="114">
         <f>SUM(D50:D58)</f>
         <v>54</v>
       </c>
@@ -9966,16 +10030,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F1:L1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F2:L2"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="A4:C4"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A49:C49"/>
     <mergeCell ref="A59:C59"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="F1:L1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="F2:L2"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="A4:C4"/>
   </mergeCells>
   <phoneticPr fontId="41" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="1.1437007874015752" bottom="1.1437007874015752" header="0.75000000000000011" footer="0.75000000000000011"/>
@@ -9999,19 +10063,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="145" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="125"/>
-      <c r="C1" s="125"/>
+      <c r="B1" s="145"/>
+      <c r="C1" s="145"/>
     </row>
     <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="126" t="s">
+      <c r="A3" s="146" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="126"/>
-      <c r="C3" s="126"/>
+      <c r="B3" s="146"/>
+      <c r="C3" s="146"/>
     </row>
     <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
@@ -10120,11 +10184,11 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="126" t="s">
+      <c r="A14" s="146" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="126"/>
-      <c r="C14" s="126"/>
+      <c r="B14" s="146"/>
+      <c r="C14" s="146"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
@@ -10233,54 +10297,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="130" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="112"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="112"/>
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="130"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="130"/>
     </row>
     <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="131" t="s">
         <v>76</v>
       </c>
-      <c r="B2" s="113"/>
-      <c r="C2" s="113"/>
-      <c r="D2" s="113"/>
+      <c r="B2" s="131"/>
+      <c r="C2" s="131"/>
+      <c r="D2" s="131"/>
       <c r="E2" s="40">
         <f>Planejamento!$B$10</f>
         <v>558</v>
       </c>
       <c r="F2" s="41"/>
-      <c r="G2" s="113" t="s">
+      <c r="G2" s="131" t="s">
         <v>76</v>
       </c>
-      <c r="H2" s="113"/>
-      <c r="I2" s="113"/>
-      <c r="J2" s="113"/>
+      <c r="H2" s="131"/>
+      <c r="I2" s="131"/>
+      <c r="J2" s="131"/>
       <c r="K2" s="40"/>
     </row>
     <row r="3" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="42"/>
       <c r="B3" s="43"/>
-      <c r="C3" s="114" t="s">
+      <c r="C3" s="132" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="114"/>
-      <c r="E3" s="114"/>
+      <c r="D3" s="132"/>
+      <c r="E3" s="132"/>
       <c r="F3" s="44"/>
-      <c r="G3" s="115" t="s">
+      <c r="G3" s="133" t="s">
         <v>78</v>
       </c>
-      <c r="H3" s="115"/>
-      <c r="I3" s="115"/>
+      <c r="H3" s="133"/>
+      <c r="I3" s="133"/>
       <c r="J3" s="46"/>
       <c r="K3" s="47"/>
     </row>
@@ -10288,7 +10352,7 @@
       <c r="A4" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="165" t="s">
+      <c r="B4" s="127" t="s">
         <v>80</v>
       </c>
       <c r="C4" s="45" t="s">
@@ -10320,178 +10384,178 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="163">
+      <c r="A5" s="125">
         <v>1</v>
       </c>
-      <c r="B5" s="167" t="s">
+      <c r="B5" s="129" t="s">
+        <v>284</v>
+      </c>
+      <c r="C5" s="126" t="s">
+        <v>266</v>
+      </c>
+      <c r="D5" s="124" t="s">
+        <v>267</v>
+      </c>
+      <c r="E5" s="124">
+        <v>24</v>
+      </c>
+      <c r="F5" s="124" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="124" t="s">
+        <v>266</v>
+      </c>
+      <c r="H5" s="124" t="s">
+        <v>267</v>
+      </c>
+      <c r="I5" s="124">
+        <v>24</v>
+      </c>
+      <c r="J5" s="124" t="s">
+        <v>268</v>
+      </c>
+      <c r="K5" s="124" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="125">
+        <v>2</v>
+      </c>
+      <c r="B6" s="129" t="s">
+        <v>307</v>
+      </c>
+      <c r="C6" s="126" t="s">
+        <v>269</v>
+      </c>
+      <c r="D6" s="124" t="s">
+        <v>270</v>
+      </c>
+      <c r="E6" s="124">
+        <v>90</v>
+      </c>
+      <c r="F6" s="124" t="s">
+        <v>88</v>
+      </c>
+      <c r="G6" s="124"/>
+      <c r="H6" s="124"/>
+      <c r="I6" s="124"/>
+      <c r="J6" s="124"/>
+      <c r="K6" s="124" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="125">
+        <v>3</v>
+      </c>
+      <c r="B7" s="129" t="s">
+        <v>285</v>
+      </c>
+      <c r="C7" s="126" t="s">
+        <v>272</v>
+      </c>
+      <c r="D7" s="124" t="s">
+        <v>273</v>
+      </c>
+      <c r="E7" s="124">
+        <v>96</v>
+      </c>
+      <c r="F7" s="124" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="124"/>
+      <c r="H7" s="124"/>
+      <c r="I7" s="124"/>
+      <c r="J7" s="124"/>
+      <c r="K7" s="124" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="125">
+        <v>4</v>
+      </c>
+      <c r="B8" s="129" t="s">
+        <v>285</v>
+      </c>
+      <c r="C8" s="126" t="s">
+        <v>275</v>
+      </c>
+      <c r="D8" s="124" t="s">
+        <v>276</v>
+      </c>
+      <c r="E8" s="124">
+        <v>108</v>
+      </c>
+      <c r="F8" s="124" t="s">
+        <v>88</v>
+      </c>
+      <c r="G8" s="124"/>
+      <c r="H8" s="124"/>
+      <c r="I8" s="124"/>
+      <c r="J8" s="124"/>
+      <c r="K8" s="124" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="125">
+        <v>5</v>
+      </c>
+      <c r="B9" s="129" t="s">
         <v>286</v>
       </c>
-      <c r="C5" s="164" t="s">
-        <v>268</v>
-      </c>
-      <c r="D5" s="162" t="s">
-        <v>269</v>
-      </c>
-      <c r="E5" s="162">
-        <v>24</v>
-      </c>
-      <c r="F5" s="162" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="162" t="s">
-        <v>268</v>
-      </c>
-      <c r="H5" s="162" t="s">
-        <v>269</v>
-      </c>
-      <c r="I5" s="162">
-        <v>24</v>
-      </c>
-      <c r="J5" s="162" t="s">
-        <v>270</v>
-      </c>
-      <c r="K5" s="162" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="163">
-        <v>2</v>
-      </c>
-      <c r="B6" s="167" t="s">
+      <c r="C9" s="126" t="s">
+        <v>278</v>
+      </c>
+      <c r="D9" s="124" t="s">
+        <v>279</v>
+      </c>
+      <c r="E9" s="124">
+        <v>110</v>
+      </c>
+      <c r="F9" s="124" t="s">
+        <v>88</v>
+      </c>
+      <c r="G9" s="124"/>
+      <c r="H9" s="124"/>
+      <c r="I9" s="124"/>
+      <c r="J9" s="124"/>
+      <c r="K9" s="124" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="125">
+        <v>6</v>
+      </c>
+      <c r="B10" s="129" t="s">
         <v>286</v>
       </c>
-      <c r="C6" s="164" t="s">
-        <v>271</v>
-      </c>
-      <c r="D6" s="162" t="s">
-        <v>272</v>
-      </c>
-      <c r="E6" s="162">
-        <v>90</v>
-      </c>
-      <c r="F6" s="162" t="s">
+      <c r="C10" s="126" t="s">
+        <v>281</v>
+      </c>
+      <c r="D10" s="124" t="s">
+        <v>282</v>
+      </c>
+      <c r="E10" s="124">
+        <v>130</v>
+      </c>
+      <c r="F10" s="124" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="162"/>
-      <c r="H6" s="162"/>
-      <c r="I6" s="162"/>
-      <c r="J6" s="162"/>
-      <c r="K6" s="162" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="163">
-        <v>3</v>
-      </c>
-      <c r="B7" s="167" t="s">
-        <v>287</v>
-      </c>
-      <c r="C7" s="164" t="s">
-        <v>274</v>
-      </c>
-      <c r="D7" s="162" t="s">
-        <v>275</v>
-      </c>
-      <c r="E7" s="162">
-        <v>96</v>
-      </c>
-      <c r="F7" s="162" t="s">
-        <v>88</v>
-      </c>
-      <c r="G7" s="162"/>
-      <c r="H7" s="162"/>
-      <c r="I7" s="162"/>
-      <c r="J7" s="162"/>
-      <c r="K7" s="162" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="163">
-        <v>4</v>
-      </c>
-      <c r="B8" s="167" t="s">
-        <v>287</v>
-      </c>
-      <c r="C8" s="164" t="s">
-        <v>277</v>
-      </c>
-      <c r="D8" s="162" t="s">
-        <v>278</v>
-      </c>
-      <c r="E8" s="162">
-        <v>108</v>
-      </c>
-      <c r="F8" s="162" t="s">
-        <v>88</v>
-      </c>
-      <c r="G8" s="162"/>
-      <c r="H8" s="162"/>
-      <c r="I8" s="162"/>
-      <c r="J8" s="162"/>
-      <c r="K8" s="162" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="163">
-        <v>5</v>
-      </c>
-      <c r="B9" s="167" t="s">
-        <v>288</v>
-      </c>
-      <c r="C9" s="164" t="s">
-        <v>280</v>
-      </c>
-      <c r="D9" s="162" t="s">
-        <v>281</v>
-      </c>
-      <c r="E9" s="162">
-        <v>110</v>
-      </c>
-      <c r="F9" s="162" t="s">
-        <v>88</v>
-      </c>
-      <c r="G9" s="162"/>
-      <c r="H9" s="162"/>
-      <c r="I9" s="162"/>
-      <c r="J9" s="162"/>
-      <c r="K9" s="162" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="163">
-        <v>6</v>
-      </c>
-      <c r="B10" s="167" t="s">
-        <v>288</v>
-      </c>
-      <c r="C10" s="164" t="s">
+      <c r="G10" s="124"/>
+      <c r="H10" s="124"/>
+      <c r="I10" s="124"/>
+      <c r="J10" s="124"/>
+      <c r="K10" s="124" t="s">
         <v>283</v>
-      </c>
-      <c r="D10" s="162" t="s">
-        <v>284</v>
-      </c>
-      <c r="E10" s="162">
-        <v>130</v>
-      </c>
-      <c r="F10" s="162" t="s">
-        <v>88</v>
-      </c>
-      <c r="G10" s="162"/>
-      <c r="H10" s="162"/>
-      <c r="I10" s="162"/>
-      <c r="J10" s="162"/>
-      <c r="K10" s="162" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" s="49"/>
-      <c r="B11" s="166"/>
+      <c r="B11" s="128"/>
       <c r="C11" s="51"/>
       <c r="D11" s="50"/>
       <c r="E11" s="52">
@@ -10522,7 +10586,7 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="G3:I3"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:H10 A5:A10 C5:D10">
+  <conditionalFormatting sqref="A5:A10 C5:D10 G5:H10">
     <cfRule type="expression" dxfId="7" priority="6" stopIfTrue="1">
       <formula>OR($F5="Planned",$F5="Unplanned")</formula>
     </cfRule>
@@ -10564,7 +10628,8 @@
     <col min="5" max="5" width="8.8984375" style="57" customWidth="1"/>
     <col min="6" max="6" width="12.5" style="57" customWidth="1"/>
     <col min="7" max="7" width="9.09765625" style="57" customWidth="1"/>
-    <col min="8" max="9" width="12.19921875" style="57" customWidth="1"/>
+    <col min="8" max="8" width="12.19921875" style="57" customWidth="1"/>
+    <col min="9" max="9" width="15.8984375" style="57" customWidth="1"/>
     <col min="10" max="10" width="24.19921875" style="57" customWidth="1"/>
     <col min="11" max="11" width="27.8984375" style="57" customWidth="1"/>
     <col min="12" max="12" width="8.5" style="57" customWidth="1"/>
@@ -10613,19 +10678,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="130" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="112"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="112"/>
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="130"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="130"/>
     </row>
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -10779,10 +10844,10 @@
       </c>
     </row>
     <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="128" t="s">
+      <c r="D33" s="154" t="s">
         <v>120</v>
       </c>
-      <c r="E33" s="128"/>
+      <c r="E33" s="154"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D34" s="59">
@@ -10834,137 +10899,137 @@
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="129" t="s">
+      <c r="A41" s="155" t="s">
         <v>127</v>
       </c>
-      <c r="B41" s="129"/>
-      <c r="C41" s="129"/>
-      <c r="D41" s="129"/>
-      <c r="E41" s="129"/>
-      <c r="F41" s="129"/>
-      <c r="G41" s="129"/>
-      <c r="H41" s="129"/>
-      <c r="I41" s="129"/>
-      <c r="J41" s="129"/>
-      <c r="K41" s="129"/>
+      <c r="B41" s="155"/>
+      <c r="C41" s="155"/>
+      <c r="D41" s="155"/>
+      <c r="E41" s="155"/>
+      <c r="F41" s="155"/>
+      <c r="G41" s="155"/>
+      <c r="H41" s="155"/>
+      <c r="I41" s="155"/>
+      <c r="J41" s="155"/>
+      <c r="K41" s="155"/>
     </row>
     <row r="42" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="130" t="s">
+      <c r="A42" s="156" t="s">
         <v>128</v>
       </c>
-      <c r="B42" s="130"/>
-      <c r="C42" s="130"/>
-      <c r="D42" s="130"/>
-      <c r="E42" s="130"/>
-      <c r="F42" s="130"/>
-      <c r="G42" s="130"/>
-      <c r="H42" s="130"/>
-      <c r="I42" s="130"/>
-      <c r="J42" s="130"/>
-      <c r="K42" s="130"/>
+      <c r="B42" s="156"/>
+      <c r="C42" s="156"/>
+      <c r="D42" s="156"/>
+      <c r="E42" s="156"/>
+      <c r="F42" s="156"/>
+      <c r="G42" s="156"/>
+      <c r="H42" s="156"/>
+      <c r="I42" s="156"/>
+      <c r="J42" s="156"/>
+      <c r="K42" s="156"/>
     </row>
     <row r="43" spans="1:11" s="56" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="131" t="s">
+      <c r="A43" s="157" t="s">
         <v>129</v>
       </c>
-      <c r="B43" s="131"/>
-      <c r="C43" s="131"/>
-      <c r="D43" s="131"/>
-      <c r="E43" s="131"/>
-      <c r="F43" s="131"/>
-      <c r="G43" s="131"/>
-      <c r="H43" s="131"/>
-      <c r="I43" s="131"/>
-      <c r="J43" s="131"/>
-      <c r="K43" s="131"/>
+      <c r="B43" s="157"/>
+      <c r="C43" s="157"/>
+      <c r="D43" s="157"/>
+      <c r="E43" s="157"/>
+      <c r="F43" s="157"/>
+      <c r="G43" s="157"/>
+      <c r="H43" s="157"/>
+      <c r="I43" s="157"/>
+      <c r="J43" s="157"/>
+      <c r="K43" s="157"/>
     </row>
     <row r="44" spans="1:11" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="127" t="s">
+      <c r="A44" s="153" t="s">
         <v>130</v>
       </c>
-      <c r="B44" s="127"/>
-      <c r="C44" s="127"/>
-      <c r="D44" s="127"/>
-      <c r="E44" s="127"/>
-      <c r="F44" s="127"/>
-      <c r="G44" s="127"/>
-      <c r="H44" s="127"/>
-      <c r="I44" s="127"/>
-      <c r="J44" s="127"/>
-      <c r="K44" s="127"/>
+      <c r="B44" s="153"/>
+      <c r="C44" s="153"/>
+      <c r="D44" s="153"/>
+      <c r="E44" s="153"/>
+      <c r="F44" s="153"/>
+      <c r="G44" s="153"/>
+      <c r="H44" s="153"/>
+      <c r="I44" s="153"/>
+      <c r="J44" s="153"/>
+      <c r="K44" s="153"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="134" t="s">
+      <c r="A46" s="149" t="s">
         <v>131</v>
       </c>
-      <c r="B46" s="134"/>
-      <c r="C46" s="134"/>
-      <c r="D46" s="134"/>
-      <c r="E46" s="134"/>
-      <c r="F46" s="134"/>
-      <c r="G46" s="134"/>
-      <c r="H46" s="134"/>
-      <c r="I46" s="134"/>
-      <c r="J46" s="134"/>
-      <c r="K46" s="134"/>
+      <c r="B46" s="149"/>
+      <c r="C46" s="149"/>
+      <c r="D46" s="149"/>
+      <c r="E46" s="149"/>
+      <c r="F46" s="149"/>
+      <c r="G46" s="149"/>
+      <c r="H46" s="149"/>
+      <c r="I46" s="149"/>
+      <c r="J46" s="149"/>
+      <c r="K46" s="149"/>
     </row>
     <row r="47" spans="1:11" s="65" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="63" t="s">
         <v>132</v>
       </c>
       <c r="B47" s="64"/>
-      <c r="C47" s="135" t="s">
+      <c r="C47" s="150" t="s">
         <v>133</v>
       </c>
-      <c r="D47" s="135"/>
-      <c r="E47" s="135"/>
-      <c r="F47" s="135"/>
-      <c r="G47" s="135"/>
-      <c r="H47" s="135"/>
-      <c r="I47" s="135"/>
-      <c r="J47" s="135"/>
-      <c r="K47" s="135"/>
+      <c r="D47" s="150"/>
+      <c r="E47" s="150"/>
+      <c r="F47" s="150"/>
+      <c r="G47" s="150"/>
+      <c r="H47" s="150"/>
+      <c r="I47" s="150"/>
+      <c r="J47" s="150"/>
+      <c r="K47" s="150"/>
     </row>
     <row r="48" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="136"/>
-      <c r="B48" s="132" t="s">
+      <c r="A48" s="151"/>
+      <c r="B48" s="147" t="s">
         <v>134</v>
       </c>
-      <c r="C48" s="132" t="s">
+      <c r="C48" s="147" t="s">
         <v>135</v>
       </c>
-      <c r="D48" s="132" t="s">
+      <c r="D48" s="147" t="s">
         <v>136</v>
       </c>
-      <c r="E48" s="132" t="s">
+      <c r="E48" s="147" t="s">
         <v>105</v>
       </c>
-      <c r="F48" s="132" t="s">
+      <c r="F48" s="147" t="s">
         <v>137</v>
       </c>
-      <c r="G48" s="132" t="s">
+      <c r="G48" s="147" t="s">
         <v>109</v>
       </c>
-      <c r="H48" s="137" t="s">
+      <c r="H48" s="152" t="s">
         <v>138</v>
       </c>
-      <c r="I48" s="137"/>
-      <c r="J48" s="137"/>
-      <c r="K48" s="137"/>
+      <c r="I48" s="152"/>
+      <c r="J48" s="152"/>
+      <c r="K48" s="152"/>
     </row>
     <row r="49" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="136"/>
-      <c r="B49" s="132"/>
-      <c r="C49" s="132"/>
-      <c r="D49" s="132"/>
-      <c r="E49" s="132"/>
-      <c r="F49" s="132"/>
-      <c r="G49" s="132"/>
-      <c r="H49" s="132" t="s">
+      <c r="A49" s="151"/>
+      <c r="B49" s="147"/>
+      <c r="C49" s="147"/>
+      <c r="D49" s="147"/>
+      <c r="E49" s="147"/>
+      <c r="F49" s="147"/>
+      <c r="G49" s="147"/>
+      <c r="H49" s="147" t="s">
         <v>139</v>
       </c>
-      <c r="I49" s="132"/>
+      <c r="I49" s="147"/>
       <c r="J49" s="66" t="s">
         <v>140</v>
       </c>
@@ -10972,101 +11037,175 @@
         <v>141</v>
       </c>
     </row>
-    <row r="50" spans="1:11" s="67" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" s="67" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="68">
         <v>1</v>
       </c>
       <c r="B50" s="69" t="s">
-        <v>142</v>
+        <v>287</v>
       </c>
       <c r="C50" s="70">
-        <v>43891</v>
+        <v>46117</v>
       </c>
       <c r="D50" s="71" t="s">
         <v>103</v>
       </c>
       <c r="E50" s="71" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F50" s="72" t="str">
         <f t="shared" ref="F50:F60" si="0">IF(OR((CODE($D50)*CODE($E50))=$D$36,(CODE($D50)*CODE($E50))=$D$35),$D$15,IF(OR((CODE($D50)*CODE($E50))=$D$34,(CODE($D50)*CODE($E50))=$D$37),$D$16,IF(OR((CODE($D50)*CODE($E50))=$D$38,(CODE($D50)*CODE($E50))=$D$39),$D$17,0)))</f>
-        <v>Média</v>
+        <v>Alta</v>
       </c>
       <c r="G50" s="71" t="s">
         <v>110</v>
       </c>
-      <c r="H50" s="133"/>
-      <c r="I50" s="133"/>
-      <c r="J50" s="73"/>
+      <c r="H50" s="168" t="s">
+        <v>288</v>
+      </c>
+      <c r="I50" s="168"/>
+      <c r="J50" s="73" t="s">
+        <v>289</v>
+      </c>
       <c r="K50" s="73" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="68"/>
-      <c r="B51" s="69"/>
-      <c r="C51" s="70"/>
+        <v>290</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" s="67" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A51" s="68">
+        <v>2</v>
+      </c>
+      <c r="B51" s="69" t="s">
+        <v>291</v>
+      </c>
+      <c r="C51" s="70">
+        <v>46117</v>
+      </c>
       <c r="D51" s="71" t="s">
-        <v>102</v>
-      </c>
-      <c r="E51" s="71"/>
-      <c r="F51" s="72" t="e">
+        <v>104</v>
+      </c>
+      <c r="E51" s="71" t="s">
+        <v>108</v>
+      </c>
+      <c r="F51" s="72" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G51" s="71"/>
-      <c r="H51" s="74"/>
-      <c r="I51" s="75"/>
-      <c r="J51" s="73"/>
-      <c r="K51" s="73"/>
-    </row>
-    <row r="52" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="68"/>
-      <c r="B52" s="69"/>
-      <c r="C52" s="70"/>
-      <c r="D52" s="71"/>
-      <c r="E52" s="71"/>
-      <c r="F52" s="72" t="e">
+        <v>Alta</v>
+      </c>
+      <c r="G51" s="71" t="s">
+        <v>110</v>
+      </c>
+      <c r="H51" s="169" t="s">
+        <v>292</v>
+      </c>
+      <c r="I51" s="170"/>
+      <c r="J51" s="73" t="s">
+        <v>293</v>
+      </c>
+      <c r="K51" s="73" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" s="67" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A52" s="68">
+        <v>3</v>
+      </c>
+      <c r="B52" s="69" t="s">
+        <v>295</v>
+      </c>
+      <c r="C52" s="70">
+        <v>46117</v>
+      </c>
+      <c r="D52" s="71" t="s">
+        <v>104</v>
+      </c>
+      <c r="E52" s="71" t="s">
+        <v>108</v>
+      </c>
+      <c r="F52" s="72" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G52" s="71"/>
-      <c r="H52" s="74"/>
-      <c r="I52" s="75"/>
-      <c r="J52" s="73"/>
-      <c r="K52" s="73"/>
-    </row>
-    <row r="53" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="68"/>
-      <c r="B53" s="69"/>
-      <c r="C53" s="70"/>
-      <c r="D53" s="71"/>
-      <c r="E53" s="71"/>
-      <c r="F53" s="72" t="e">
+        <v>Alta</v>
+      </c>
+      <c r="G52" s="71" t="s">
+        <v>110</v>
+      </c>
+      <c r="H52" s="169" t="s">
+        <v>296</v>
+      </c>
+      <c r="I52" s="170"/>
+      <c r="J52" s="73" t="s">
+        <v>297</v>
+      </c>
+      <c r="K52" s="73" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" s="67" customFormat="1" ht="30.6" x14ac:dyDescent="0.25">
+      <c r="A53" s="68">
+        <v>4</v>
+      </c>
+      <c r="B53" s="69" t="s">
+        <v>299</v>
+      </c>
+      <c r="C53" s="70">
+        <v>46117</v>
+      </c>
+      <c r="D53" s="71" t="s">
+        <v>103</v>
+      </c>
+      <c r="E53" s="71" t="s">
+        <v>107</v>
+      </c>
+      <c r="F53" s="72" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G53" s="71"/>
-      <c r="H53" s="74"/>
-      <c r="I53" s="75"/>
-      <c r="J53" s="73"/>
-      <c r="K53" s="73"/>
-    </row>
-    <row r="54" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="68"/>
-      <c r="B54" s="69"/>
-      <c r="C54" s="70"/>
-      <c r="D54" s="71"/>
-      <c r="E54" s="71"/>
-      <c r="F54" s="72" t="e">
+        <v>Média</v>
+      </c>
+      <c r="G53" s="71" t="s">
+        <v>110</v>
+      </c>
+      <c r="H53" s="169" t="s">
+        <v>300</v>
+      </c>
+      <c r="I53" s="170"/>
+      <c r="J53" s="73" t="s">
+        <v>301</v>
+      </c>
+      <c r="K53" s="73" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" s="67" customFormat="1" ht="30.6" x14ac:dyDescent="0.25">
+      <c r="A54" s="68">
+        <v>5</v>
+      </c>
+      <c r="B54" s="69" t="s">
+        <v>303</v>
+      </c>
+      <c r="C54" s="70">
+        <v>46117</v>
+      </c>
+      <c r="D54" s="71" t="s">
+        <v>103</v>
+      </c>
+      <c r="E54" s="71" t="s">
+        <v>108</v>
+      </c>
+      <c r="F54" s="72" t="str">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G54" s="71"/>
-      <c r="H54" s="74"/>
-      <c r="I54" s="75"/>
-      <c r="J54" s="73"/>
-      <c r="K54" s="73"/>
+        <v>Alta</v>
+      </c>
+      <c r="G54" s="71" t="s">
+        <v>110</v>
+      </c>
+      <c r="H54" s="169" t="s">
+        <v>304</v>
+      </c>
+      <c r="I54" s="170"/>
+      <c r="J54" s="73" t="s">
+        <v>305</v>
+      </c>
+      <c r="K54" s="73" t="s">
+        <v>306</v>
+      </c>
     </row>
     <row r="55" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="68"/>
@@ -11143,8 +11282,8 @@
         <v>#VALUE!</v>
       </c>
       <c r="G59" s="71"/>
-      <c r="H59" s="133"/>
-      <c r="I59" s="133"/>
+      <c r="H59" s="148"/>
+      <c r="I59" s="148"/>
       <c r="J59" s="73"/>
       <c r="K59" s="73"/>
     </row>
@@ -11159,13 +11298,21 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="71"/>
-      <c r="H60" s="133"/>
-      <c r="I60" s="133"/>
+      <c r="H60" s="148"/>
+      <c r="I60" s="148"/>
       <c r="J60" s="73"/>
       <c r="K60" s="73"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="24">
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
@@ -11180,12 +11327,8 @@
     <mergeCell ref="F48:F49"/>
     <mergeCell ref="G48:G49"/>
     <mergeCell ref="H48:K48"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="H52:I52"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
     <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="equal">
@@ -11243,167 +11386,167 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="140" t="s">
+      <c r="A1" s="160" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="160"/>
+      <c r="C1" s="160"/>
+      <c r="D1" s="160"/>
+      <c r="E1" s="160"/>
+      <c r="F1" s="160"/>
+      <c r="G1" s="160"/>
+      <c r="H1" s="160"/>
+      <c r="I1" s="160"/>
+      <c r="J1" s="160"/>
+      <c r="K1" s="160"/>
+      <c r="L1" s="160"/>
+      <c r="M1" s="160"/>
+      <c r="N1" s="160"/>
+    </row>
+    <row r="2" spans="1:23" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="161" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="161"/>
+      <c r="C2" s="161"/>
+      <c r="D2" s="161"/>
+      <c r="E2" s="161"/>
+      <c r="F2" s="161"/>
+      <c r="G2" s="161"/>
+      <c r="H2" s="161"/>
+      <c r="I2" s="161"/>
+      <c r="J2" s="161"/>
+      <c r="K2" s="161"/>
+      <c r="L2" s="161"/>
+      <c r="M2" s="161"/>
+      <c r="N2" s="161"/>
+    </row>
+    <row r="3" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="162" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3" s="162"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="162"/>
+      <c r="G3" s="162"/>
+      <c r="H3" s="162"/>
+      <c r="I3" s="162"/>
+      <c r="J3" s="162"/>
+      <c r="K3" s="162"/>
+      <c r="L3" s="162"/>
+      <c r="M3" s="162"/>
+      <c r="N3" s="162"/>
+    </row>
+    <row r="4" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="163" t="s">
         <v>144</v>
       </c>
-      <c r="B1" s="140"/>
-      <c r="C1" s="140"/>
-      <c r="D1" s="140"/>
-      <c r="E1" s="140"/>
-      <c r="F1" s="140"/>
-      <c r="G1" s="140"/>
-      <c r="H1" s="140"/>
-      <c r="I1" s="140"/>
-      <c r="J1" s="140"/>
-      <c r="K1" s="140"/>
-      <c r="L1" s="140"/>
-      <c r="M1" s="140"/>
-      <c r="N1" s="140"/>
-    </row>
-    <row r="2" spans="1:23" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="141" t="s">
-        <v>127</v>
-      </c>
-      <c r="B2" s="141"/>
-      <c r="C2" s="141"/>
-      <c r="D2" s="141"/>
-      <c r="E2" s="141"/>
-      <c r="F2" s="141"/>
-      <c r="G2" s="141"/>
-      <c r="H2" s="141"/>
-      <c r="I2" s="141"/>
-      <c r="J2" s="141"/>
-      <c r="K2" s="141"/>
-      <c r="L2" s="141"/>
-      <c r="M2" s="141"/>
-      <c r="N2" s="141"/>
-    </row>
-    <row r="3" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="142" t="s">
+      <c r="B4" s="163"/>
+      <c r="C4" s="163"/>
+      <c r="D4" s="163"/>
+      <c r="E4" s="163"/>
+      <c r="F4" s="163"/>
+      <c r="G4" s="163"/>
+      <c r="H4" s="163"/>
+      <c r="I4" s="163"/>
+      <c r="J4" s="163"/>
+      <c r="K4" s="163"/>
+      <c r="L4" s="163"/>
+      <c r="M4" s="163"/>
+      <c r="N4" s="163"/>
+    </row>
+    <row r="5" spans="1:23" s="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="164" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="142"/>
-      <c r="C3" s="142"/>
-      <c r="D3" s="142"/>
-      <c r="E3" s="142"/>
-      <c r="F3" s="142"/>
-      <c r="G3" s="142"/>
-      <c r="H3" s="142"/>
-      <c r="I3" s="142"/>
-      <c r="J3" s="142"/>
-      <c r="K3" s="142"/>
-      <c r="L3" s="142"/>
-      <c r="M3" s="142"/>
-      <c r="N3" s="142"/>
-    </row>
-    <row r="4" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="143" t="s">
-        <v>146</v>
-      </c>
-      <c r="B4" s="143"/>
-      <c r="C4" s="143"/>
-      <c r="D4" s="143"/>
-      <c r="E4" s="143"/>
-      <c r="F4" s="143"/>
-      <c r="G4" s="143"/>
-      <c r="H4" s="143"/>
-      <c r="I4" s="143"/>
-      <c r="J4" s="143"/>
-      <c r="K4" s="143"/>
-      <c r="L4" s="143"/>
-      <c r="M4" s="143"/>
-      <c r="N4" s="143"/>
-    </row>
-    <row r="5" spans="1:23" s="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="144" t="s">
-        <v>147</v>
-      </c>
-      <c r="B5" s="144"/>
-      <c r="C5" s="144"/>
-      <c r="D5" s="144"/>
-      <c r="E5" s="144"/>
-      <c r="F5" s="144"/>
-      <c r="G5" s="144"/>
-      <c r="H5" s="144"/>
-      <c r="I5" s="144"/>
-      <c r="J5" s="144"/>
-      <c r="K5" s="144"/>
-      <c r="L5" s="144"/>
-      <c r="M5" s="144"/>
-      <c r="N5" s="144"/>
+      <c r="B5" s="164"/>
+      <c r="C5" s="164"/>
+      <c r="D5" s="164"/>
+      <c r="E5" s="164"/>
+      <c r="F5" s="164"/>
+      <c r="G5" s="164"/>
+      <c r="H5" s="164"/>
+      <c r="I5" s="164"/>
+      <c r="J5" s="164"/>
+      <c r="K5" s="164"/>
+      <c r="L5" s="164"/>
+      <c r="M5" s="164"/>
+      <c r="N5" s="164"/>
     </row>
     <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="138" t="s">
+      <c r="A7" s="158" t="s">
+        <v>146</v>
+      </c>
+      <c r="B7" s="158"/>
+      <c r="D7" s="158" t="s">
+        <v>147</v>
+      </c>
+      <c r="E7" s="158"/>
+      <c r="G7" s="158" t="s">
         <v>148</v>
       </c>
-      <c r="B7" s="138"/>
-      <c r="D7" s="138" t="s">
+      <c r="H7" s="158"/>
+      <c r="I7" s="158"/>
+      <c r="J7" s="158"/>
+      <c r="K7" s="158"/>
+      <c r="M7" s="158" t="s">
         <v>149</v>
       </c>
-      <c r="E7" s="138"/>
-      <c r="G7" s="138" t="s">
-        <v>150</v>
-      </c>
-      <c r="H7" s="138"/>
-      <c r="I7" s="138"/>
-      <c r="J7" s="138"/>
-      <c r="K7" s="138"/>
-      <c r="M7" s="138" t="s">
-        <v>151</v>
-      </c>
-      <c r="N7" s="138"/>
+      <c r="N7" s="158"/>
     </row>
     <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="79" t="s">
+        <v>150</v>
+      </c>
+      <c r="B8" s="80" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8" s="79" t="s">
         <v>152</v>
       </c>
-      <c r="B8" s="80" t="s">
+      <c r="E8" s="80" t="s">
+        <v>151</v>
+      </c>
+      <c r="G8" s="79" t="s">
         <v>153</v>
       </c>
-      <c r="D8" s="79" t="s">
+      <c r="H8" s="79" t="s">
         <v>154</v>
-      </c>
-      <c r="E8" s="80" t="s">
-        <v>153</v>
-      </c>
-      <c r="G8" s="79" t="s">
-        <v>155</v>
-      </c>
-      <c r="H8" s="79" t="s">
-        <v>156</v>
       </c>
       <c r="I8" s="79" t="s">
         <v>103</v>
       </c>
       <c r="J8" s="80" t="s">
+        <v>155</v>
+      </c>
+      <c r="K8" s="80" t="s">
+        <v>156</v>
+      </c>
+      <c r="M8" s="80" t="s">
         <v>157</v>
       </c>
-      <c r="K8" s="80" t="s">
+      <c r="N8" s="80" t="s">
         <v>158</v>
-      </c>
-      <c r="M8" s="80" t="s">
-        <v>159</v>
-      </c>
-      <c r="N8" s="80" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A9" s="77" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" s="78" t="s">
+        <v>154</v>
+      </c>
+      <c r="D9" s="77" t="s">
+        <v>160</v>
+      </c>
+      <c r="E9" s="78" t="s">
+        <v>154</v>
+      </c>
+      <c r="G9" s="79" t="s">
         <v>161</v>
-      </c>
-      <c r="B9" s="78" t="s">
-        <v>156</v>
-      </c>
-      <c r="D9" s="77" t="s">
-        <v>162</v>
-      </c>
-      <c r="E9" s="78" t="s">
-        <v>156</v>
-      </c>
-      <c r="G9" s="79" t="s">
-        <v>163</v>
       </c>
       <c r="H9" s="77">
         <v>2</v>
@@ -11419,21 +11562,21 @@
         <v>8</v>
       </c>
       <c r="M9" s="81" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="N9" s="82"/>
     </row>
     <row r="10" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A10" s="77" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B10" s="78" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D10" s="77"/>
       <c r="E10" s="78"/>
       <c r="G10" s="79" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H10" s="77"/>
       <c r="I10" s="77"/>
@@ -11443,7 +11586,7 @@
         <v>0</v>
       </c>
       <c r="M10" s="81" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="N10" s="82"/>
     </row>
@@ -11452,15 +11595,15 @@
       <c r="B11" s="78"/>
       <c r="D11" s="77"/>
       <c r="E11" s="78"/>
-      <c r="G11" s="138" t="s">
-        <v>168</v>
-      </c>
-      <c r="H11" s="138"/>
-      <c r="I11" s="138"/>
-      <c r="J11" s="138"/>
-      <c r="K11" s="138"/>
+      <c r="G11" s="158" t="s">
+        <v>166</v>
+      </c>
+      <c r="H11" s="158"/>
+      <c r="I11" s="158"/>
+      <c r="J11" s="158"/>
+      <c r="K11" s="158"/>
       <c r="M11" s="81" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="N11" s="82"/>
     </row>
@@ -11470,22 +11613,22 @@
       <c r="D12" s="77"/>
       <c r="E12" s="78"/>
       <c r="G12" s="79" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H12" s="79" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="I12" s="79" t="s">
         <v>103</v>
       </c>
       <c r="J12" s="80" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="K12" s="80" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="M12" s="81" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="N12" s="82"/>
     </row>
@@ -11495,7 +11638,7 @@
       <c r="D13" s="77"/>
       <c r="E13" s="78"/>
       <c r="G13" s="79" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H13" s="77">
         <v>1</v>
@@ -11507,11 +11650,11 @@
         <v>3</v>
       </c>
       <c r="M13" s="81" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="N13" s="82"/>
       <c r="W13" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
@@ -11520,7 +11663,7 @@
       <c r="D14" s="77"/>
       <c r="E14" s="78"/>
       <c r="G14" s="79" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H14" s="77"/>
       <c r="I14" s="77"/>
@@ -11530,7 +11673,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="81" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="N14" s="82"/>
     </row>
@@ -11540,7 +11683,7 @@
       <c r="D15" s="77"/>
       <c r="E15" s="78"/>
       <c r="G15" s="79" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H15" s="77">
         <v>1</v>
@@ -11552,7 +11695,7 @@
         <v>3</v>
       </c>
       <c r="M15" s="81" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="N15" s="82"/>
     </row>
@@ -11561,18 +11704,18 @@
       <c r="B16" s="78"/>
       <c r="D16" s="77"/>
       <c r="E16" s="78"/>
-      <c r="G16" s="139" t="s">
-        <v>178</v>
-      </c>
-      <c r="H16" s="139"/>
-      <c r="I16" s="139"/>
-      <c r="J16" s="139"/>
+      <c r="G16" s="159" t="s">
+        <v>176</v>
+      </c>
+      <c r="H16" s="159"/>
+      <c r="I16" s="159"/>
+      <c r="J16" s="159"/>
       <c r="K16" s="83">
         <f>SUM(K9,K10,K13,K14,K15)</f>
         <v>14</v>
       </c>
       <c r="M16" s="81" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="N16" s="82"/>
     </row>
@@ -11582,7 +11725,7 @@
       <c r="D17" s="77"/>
       <c r="E17" s="78"/>
       <c r="M17" s="81" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="N17" s="82"/>
     </row>
@@ -11592,7 +11735,7 @@
       <c r="D18" s="77"/>
       <c r="E18" s="78"/>
       <c r="M18" s="81" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="N18" s="82"/>
     </row>
@@ -11602,7 +11745,7 @@
       <c r="D19" s="77"/>
       <c r="E19" s="78"/>
       <c r="M19" s="81" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="N19" s="82"/>
     </row>
@@ -11612,25 +11755,25 @@
       <c r="D20" s="77"/>
       <c r="E20" s="78"/>
       <c r="M20" s="81" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="N20" s="82"/>
     </row>
     <row r="21" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M21" s="81" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="N21" s="82"/>
     </row>
     <row r="22" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M22" s="81" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="N22" s="82"/>
     </row>
     <row r="23" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M23" s="84" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="N23" s="85">
         <f>SUM(N9:N22)</f>
@@ -11639,7 +11782,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M24" s="84" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="N24" s="83">
         <f>(N23*0.01)+0.65</f>
@@ -11648,7 +11791,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M25" s="84" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="N25" s="86">
         <f>K16*N24</f>
@@ -11657,7 +11800,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M26" s="84" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="N26" s="87">
         <v>19</v>
@@ -11665,7 +11808,7 @@
     </row>
     <row r="27" spans="1:14" ht="21" x14ac:dyDescent="0.3">
       <c r="M27" s="88" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="N27" s="89">
         <f>N25*N26</f>
@@ -11726,46 +11869,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="140" t="s">
+      <c r="A1" s="160" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="140"/>
-      <c r="C1" s="140"/>
-      <c r="D1" s="140"/>
-      <c r="E1" s="140"/>
-      <c r="F1" s="140"/>
-      <c r="G1" s="140"/>
-      <c r="H1" s="140"/>
-      <c r="I1" s="140"/>
-      <c r="J1" s="140"/>
-      <c r="K1" s="140"/>
-      <c r="L1" s="140"/>
-      <c r="M1" s="140"/>
-      <c r="N1" s="140"/>
+      <c r="B1" s="160"/>
+      <c r="C1" s="160"/>
+      <c r="D1" s="160"/>
+      <c r="E1" s="160"/>
+      <c r="F1" s="160"/>
+      <c r="G1" s="160"/>
+      <c r="H1" s="160"/>
+      <c r="I1" s="160"/>
+      <c r="J1" s="160"/>
+      <c r="K1" s="160"/>
+      <c r="L1" s="160"/>
+      <c r="M1" s="160"/>
+      <c r="N1" s="160"/>
     </row>
     <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="146" t="s">
+      <c r="A3" s="166" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="146"/>
-      <c r="C3" s="146"/>
-      <c r="E3" s="146" t="s">
-        <v>191</v>
-      </c>
-      <c r="F3" s="146"/>
-      <c r="G3" s="146"/>
-      <c r="H3" s="146"/>
-      <c r="I3" s="146"/>
-      <c r="J3" s="146"/>
-      <c r="K3" s="146"/>
-      <c r="L3" s="146"/>
-      <c r="M3" s="146"/>
-      <c r="N3" s="146"/>
+      <c r="B3" s="166"/>
+      <c r="C3" s="166"/>
+      <c r="E3" s="166" t="s">
+        <v>189</v>
+      </c>
+      <c r="F3" s="166"/>
+      <c r="G3" s="166"/>
+      <c r="H3" s="166"/>
+      <c r="I3" s="166"/>
+      <c r="J3" s="166"/>
+      <c r="K3" s="166"/>
+      <c r="L3" s="166"/>
+      <c r="M3" s="166"/>
+      <c r="N3" s="166"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="90" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B4" s="91">
         <f>'#Estimativa-APF#'!$N$27</f>
@@ -11774,25 +11917,25 @@
       <c r="C4" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="147" t="s">
-        <v>193</v>
-      </c>
-      <c r="F4" s="145" t="s">
+      <c r="E4" s="167" t="s">
+        <v>191</v>
+      </c>
+      <c r="F4" s="165" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="145"/>
-      <c r="H4" s="145" t="s">
+      <c r="G4" s="165"/>
+      <c r="H4" s="165" t="s">
         <v>31</v>
       </c>
-      <c r="I4" s="145"/>
-      <c r="J4" s="145" t="s">
+      <c r="I4" s="165"/>
+      <c r="J4" s="165" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="145"/>
-      <c r="L4" s="145" t="s">
+      <c r="K4" s="165"/>
+      <c r="L4" s="165" t="s">
         <v>41</v>
       </c>
-      <c r="M4" s="145"/>
+      <c r="M4" s="165"/>
       <c r="N4" s="92"/>
     </row>
     <row r="5" spans="1:14" ht="18" x14ac:dyDescent="0.35">
@@ -11803,32 +11946,32 @@
         <v>0</v>
       </c>
       <c r="C5" s="34" t="s">
-        <v>194</v>
-      </c>
-      <c r="E5" s="147"/>
-      <c r="F5" s="145" t="s">
+        <v>192</v>
+      </c>
+      <c r="E5" s="167"/>
+      <c r="F5" s="165" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="145"/>
-      <c r="H5" s="145" t="s">
+      <c r="G5" s="165"/>
+      <c r="H5" s="165" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="145"/>
-      <c r="J5" s="145" t="s">
+      <c r="I5" s="165"/>
+      <c r="J5" s="165" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="145"/>
-      <c r="L5" s="145" t="s">
+      <c r="K5" s="165"/>
+      <c r="L5" s="165" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="145"/>
+      <c r="M5" s="165"/>
       <c r="N5" s="37" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="93" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B6" s="94">
         <f>B4+(B4*B5)</f>
@@ -11837,7 +11980,7 @@
       <c r="C6" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="147"/>
+      <c r="E6" s="167"/>
       <c r="F6" s="95">
         <f>B6*G6</f>
         <v>8.6450000000000014</v>
@@ -11870,14 +12013,14 @@
     </row>
     <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B7" s="27">
         <v>1</v>
       </c>
       <c r="C7" s="26"/>
       <c r="E7" s="97" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F7" s="95">
         <f>F6*G7</f>
@@ -11914,16 +12057,16 @@
     </row>
     <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B8" s="27">
         <v>40</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E8" s="97" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="F8" s="95">
         <f>F6*G8</f>
@@ -11960,7 +12103,7 @@
     </row>
     <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B9" s="27">
         <v>2</v>
@@ -11969,7 +12112,7 @@
         <v>63</v>
       </c>
       <c r="E9" s="97" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="F9" s="95">
         <f>F6*G9</f>
@@ -12006,7 +12149,7 @@
     </row>
     <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="99" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B10" s="100">
         <f>(B7*B8)*B9</f>
@@ -12016,7 +12159,7 @@
         <v>52</v>
       </c>
       <c r="E10" s="97" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F10" s="95">
         <f>F6*G10</f>
@@ -12053,7 +12196,7 @@
     </row>
     <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="90" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B11" s="101">
         <f>B6/B10*2</f>
@@ -12063,7 +12206,7 @@
         <v>63</v>
       </c>
       <c r="E11" s="97" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F11" s="95">
         <f>F6*G11</f>
@@ -12100,7 +12243,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="90" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B12" s="101">
         <f>B11/4</f>
@@ -12110,7 +12253,7 @@
         <v>65</v>
       </c>
       <c r="E12" s="102" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F12" s="103">
         <f t="shared" ref="F12:M12" si="0">SUM(F7:F11)</f>
@@ -12148,17 +12291,17 @@
     </row>
     <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="99" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B13" s="105">
         <f>B11/B9</f>
         <v>2.1612499999999999</v>
       </c>
       <c r="C13" s="99" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E13" s="97" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F13" s="95">
         <f>F6*G13</f>
@@ -12195,7 +12338,7 @@
     </row>
     <row r="14" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="E14" s="97" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F14" s="95">
         <f>F6*G14</f>
@@ -12232,7 +12375,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E15" s="102" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F15" s="103">
         <f t="shared" ref="F15:M15" si="1">SUM(F13:F14)</f>
@@ -12269,13 +12412,13 @@
       <c r="N15" s="102"/>
     </row>
     <row r="16" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A16" s="146" t="s">
+      <c r="A16" s="166" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="146"/>
-      <c r="C16" s="146"/>
+      <c r="B16" s="166"/>
+      <c r="C16" s="166"/>
       <c r="E16" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F16" s="106">
         <f t="shared" ref="F16:M16" si="2">F12+F15</f>
@@ -12360,7 +12503,7 @@
     </row>
     <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B21" s="110">
         <f>B18+B20</f>
@@ -12391,7 +12534,7 @@
     </row>
     <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B24" s="110">
         <f>B21+B23</f>

</xml_diff>

<commit_message>
doc: alteração dos sprints
Realizada alteração no cronograma dos sprints para adequação com as novas entregas. Feita adequação das horas semanais dos desenvolvedores, gerando mais um sprint.
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/INST360 - Planejamento e Controle do Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/INST360 - Planejamento e Controle do Projeto.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiag\OneDrive\Documentos\GitHub\INST360\6.Gerenciamento de Projeto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eacddf4c3ed15e81/Documentos/GitHub/INST360/6.Gerenciamento de Projeto/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A967EC93-9336-4C19-87ED-FCD4293988F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{A967EC93-9336-4C19-87ED-FCD4293988F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9B217F6-1FF9-4FD7-83F0-91118253A4C5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -4738,7 +4738,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="301">
   <si>
     <t>Equipe</t>
   </si>
@@ -4826,9 +4826,6 @@
   </si>
   <si>
     <t>Planejar o projeto</t>
-  </si>
-  <si>
-    <t>Aplicar Checlist da fase</t>
   </si>
   <si>
     <t>Revisar planejamento</t>
@@ -5635,60 +5632,21 @@
     <t>-</t>
   </si>
   <si>
-    <t>26/03/2026</t>
-  </si>
-  <si>
-    <t>08/04/2026</t>
-  </si>
-  <si>
     <t>1.1</t>
   </si>
   <si>
-    <t>09/04/2026</t>
-  </si>
-  <si>
-    <t>22/04/2026</t>
-  </si>
-  <si>
     <t>1.2</t>
   </si>
   <si>
-    <t>23/04/2026</t>
-  </si>
-  <si>
-    <t>06/05/2026</t>
-  </si>
-  <si>
     <t>1.3</t>
   </si>
   <si>
-    <t>07/05/2026</t>
-  </si>
-  <si>
-    <t>20/05/2026</t>
-  </si>
-  <si>
     <t>1.4</t>
   </si>
   <si>
-    <t>21/05/2026</t>
-  </si>
-  <si>
-    <t>03/06/2026</t>
-  </si>
-  <si>
     <t>2.0</t>
   </si>
   <si>
-    <t>1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 14, 15</t>
-  </si>
-  <si>
-    <t>19, 20, 23, 24, 25, 26</t>
-  </si>
-  <si>
-    <t>37, 38, 39, 40, 45, 46, 47</t>
-  </si>
-  <si>
     <t>Não adoção da aplicação por parte dos envolvidos</t>
   </si>
   <si>
@@ -5749,7 +5707,28 @@
     <t>Redistribuir tarefas entre os membros e concentrar a equipe nas atividades prioritárias</t>
   </si>
   <si>
-    <t>11, 12, 13, 16, 17, 18, 21, 22, 29, 30, 31, 32</t>
+    <t>10 a 15</t>
+  </si>
+  <si>
+    <t>1 a 9</t>
+  </si>
+  <si>
+    <t>45 a 48</t>
+  </si>
+  <si>
+    <t>49 a 53</t>
+  </si>
+  <si>
+    <t>33 a 42</t>
+  </si>
+  <si>
+    <t>25 a 32</t>
+  </si>
+  <si>
+    <t>16 a 24</t>
+  </si>
+  <si>
+    <t>Em execução</t>
   </si>
 </sst>
 </file>
@@ -6056,7 +6035,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -6151,6 +6130,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -6340,7 +6325,7 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="177">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="10" applyProtection="1"/>
     <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6733,6 +6718,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -6749,26 +6746,38 @@
     <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="21" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="30" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="31" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6781,21 +6790,6 @@
     <xf numFmtId="164" fontId="30" fillId="13" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="17" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6826,14 +6820,22 @@
     <xf numFmtId="164" fontId="28" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="164" fontId="23" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="15" borderId="1" xfId="17" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="15" borderId="9" xfId="17" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="42" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -8729,7 +8731,7 @@
     </row>
     <row r="2" spans="1:3" ht="24.6" x14ac:dyDescent="0.3">
       <c r="A2" s="135" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B2" s="135"/>
       <c r="C2" s="135"/>
@@ -8750,10 +8752,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C4" s="111" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -8761,7 +8763,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -8770,10 +8772,10 @@
         <v>6</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C6" s="111" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -8781,10 +8783,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C7" s="111" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -8792,10 +8794,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C8" s="111" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -8803,10 +8805,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C9" s="111" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -8888,38 +8890,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="140" t="s">
+      <c r="A1" s="144" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="140"/>
-      <c r="C1" s="140"/>
-      <c r="D1" s="140"/>
-      <c r="F1" s="141" t="s">
+      <c r="B1" s="144"/>
+      <c r="C1" s="144"/>
+      <c r="D1" s="144"/>
+      <c r="F1" s="136" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="141"/>
-      <c r="H1" s="141"/>
-      <c r="I1" s="141"/>
-      <c r="J1" s="141"/>
-      <c r="K1" s="141"/>
-      <c r="L1" s="141"/>
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="136"/>
+      <c r="J1" s="136"/>
+      <c r="K1" s="136"/>
+      <c r="L1" s="136"/>
     </row>
     <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="142" t="s">
+      <c r="A2" s="137" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="142"/>
-      <c r="C2" s="142"/>
-      <c r="D2" s="142"/>
-      <c r="F2" s="143" t="s">
+      <c r="B2" s="137"/>
+      <c r="C2" s="137"/>
+      <c r="D2" s="137"/>
+      <c r="F2" s="138" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="143"/>
-      <c r="H2" s="143"/>
-      <c r="I2" s="143"/>
-      <c r="J2" s="143"/>
-      <c r="K2" s="143"/>
-      <c r="L2" s="143"/>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="138"/>
+      <c r="J2" s="138"/>
+      <c r="K2" s="138"/>
+      <c r="L2" s="138"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
@@ -8940,20 +8942,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="144" t="s">
+      <c r="H3" s="139" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="144"/>
-      <c r="J3" s="144"/>
-      <c r="K3" s="144"/>
-      <c r="L3" s="144"/>
+      <c r="I3" s="139"/>
+      <c r="J3" s="139"/>
+      <c r="K3" s="139"/>
+      <c r="L3" s="139"/>
     </row>
     <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="136" t="s">
+      <c r="A4" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="136"/>
-      <c r="C4" s="136"/>
+      <c r="B4" s="140"/>
+      <c r="C4" s="140"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -8996,7 +8998,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="123" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H5" s="124">
         <v>8</v>
@@ -9032,7 +9034,7 @@
         <v>2</v>
       </c>
       <c r="G6" s="123" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H6" s="124">
         <v>7</v>
@@ -9068,7 +9070,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="123" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H7" s="124">
         <v>9</v>
@@ -9104,7 +9106,7 @@
         <v>4</v>
       </c>
       <c r="G8" s="123" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H8" s="124">
         <v>10</v>
@@ -9131,7 +9133,7 @@
         <v>16</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="D9" s="13">
         <v>10</v>
@@ -9140,7 +9142,7 @@
         <v>5</v>
       </c>
       <c r="G9" s="123" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H9" s="124">
         <v>10</v>
@@ -9167,7 +9169,7 @@
         <v>16</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D10" s="13">
         <v>2</v>
@@ -9176,7 +9178,7 @@
         <v>6</v>
       </c>
       <c r="G10" s="123" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="H10" s="124">
         <v>7</v>
@@ -9196,11 +9198,11 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="136" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="136"/>
-      <c r="C11" s="136"/>
+      <c r="A11" s="140" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="140"/>
+      <c r="C11" s="140"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>62</v>
@@ -9209,7 +9211,7 @@
         <v>7</v>
       </c>
       <c r="G11" s="123" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="H11" s="124">
         <v>9</v>
@@ -9233,10 +9235,10 @@
         <v>7</v>
       </c>
       <c r="B12" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>31</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>32</v>
       </c>
       <c r="D12" s="13">
         <v>2</v>
@@ -9245,7 +9247,7 @@
         <v>8</v>
       </c>
       <c r="G12" s="123" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="H12" s="124">
         <v>8</v>
@@ -9269,10 +9271,10 @@
         <v>8</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D13" s="13">
         <v>20</v>
@@ -9281,7 +9283,7 @@
         <v>9</v>
       </c>
       <c r="G13" s="123" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="H13" s="124">
         <v>9</v>
@@ -9305,10 +9307,10 @@
         <v>9</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D14" s="13">
         <v>3</v>
@@ -9317,7 +9319,7 @@
         <v>10</v>
       </c>
       <c r="G14" s="123" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H14" s="124">
         <v>8</v>
@@ -9341,10 +9343,10 @@
         <v>10</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" s="117" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D15" s="13">
         <v>7</v>
@@ -9353,7 +9355,7 @@
         <v>11</v>
       </c>
       <c r="G15" s="123" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H15" s="124">
         <v>8</v>
@@ -9377,10 +9379,10 @@
         <v>11</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C16" s="118" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D16" s="13">
         <v>20</v>
@@ -9389,7 +9391,7 @@
         <v>12</v>
       </c>
       <c r="G16" s="123" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="H16" s="124">
         <v>6</v>
@@ -9413,10 +9415,10 @@
         <v>12</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D17" s="13">
         <v>7</v>
@@ -9432,10 +9434,10 @@
         <v>13</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" s="13">
         <v>22</v>
@@ -9451,10 +9453,10 @@
         <v>14</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C19" s="16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D19" s="13">
         <v>4</v>
@@ -9470,10 +9472,10 @@
         <v>15</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D20" s="13">
         <v>7</v>
@@ -9485,11 +9487,11 @@
       <c r="L20" s="17"/>
     </row>
     <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="136" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" s="136"/>
-      <c r="C21" s="137"/>
+      <c r="A21" s="140" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="140"/>
+      <c r="C21" s="141"/>
       <c r="D21" s="113">
         <f>SUM(D12:D20)</f>
         <v>92</v>
@@ -9500,10 +9502,10 @@
         <v>16</v>
       </c>
       <c r="B22" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22" s="115" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D22" s="116">
         <v>4</v>
@@ -9514,10 +9516,10 @@
         <v>17</v>
       </c>
       <c r="B23" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C23" s="115" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D23" s="116">
         <v>4</v>
@@ -9528,10 +9530,10 @@
         <v>18</v>
       </c>
       <c r="B24" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C24" s="115" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D24" s="116">
         <v>12</v>
@@ -9542,10 +9544,10 @@
         <v>19</v>
       </c>
       <c r="B25" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" s="115" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D25" s="116">
         <v>4</v>
@@ -9556,10 +9558,10 @@
         <v>20</v>
       </c>
       <c r="B26" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C26" s="115" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D26" s="116">
         <v>10</v>
@@ -9570,10 +9572,10 @@
         <v>21</v>
       </c>
       <c r="B27" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C27" s="115" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D27" s="116">
         <v>4</v>
@@ -9584,10 +9586,10 @@
         <v>22</v>
       </c>
       <c r="B28" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C28" s="115" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D28" s="116">
         <v>10</v>
@@ -9598,10 +9600,10 @@
         <v>23</v>
       </c>
       <c r="B29" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C29" s="115" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D29" s="116">
         <v>4</v>
@@ -9615,10 +9617,10 @@
         <v>24</v>
       </c>
       <c r="B30" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C30" s="115" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D30" s="116">
         <v>12</v>
@@ -9629,10 +9631,10 @@
         <v>25</v>
       </c>
       <c r="B31" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C31" s="115" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D31" s="116">
         <v>3</v>
@@ -9643,10 +9645,10 @@
         <v>26</v>
       </c>
       <c r="B32" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C32" s="115" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D32" s="116">
         <v>8</v>
@@ -9657,10 +9659,10 @@
         <v>27</v>
       </c>
       <c r="B33" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C33" s="115" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D33" s="116">
         <v>3</v>
@@ -9671,10 +9673,10 @@
         <v>28</v>
       </c>
       <c r="B34" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C34" s="115" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D34" s="116">
         <v>8</v>
@@ -9685,10 +9687,10 @@
         <v>29</v>
       </c>
       <c r="B35" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C35" s="115" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D35" s="116">
         <v>3</v>
@@ -9699,10 +9701,10 @@
         <v>30</v>
       </c>
       <c r="B36" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C36" s="115" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D36" s="116">
         <v>8</v>
@@ -9713,10 +9715,10 @@
         <v>31</v>
       </c>
       <c r="B37" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C37" s="115" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D37" s="116">
         <v>3</v>
@@ -9727,10 +9729,10 @@
         <v>32</v>
       </c>
       <c r="B38" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C38" s="115" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D38" s="116">
         <v>8</v>
@@ -9741,10 +9743,10 @@
         <v>33</v>
       </c>
       <c r="B39" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C39" s="115" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D39" s="116">
         <v>4</v>
@@ -9755,10 +9757,10 @@
         <v>34</v>
       </c>
       <c r="B40" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C40" s="115" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D40" s="116">
         <v>10</v>
@@ -9769,10 +9771,10 @@
         <v>35</v>
       </c>
       <c r="B41" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C41" s="115" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D41" s="116">
         <v>4</v>
@@ -9783,10 +9785,10 @@
         <v>36</v>
       </c>
       <c r="B42" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" s="115" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D42" s="116">
         <v>10</v>
@@ -9797,10 +9799,10 @@
         <v>37</v>
       </c>
       <c r="B43" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C43" s="115" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D43" s="116">
         <v>3</v>
@@ -9811,10 +9813,10 @@
         <v>38</v>
       </c>
       <c r="B44" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" s="115" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D44" s="116">
         <v>8</v>
@@ -9825,10 +9827,10 @@
         <v>39</v>
       </c>
       <c r="B45" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C45" s="115" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D45" s="116">
         <v>3</v>
@@ -9839,10 +9841,10 @@
         <v>40</v>
       </c>
       <c r="B46" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C46" s="115" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D46" s="116">
         <v>8</v>
@@ -9853,10 +9855,10 @@
         <v>41</v>
       </c>
       <c r="B47" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C47" s="115" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D47" s="116">
         <v>3</v>
@@ -9867,21 +9869,21 @@
         <v>42</v>
       </c>
       <c r="B48" s="112" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C48" s="115" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D48" s="116">
         <v>3</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="136" t="s">
-        <v>41</v>
-      </c>
-      <c r="B49" s="136"/>
-      <c r="C49" s="138"/>
+      <c r="A49" s="140" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" s="140"/>
+      <c r="C49" s="142"/>
       <c r="D49" s="121">
         <f>SUM(D22:D48)</f>
         <v>164</v>
@@ -9892,10 +9894,10 @@
         <v>45</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C50" s="119" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D50" s="122">
         <v>3</v>
@@ -9906,10 +9908,10 @@
         <v>46</v>
       </c>
       <c r="B51" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C51" s="120" t="s">
         <v>41</v>
-      </c>
-      <c r="C51" s="120" t="s">
-        <v>42</v>
       </c>
       <c r="D51" s="122">
         <v>6</v>
@@ -9920,10 +9922,10 @@
         <v>47</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C52" s="120" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D52" s="122">
         <v>10</v>
@@ -9934,10 +9936,10 @@
         <v>48</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C53" s="120" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D53" s="122">
         <v>10</v>
@@ -9948,10 +9950,10 @@
         <v>49</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C54" s="119" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D54" s="122">
         <v>5</v>
@@ -9962,10 +9964,10 @@
         <v>50</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C55" s="119" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D55" s="122">
         <v>6</v>
@@ -9976,10 +9978,10 @@
         <v>51</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C56" s="119" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D56" s="122">
         <v>6</v>
@@ -9990,10 +9992,10 @@
         <v>52</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C57" s="119" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D57" s="122">
         <v>5</v>
@@ -10004,19 +10006,19 @@
         <v>53</v>
       </c>
       <c r="B58" s="18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C58" s="120" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D58" s="122">
         <v>3</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="139"/>
-      <c r="B59" s="139"/>
-      <c r="C59" s="139"/>
+      <c r="A59" s="143"/>
+      <c r="B59" s="143"/>
+      <c r="C59" s="143"/>
       <c r="D59" s="114">
         <f>SUM(D50:D58)</f>
         <v>54</v>
@@ -10030,16 +10032,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="F1:L1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="F2:L2"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <phoneticPr fontId="41" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="1.1437007874015752" bottom="1.1437007874015752" header="0.75000000000000011" footer="0.75000000000000011"/>
@@ -10064,7 +10066,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="145" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B1" s="145"/>
       <c r="C1" s="145"/>
@@ -10072,40 +10074,40 @@
     <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="146" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B3" s="146"/>
       <c r="C3" s="146"/>
     </row>
     <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" s="23">
         <f>Backlog_Produto!$D$60</f>
         <v>372</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B5" s="25">
         <v>0.5</v>
       </c>
       <c r="C5" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B6" s="27">
         <v>5</v>
@@ -10114,85 +10116,85 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B7" s="27">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B8" s="28">
         <f>B6*B7*2</f>
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="19.8" x14ac:dyDescent="0.4">
       <c r="A9" s="29" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B9" s="30">
         <f>B11/2</f>
-        <v>5.58</v>
+        <v>6.9749999999999996</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="19.8" x14ac:dyDescent="0.4">
       <c r="A10" s="31" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B10" s="30">
         <f>B4+(B4*B5)</f>
         <v>558</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B11" s="28">
         <f>B10/B8*2</f>
-        <v>11.16</v>
+        <v>13.95</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B12" s="32">
         <f>B11/4</f>
-        <v>2.79</v>
+        <v>3.4874999999999998</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="146" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B14" s="146"/>
       <c r="C14" s="146"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" s="33">
         <v>10</v>
@@ -10201,7 +10203,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B16" s="35">
         <f>B10*B15</f>
@@ -10211,7 +10213,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B17" s="25">
         <v>0.2</v>
@@ -10220,7 +10222,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18" s="36">
         <f>B16*B17</f>
@@ -10230,7 +10232,7 @@
     </row>
     <row r="19" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19" s="38">
         <f>B16+B18</f>
@@ -10240,7 +10242,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B20" s="25">
         <v>0.1</v>
@@ -10249,7 +10251,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B21" s="39">
         <f>B19*B20</f>
@@ -10259,7 +10261,7 @@
     </row>
     <row r="22" spans="1:3" ht="18" x14ac:dyDescent="0.35">
       <c r="A22" s="37" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B22" s="38">
         <f>B19+B21</f>
@@ -10282,7 +10284,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9939D1DA-E220-439A-8C7F-F35A70866D36}">
-  <dimension ref="A1:AMJ12"/>
+  <dimension ref="A1:AMJ13"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.09765625" style="55" customWidth="1"/>
@@ -10298,7 +10300,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="130" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B1" s="130"/>
       <c r="C1" s="130"/>
@@ -10313,7 +10315,7 @@
     </row>
     <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="131" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="131"/>
       <c r="C2" s="131"/>
@@ -10324,7 +10326,7 @@
       </c>
       <c r="F2" s="41"/>
       <c r="G2" s="131" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H2" s="131"/>
       <c r="I2" s="131"/>
@@ -10335,13 +10337,13 @@
       <c r="A3" s="42"/>
       <c r="B3" s="43"/>
       <c r="C3" s="132" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D3" s="132"/>
       <c r="E3" s="132"/>
       <c r="F3" s="44"/>
       <c r="G3" s="133" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H3" s="133"/>
       <c r="I3" s="133"/>
@@ -10350,37 +10352,37 @@
     </row>
     <row r="4" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="45" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="127" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="127" t="s">
+      <c r="C4" s="45" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="45" t="s">
+      <c r="D4" s="45" t="s">
         <v>81</v>
-      </c>
-      <c r="D4" s="45" t="s">
-        <v>82</v>
       </c>
       <c r="E4" s="45" t="s">
         <v>17</v>
       </c>
       <c r="F4" s="45" t="s">
+        <v>82</v>
+      </c>
+      <c r="G4" s="45" t="s">
+        <v>80</v>
+      </c>
+      <c r="H4" s="45" t="s">
         <v>83</v>
-      </c>
-      <c r="G4" s="45" t="s">
-        <v>81</v>
-      </c>
-      <c r="H4" s="45" t="s">
-        <v>84</v>
       </c>
       <c r="I4" s="45" t="s">
         <v>17</v>
       </c>
       <c r="J4" s="48" t="s">
+        <v>84</v>
+      </c>
+      <c r="K4" s="45" t="s">
         <v>85</v>
-      </c>
-      <c r="K4" s="45" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
@@ -10388,34 +10390,34 @@
         <v>1</v>
       </c>
       <c r="B5" s="129" t="s">
-        <v>284</v>
+        <v>294</v>
       </c>
       <c r="C5" s="126" t="s">
+        <v>265</v>
+      </c>
+      <c r="D5" s="124" t="s">
         <v>266</v>
       </c>
-      <c r="D5" s="124" t="s">
+      <c r="E5" s="124">
+        <v>87</v>
+      </c>
+      <c r="F5" s="124" t="s">
+        <v>86</v>
+      </c>
+      <c r="G5" s="124" t="s">
+        <v>265</v>
+      </c>
+      <c r="H5" s="174">
+        <v>46120</v>
+      </c>
+      <c r="I5" s="124">
+        <v>87</v>
+      </c>
+      <c r="J5" s="124" t="s">
         <v>267</v>
       </c>
-      <c r="E5" s="124">
-        <v>24</v>
-      </c>
-      <c r="F5" s="124" t="s">
-        <v>87</v>
-      </c>
-      <c r="G5" s="124" t="s">
-        <v>266</v>
-      </c>
-      <c r="H5" s="124" t="s">
-        <v>267</v>
-      </c>
-      <c r="I5" s="124">
-        <v>24</v>
-      </c>
-      <c r="J5" s="124" t="s">
-        <v>268</v>
-      </c>
       <c r="K5" s="124" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
@@ -10423,26 +10425,26 @@
         <v>2</v>
       </c>
       <c r="B6" s="129" t="s">
-        <v>307</v>
-      </c>
-      <c r="C6" s="126" t="s">
-        <v>269</v>
-      </c>
-      <c r="D6" s="124" t="s">
-        <v>270</v>
+        <v>293</v>
+      </c>
+      <c r="C6" s="175">
+        <v>46121</v>
+      </c>
+      <c r="D6" s="174">
+        <v>46127</v>
       </c>
       <c r="E6" s="124">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="F6" s="124" t="s">
-        <v>88</v>
+        <v>300</v>
       </c>
       <c r="G6" s="124"/>
       <c r="H6" s="124"/>
       <c r="I6" s="124"/>
       <c r="J6" s="124"/>
       <c r="K6" s="124" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
@@ -10450,26 +10452,26 @@
         <v>3</v>
       </c>
       <c r="B7" s="129" t="s">
-        <v>285</v>
-      </c>
-      <c r="C7" s="126" t="s">
-        <v>272</v>
-      </c>
-      <c r="D7" s="124" t="s">
-        <v>273</v>
+        <v>299</v>
+      </c>
+      <c r="C7" s="175">
+        <v>46128</v>
+      </c>
+      <c r="D7" s="174">
+        <v>46141</v>
       </c>
       <c r="E7" s="124">
-        <v>96</v>
+        <v>64</v>
       </c>
       <c r="F7" s="124" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G7" s="124"/>
       <c r="H7" s="124"/>
       <c r="I7" s="124"/>
       <c r="J7" s="124"/>
       <c r="K7" s="124" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
@@ -10477,26 +10479,26 @@
         <v>4</v>
       </c>
       <c r="B8" s="129" t="s">
-        <v>285</v>
-      </c>
-      <c r="C8" s="126" t="s">
-        <v>275</v>
-      </c>
-      <c r="D8" s="124" t="s">
-        <v>276</v>
+        <v>298</v>
+      </c>
+      <c r="C8" s="175">
+        <v>46142</v>
+      </c>
+      <c r="D8" s="174">
+        <v>46155</v>
       </c>
       <c r="E8" s="124">
-        <v>108</v>
+        <v>44</v>
       </c>
       <c r="F8" s="124" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G8" s="124"/>
       <c r="H8" s="124"/>
       <c r="I8" s="124"/>
       <c r="J8" s="124"/>
       <c r="K8" s="124" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
@@ -10504,26 +10506,26 @@
         <v>5</v>
       </c>
       <c r="B9" s="129" t="s">
-        <v>286</v>
-      </c>
-      <c r="C9" s="126" t="s">
-        <v>278</v>
-      </c>
-      <c r="D9" s="124" t="s">
-        <v>279</v>
+        <v>297</v>
+      </c>
+      <c r="C9" s="175">
+        <v>46156</v>
+      </c>
+      <c r="D9" s="174">
+        <v>46169</v>
       </c>
       <c r="E9" s="124">
-        <v>110</v>
+        <v>56</v>
       </c>
       <c r="F9" s="124" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G9" s="124"/>
       <c r="H9" s="124"/>
       <c r="I9" s="124"/>
       <c r="J9" s="124"/>
       <c r="K9" s="124" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
@@ -10531,52 +10533,79 @@
         <v>6</v>
       </c>
       <c r="B10" s="129" t="s">
-        <v>286</v>
-      </c>
-      <c r="C10" s="126" t="s">
-        <v>281</v>
-      </c>
-      <c r="D10" s="124" t="s">
-        <v>282</v>
+        <v>295</v>
+      </c>
+      <c r="C10" s="175">
+        <v>46170</v>
+      </c>
+      <c r="D10" s="174">
+        <v>46183</v>
       </c>
       <c r="E10" s="124">
-        <v>130</v>
+        <v>29</v>
       </c>
       <c r="F10" s="124" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G10" s="124"/>
       <c r="H10" s="124"/>
       <c r="I10" s="124"/>
       <c r="J10" s="124"/>
       <c r="K10" s="124" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="49"/>
-      <c r="B11" s="128"/>
-      <c r="C11" s="51"/>
-      <c r="D11" s="50"/>
-      <c r="E11" s="52">
-        <f>SUM(E5:E10)</f>
-        <v>558</v>
-      </c>
-      <c r="F11" s="50"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
-      <c r="I11" s="52">
+      <c r="A11" s="171">
+        <v>7</v>
+      </c>
+      <c r="B11" s="172" t="s">
+        <v>296</v>
+      </c>
+      <c r="C11" s="176">
+        <v>46184</v>
+      </c>
+      <c r="D11" s="176">
+        <v>46197</v>
+      </c>
+      <c r="E11" s="173">
+        <v>25</v>
+      </c>
+      <c r="F11" s="173" t="s">
+        <v>87</v>
+      </c>
+      <c r="G11" s="173"/>
+      <c r="H11" s="173"/>
+      <c r="I11" s="173"/>
+      <c r="J11" s="173"/>
+      <c r="K11" s="173" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A12" s="49"/>
+      <c r="B12" s="128"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="50"/>
+      <c r="E12" s="52">
+        <f>SUM(E5:E11)</f>
+        <v>372</v>
+      </c>
+      <c r="F12" s="50"/>
+      <c r="G12" s="53"/>
+      <c r="H12" s="53"/>
+      <c r="I12" s="52">
         <f>SUM(I5:I10)</f>
-        <v>24</v>
-      </c>
-      <c r="J11" s="54">
+        <v>87</v>
+      </c>
+      <c r="J12" s="54">
         <f>SUM(J5:J10)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="53"/>
-    </row>
-    <row r="12" spans="1:11" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
-      <c r="J12" s="19"/>
+      <c r="K12" s="53"/>
+    </row>
+    <row r="13" spans="1:11" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+      <c r="J13" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -10679,7 +10708,7 @@
   <sheetData>
     <row r="1" spans="1:11" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="130" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="130"/>
       <c r="C1" s="130"/>
@@ -10695,166 +10724,166 @@
     <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D3" s="58" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D4" s="59" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D5" s="59" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D6" s="59" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D7" s="59" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D8" s="59" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D9" s="59" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D10" s="59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D11" s="59" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D12" s="59" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D13" s="59" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
       <c r="D14" s="58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D15" s="59" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D16" s="59" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D17" s="59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D18" s="58" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D19" s="59" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D20" s="59" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D21" s="59" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D22" s="58" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D23" s="59" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D24" s="59" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D25" s="59" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D26" s="59" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D27" s="58" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="28" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D28" s="59" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D29" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D30" s="59" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="4:4" s="60" customFormat="1" ht="10.199999999999999" hidden="1" x14ac:dyDescent="0.2">
       <c r="D31" s="61" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="D32" s="62" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D33" s="150" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="154" t="s">
-        <v>120</v>
-      </c>
-      <c r="E33" s="154"/>
+      <c r="E33" s="150"/>
     </row>
     <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="D34" s="59">
         <v>4290</v>
       </c>
       <c r="E34" s="59" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
@@ -10862,7 +10891,7 @@
         <v>5082</v>
       </c>
       <c r="E35" s="59" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="36" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
@@ -10870,7 +10899,7 @@
         <v>4356</v>
       </c>
       <c r="E36" s="59" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
@@ -10878,7 +10907,7 @@
         <v>5929</v>
       </c>
       <c r="E37" s="59" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -10886,7 +10915,7 @@
         <v>5005</v>
       </c>
       <c r="E38" s="59" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
@@ -10894,147 +10923,147 @@
         <v>4225</v>
       </c>
       <c r="E39" s="59" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="155" t="s">
+      <c r="A41" s="151" t="s">
+        <v>126</v>
+      </c>
+      <c r="B41" s="151"/>
+      <c r="C41" s="151"/>
+      <c r="D41" s="151"/>
+      <c r="E41" s="151"/>
+      <c r="F41" s="151"/>
+      <c r="G41" s="151"/>
+      <c r="H41" s="151"/>
+      <c r="I41" s="151"/>
+      <c r="J41" s="151"/>
+      <c r="K41" s="151"/>
+    </row>
+    <row r="42" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="152" t="s">
         <v>127</v>
       </c>
-      <c r="B41" s="155"/>
-      <c r="C41" s="155"/>
-      <c r="D41" s="155"/>
-      <c r="E41" s="155"/>
-      <c r="F41" s="155"/>
-      <c r="G41" s="155"/>
-      <c r="H41" s="155"/>
-      <c r="I41" s="155"/>
-      <c r="J41" s="155"/>
-      <c r="K41" s="155"/>
-    </row>
-    <row r="42" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="156" t="s">
+      <c r="B42" s="152"/>
+      <c r="C42" s="152"/>
+      <c r="D42" s="152"/>
+      <c r="E42" s="152"/>
+      <c r="F42" s="152"/>
+      <c r="G42" s="152"/>
+      <c r="H42" s="152"/>
+      <c r="I42" s="152"/>
+      <c r="J42" s="152"/>
+      <c r="K42" s="152"/>
+    </row>
+    <row r="43" spans="1:11" s="56" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="153" t="s">
         <v>128</v>
       </c>
-      <c r="B42" s="156"/>
-      <c r="C42" s="156"/>
-      <c r="D42" s="156"/>
-      <c r="E42" s="156"/>
-      <c r="F42" s="156"/>
-      <c r="G42" s="156"/>
-      <c r="H42" s="156"/>
-      <c r="I42" s="156"/>
-      <c r="J42" s="156"/>
-      <c r="K42" s="156"/>
-    </row>
-    <row r="43" spans="1:11" s="56" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="157" t="s">
+      <c r="B43" s="153"/>
+      <c r="C43" s="153"/>
+      <c r="D43" s="153"/>
+      <c r="E43" s="153"/>
+      <c r="F43" s="153"/>
+      <c r="G43" s="153"/>
+      <c r="H43" s="153"/>
+      <c r="I43" s="153"/>
+      <c r="J43" s="153"/>
+      <c r="K43" s="153"/>
+    </row>
+    <row r="44" spans="1:11" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="149" t="s">
         <v>129</v>
       </c>
-      <c r="B43" s="157"/>
-      <c r="C43" s="157"/>
-      <c r="D43" s="157"/>
-      <c r="E43" s="157"/>
-      <c r="F43" s="157"/>
-      <c r="G43" s="157"/>
-      <c r="H43" s="157"/>
-      <c r="I43" s="157"/>
-      <c r="J43" s="157"/>
-      <c r="K43" s="157"/>
-    </row>
-    <row r="44" spans="1:11" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="153" t="s">
-        <v>130</v>
-      </c>
-      <c r="B44" s="153"/>
-      <c r="C44" s="153"/>
-      <c r="D44" s="153"/>
-      <c r="E44" s="153"/>
-      <c r="F44" s="153"/>
-      <c r="G44" s="153"/>
-      <c r="H44" s="153"/>
-      <c r="I44" s="153"/>
-      <c r="J44" s="153"/>
-      <c r="K44" s="153"/>
+      <c r="B44" s="149"/>
+      <c r="C44" s="149"/>
+      <c r="D44" s="149"/>
+      <c r="E44" s="149"/>
+      <c r="F44" s="149"/>
+      <c r="G44" s="149"/>
+      <c r="H44" s="149"/>
+      <c r="I44" s="149"/>
+      <c r="J44" s="149"/>
+      <c r="K44" s="149"/>
     </row>
     <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="149" t="s">
-        <v>131</v>
-      </c>
-      <c r="B46" s="149"/>
-      <c r="C46" s="149"/>
-      <c r="D46" s="149"/>
-      <c r="E46" s="149"/>
-      <c r="F46" s="149"/>
-      <c r="G46" s="149"/>
-      <c r="H46" s="149"/>
-      <c r="I46" s="149"/>
-      <c r="J46" s="149"/>
-      <c r="K46" s="149"/>
+      <c r="A46" s="157" t="s">
+        <v>130</v>
+      </c>
+      <c r="B46" s="157"/>
+      <c r="C46" s="157"/>
+      <c r="D46" s="157"/>
+      <c r="E46" s="157"/>
+      <c r="F46" s="157"/>
+      <c r="G46" s="157"/>
+      <c r="H46" s="157"/>
+      <c r="I46" s="157"/>
+      <c r="J46" s="157"/>
+      <c r="K46" s="157"/>
     </row>
     <row r="47" spans="1:11" s="65" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="63" t="s">
+        <v>131</v>
+      </c>
+      <c r="B47" s="64"/>
+      <c r="C47" s="158" t="s">
         <v>132</v>
       </c>
-      <c r="B47" s="64"/>
-      <c r="C47" s="150" t="s">
+      <c r="D47" s="158"/>
+      <c r="E47" s="158"/>
+      <c r="F47" s="158"/>
+      <c r="G47" s="158"/>
+      <c r="H47" s="158"/>
+      <c r="I47" s="158"/>
+      <c r="J47" s="158"/>
+      <c r="K47" s="158"/>
+    </row>
+    <row r="48" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="159"/>
+      <c r="B48" s="154" t="s">
         <v>133</v>
       </c>
-      <c r="D47" s="150"/>
-      <c r="E47" s="150"/>
-      <c r="F47" s="150"/>
-      <c r="G47" s="150"/>
-      <c r="H47" s="150"/>
-      <c r="I47" s="150"/>
-      <c r="J47" s="150"/>
-      <c r="K47" s="150"/>
-    </row>
-    <row r="48" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="151"/>
-      <c r="B48" s="147" t="s">
+      <c r="C48" s="154" t="s">
         <v>134</v>
       </c>
-      <c r="C48" s="147" t="s">
+      <c r="D48" s="154" t="s">
         <v>135</v>
       </c>
-      <c r="D48" s="147" t="s">
+      <c r="E48" s="154" t="s">
+        <v>104</v>
+      </c>
+      <c r="F48" s="154" t="s">
         <v>136</v>
       </c>
-      <c r="E48" s="147" t="s">
-        <v>105</v>
-      </c>
-      <c r="F48" s="147" t="s">
+      <c r="G48" s="154" t="s">
+        <v>108</v>
+      </c>
+      <c r="H48" s="160" t="s">
         <v>137</v>
       </c>
-      <c r="G48" s="147" t="s">
-        <v>109</v>
-      </c>
-      <c r="H48" s="152" t="s">
+      <c r="I48" s="160"/>
+      <c r="J48" s="160"/>
+      <c r="K48" s="160"/>
+    </row>
+    <row r="49" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="159"/>
+      <c r="B49" s="154"/>
+      <c r="C49" s="154"/>
+      <c r="D49" s="154"/>
+      <c r="E49" s="154"/>
+      <c r="F49" s="154"/>
+      <c r="G49" s="154"/>
+      <c r="H49" s="154" t="s">
         <v>138</v>
       </c>
-      <c r="I48" s="152"/>
-      <c r="J48" s="152"/>
-      <c r="K48" s="152"/>
-    </row>
-    <row r="49" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="151"/>
-      <c r="B49" s="147"/>
-      <c r="C49" s="147"/>
-      <c r="D49" s="147"/>
-      <c r="E49" s="147"/>
-      <c r="F49" s="147"/>
-      <c r="G49" s="147"/>
-      <c r="H49" s="147" t="s">
+      <c r="I49" s="154"/>
+      <c r="J49" s="66" t="s">
         <v>139</v>
       </c>
-      <c r="I49" s="147"/>
-      <c r="J49" s="66" t="s">
+      <c r="K49" s="66" t="s">
         <v>140</v>
-      </c>
-      <c r="K49" s="66" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:11" s="67" customFormat="1" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -11042,33 +11071,33 @@
         <v>1</v>
       </c>
       <c r="B50" s="69" t="s">
-        <v>287</v>
+        <v>273</v>
       </c>
       <c r="C50" s="70">
         <v>46117</v>
       </c>
       <c r="D50" s="71" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E50" s="71" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F50" s="72" t="str">
         <f t="shared" ref="F50:F60" si="0">IF(OR((CODE($D50)*CODE($E50))=$D$36,(CODE($D50)*CODE($E50))=$D$35),$D$15,IF(OR((CODE($D50)*CODE($E50))=$D$34,(CODE($D50)*CODE($E50))=$D$37),$D$16,IF(OR((CODE($D50)*CODE($E50))=$D$38,(CODE($D50)*CODE($E50))=$D$39),$D$17,0)))</f>
         <v>Alta</v>
       </c>
       <c r="G50" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="H50" s="168" t="s">
-        <v>288</v>
-      </c>
-      <c r="I50" s="168"/>
+        <v>109</v>
+      </c>
+      <c r="H50" s="155" t="s">
+        <v>274</v>
+      </c>
+      <c r="I50" s="155"/>
       <c r="J50" s="73" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="K50" s="73" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
     </row>
     <row r="51" spans="1:11" s="67" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.25">
@@ -11076,33 +11105,33 @@
         <v>2</v>
       </c>
       <c r="B51" s="69" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="C51" s="70">
         <v>46117</v>
       </c>
       <c r="D51" s="71" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E51" s="71" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F51" s="72" t="str">
         <f t="shared" si="0"/>
         <v>Alta</v>
       </c>
       <c r="G51" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="H51" s="169" t="s">
-        <v>292</v>
-      </c>
-      <c r="I51" s="170"/>
+        <v>109</v>
+      </c>
+      <c r="H51" s="147" t="s">
+        <v>278</v>
+      </c>
+      <c r="I51" s="148"/>
       <c r="J51" s="73" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="K51" s="73" t="s">
-        <v>294</v>
+        <v>280</v>
       </c>
     </row>
     <row r="52" spans="1:11" s="67" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.25">
@@ -11110,33 +11139,33 @@
         <v>3</v>
       </c>
       <c r="B52" s="69" t="s">
-        <v>295</v>
+        <v>281</v>
       </c>
       <c r="C52" s="70">
         <v>46117</v>
       </c>
       <c r="D52" s="71" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E52" s="71" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F52" s="72" t="str">
         <f t="shared" si="0"/>
         <v>Alta</v>
       </c>
       <c r="G52" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="H52" s="169" t="s">
-        <v>296</v>
-      </c>
-      <c r="I52" s="170"/>
+        <v>109</v>
+      </c>
+      <c r="H52" s="147" t="s">
+        <v>282</v>
+      </c>
+      <c r="I52" s="148"/>
       <c r="J52" s="73" t="s">
-        <v>297</v>
+        <v>283</v>
       </c>
       <c r="K52" s="73" t="s">
-        <v>298</v>
+        <v>284</v>
       </c>
     </row>
     <row r="53" spans="1:11" s="67" customFormat="1" ht="30.6" x14ac:dyDescent="0.25">
@@ -11144,33 +11173,33 @@
         <v>4</v>
       </c>
       <c r="B53" s="69" t="s">
-        <v>299</v>
+        <v>285</v>
       </c>
       <c r="C53" s="70">
         <v>46117</v>
       </c>
       <c r="D53" s="71" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E53" s="71" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F53" s="72" t="str">
         <f t="shared" si="0"/>
         <v>Média</v>
       </c>
       <c r="G53" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="H53" s="169" t="s">
-        <v>300</v>
-      </c>
-      <c r="I53" s="170"/>
+        <v>109</v>
+      </c>
+      <c r="H53" s="147" t="s">
+        <v>286</v>
+      </c>
+      <c r="I53" s="148"/>
       <c r="J53" s="73" t="s">
-        <v>301</v>
+        <v>287</v>
       </c>
       <c r="K53" s="73" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
     </row>
     <row r="54" spans="1:11" s="67" customFormat="1" ht="30.6" x14ac:dyDescent="0.25">
@@ -11178,33 +11207,33 @@
         <v>5</v>
       </c>
       <c r="B54" s="69" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="C54" s="70">
         <v>46117</v>
       </c>
       <c r="D54" s="71" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E54" s="71" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F54" s="72" t="str">
         <f t="shared" si="0"/>
         <v>Alta</v>
       </c>
       <c r="G54" s="71" t="s">
-        <v>110</v>
-      </c>
-      <c r="H54" s="169" t="s">
-        <v>304</v>
-      </c>
-      <c r="I54" s="170"/>
+        <v>109</v>
+      </c>
+      <c r="H54" s="147" t="s">
+        <v>290</v>
+      </c>
+      <c r="I54" s="148"/>
       <c r="J54" s="73" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="K54" s="73" t="s">
-        <v>306</v>
+        <v>292</v>
       </c>
     </row>
     <row r="55" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -11282,8 +11311,8 @@
         <v>#VALUE!</v>
       </c>
       <c r="G59" s="71"/>
-      <c r="H59" s="148"/>
-      <c r="I59" s="148"/>
+      <c r="H59" s="156"/>
+      <c r="I59" s="156"/>
       <c r="J59" s="73"/>
       <c r="K59" s="73"/>
     </row>
@@ -11298,23 +11327,13 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="71"/>
-      <c r="H60" s="148"/>
-      <c r="I60" s="148"/>
+      <c r="H60" s="156"/>
+      <c r="I60" s="156"/>
       <c r="J60" s="73"/>
       <c r="K60" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
-    <mergeCell ref="H49:I49"/>
-    <mergeCell ref="H50:I50"/>
     <mergeCell ref="H59:I59"/>
     <mergeCell ref="H60:I60"/>
     <mergeCell ref="A46:K46"/>
@@ -11329,6 +11348,16 @@
     <mergeCell ref="H48:K48"/>
     <mergeCell ref="H51:I51"/>
     <mergeCell ref="H52:I52"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="H50:I50"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
     <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="equal">
@@ -11386,167 +11415,167 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="163" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" s="163"/>
+      <c r="C1" s="163"/>
+      <c r="D1" s="163"/>
+      <c r="E1" s="163"/>
+      <c r="F1" s="163"/>
+      <c r="G1" s="163"/>
+      <c r="H1" s="163"/>
+      <c r="I1" s="163"/>
+      <c r="J1" s="163"/>
+      <c r="K1" s="163"/>
+      <c r="L1" s="163"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="163"/>
+    </row>
+    <row r="2" spans="1:23" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="164" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="164"/>
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="F2" s="164"/>
+      <c r="G2" s="164"/>
+      <c r="H2" s="164"/>
+      <c r="I2" s="164"/>
+      <c r="J2" s="164"/>
+      <c r="K2" s="164"/>
+      <c r="L2" s="164"/>
+      <c r="M2" s="164"/>
+      <c r="N2" s="164"/>
+    </row>
+    <row r="3" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="165" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
-      <c r="J1" s="160"/>
-      <c r="K1" s="160"/>
-      <c r="L1" s="160"/>
-      <c r="M1" s="160"/>
-      <c r="N1" s="160"/>
-    </row>
-    <row r="2" spans="1:23" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="161" t="s">
-        <v>127</v>
-      </c>
-      <c r="B2" s="161"/>
-      <c r="C2" s="161"/>
-      <c r="D2" s="161"/>
-      <c r="E2" s="161"/>
-      <c r="F2" s="161"/>
-      <c r="G2" s="161"/>
-      <c r="H2" s="161"/>
-      <c r="I2" s="161"/>
-      <c r="J2" s="161"/>
-      <c r="K2" s="161"/>
-      <c r="L2" s="161"/>
-      <c r="M2" s="161"/>
-      <c r="N2" s="161"/>
-    </row>
-    <row r="3" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="162" t="s">
+      <c r="B3" s="165"/>
+      <c r="C3" s="165"/>
+      <c r="D3" s="165"/>
+      <c r="E3" s="165"/>
+      <c r="F3" s="165"/>
+      <c r="G3" s="165"/>
+      <c r="H3" s="165"/>
+      <c r="I3" s="165"/>
+      <c r="J3" s="165"/>
+      <c r="K3" s="165"/>
+      <c r="L3" s="165"/>
+      <c r="M3" s="165"/>
+      <c r="N3" s="165"/>
+    </row>
+    <row r="4" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="166" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="162"/>
-      <c r="C3" s="162"/>
-      <c r="D3" s="162"/>
-      <c r="E3" s="162"/>
-      <c r="F3" s="162"/>
-      <c r="G3" s="162"/>
-      <c r="H3" s="162"/>
-      <c r="I3" s="162"/>
-      <c r="J3" s="162"/>
-      <c r="K3" s="162"/>
-      <c r="L3" s="162"/>
-      <c r="M3" s="162"/>
-      <c r="N3" s="162"/>
-    </row>
-    <row r="4" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="163" t="s">
+      <c r="B4" s="166"/>
+      <c r="C4" s="166"/>
+      <c r="D4" s="166"/>
+      <c r="E4" s="166"/>
+      <c r="F4" s="166"/>
+      <c r="G4" s="166"/>
+      <c r="H4" s="166"/>
+      <c r="I4" s="166"/>
+      <c r="J4" s="166"/>
+      <c r="K4" s="166"/>
+      <c r="L4" s="166"/>
+      <c r="M4" s="166"/>
+      <c r="N4" s="166"/>
+    </row>
+    <row r="5" spans="1:23" s="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="167" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="163"/>
-      <c r="C4" s="163"/>
-      <c r="D4" s="163"/>
-      <c r="E4" s="163"/>
-      <c r="F4" s="163"/>
-      <c r="G4" s="163"/>
-      <c r="H4" s="163"/>
-      <c r="I4" s="163"/>
-      <c r="J4" s="163"/>
-      <c r="K4" s="163"/>
-      <c r="L4" s="163"/>
-      <c r="M4" s="163"/>
-      <c r="N4" s="163"/>
-    </row>
-    <row r="5" spans="1:23" s="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="164" t="s">
-        <v>145</v>
-      </c>
-      <c r="B5" s="164"/>
-      <c r="C5" s="164"/>
-      <c r="D5" s="164"/>
-      <c r="E5" s="164"/>
-      <c r="F5" s="164"/>
-      <c r="G5" s="164"/>
-      <c r="H5" s="164"/>
-      <c r="I5" s="164"/>
-      <c r="J5" s="164"/>
-      <c r="K5" s="164"/>
-      <c r="L5" s="164"/>
-      <c r="M5" s="164"/>
-      <c r="N5" s="164"/>
+      <c r="B5" s="167"/>
+      <c r="C5" s="167"/>
+      <c r="D5" s="167"/>
+      <c r="E5" s="167"/>
+      <c r="F5" s="167"/>
+      <c r="G5" s="167"/>
+      <c r="H5" s="167"/>
+      <c r="I5" s="167"/>
+      <c r="J5" s="167"/>
+      <c r="K5" s="167"/>
+      <c r="L5" s="167"/>
+      <c r="M5" s="167"/>
+      <c r="N5" s="167"/>
     </row>
     <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="158" t="s">
+      <c r="A7" s="161" t="s">
+        <v>145</v>
+      </c>
+      <c r="B7" s="161"/>
+      <c r="D7" s="161" t="s">
         <v>146</v>
       </c>
-      <c r="B7" s="158"/>
-      <c r="D7" s="158" t="s">
+      <c r="E7" s="161"/>
+      <c r="G7" s="161" t="s">
         <v>147</v>
       </c>
-      <c r="E7" s="158"/>
-      <c r="G7" s="158" t="s">
+      <c r="H7" s="161"/>
+      <c r="I7" s="161"/>
+      <c r="J7" s="161"/>
+      <c r="K7" s="161"/>
+      <c r="M7" s="161" t="s">
         <v>148</v>
       </c>
-      <c r="H7" s="158"/>
-      <c r="I7" s="158"/>
-      <c r="J7" s="158"/>
-      <c r="K7" s="158"/>
-      <c r="M7" s="158" t="s">
-        <v>149</v>
-      </c>
-      <c r="N7" s="158"/>
+      <c r="N7" s="161"/>
     </row>
     <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="B8" s="80" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="80" t="s">
+      <c r="D8" s="79" t="s">
         <v>151</v>
       </c>
-      <c r="D8" s="79" t="s">
+      <c r="E8" s="80" t="s">
+        <v>150</v>
+      </c>
+      <c r="G8" s="79" t="s">
         <v>152</v>
       </c>
-      <c r="E8" s="80" t="s">
-        <v>151</v>
-      </c>
-      <c r="G8" s="79" t="s">
+      <c r="H8" s="79" t="s">
         <v>153</v>
       </c>
-      <c r="H8" s="79" t="s">
+      <c r="I8" s="79" t="s">
+        <v>102</v>
+      </c>
+      <c r="J8" s="80" t="s">
         <v>154</v>
       </c>
-      <c r="I8" s="79" t="s">
-        <v>103</v>
-      </c>
-      <c r="J8" s="80" t="s">
+      <c r="K8" s="80" t="s">
         <v>155</v>
       </c>
-      <c r="K8" s="80" t="s">
+      <c r="M8" s="80" t="s">
         <v>156</v>
       </c>
-      <c r="M8" s="80" t="s">
+      <c r="N8" s="80" t="s">
         <v>157</v>
-      </c>
-      <c r="N8" s="80" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="9" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A9" s="77" t="s">
+        <v>158</v>
+      </c>
+      <c r="B9" s="78" t="s">
+        <v>153</v>
+      </c>
+      <c r="D9" s="77" t="s">
         <v>159</v>
       </c>
-      <c r="B9" s="78" t="s">
-        <v>154</v>
-      </c>
-      <c r="D9" s="77" t="s">
+      <c r="E9" s="78" t="s">
+        <v>153</v>
+      </c>
+      <c r="G9" s="79" t="s">
         <v>160</v>
-      </c>
-      <c r="E9" s="78" t="s">
-        <v>154</v>
-      </c>
-      <c r="G9" s="79" t="s">
-        <v>161</v>
       </c>
       <c r="H9" s="77">
         <v>2</v>
@@ -11562,21 +11591,21 @@
         <v>8</v>
       </c>
       <c r="M9" s="81" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="N9" s="82"/>
     </row>
     <row r="10" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="A10" s="77" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B10" s="78" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D10" s="77"/>
       <c r="E10" s="78"/>
       <c r="G10" s="79" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H10" s="77"/>
       <c r="I10" s="77"/>
@@ -11586,7 +11615,7 @@
         <v>0</v>
       </c>
       <c r="M10" s="81" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N10" s="82"/>
     </row>
@@ -11595,15 +11624,15 @@
       <c r="B11" s="78"/>
       <c r="D11" s="77"/>
       <c r="E11" s="78"/>
-      <c r="G11" s="158" t="s">
+      <c r="G11" s="161" t="s">
+        <v>165</v>
+      </c>
+      <c r="H11" s="161"/>
+      <c r="I11" s="161"/>
+      <c r="J11" s="161"/>
+      <c r="K11" s="161"/>
+      <c r="M11" s="81" t="s">
         <v>166</v>
-      </c>
-      <c r="H11" s="158"/>
-      <c r="I11" s="158"/>
-      <c r="J11" s="158"/>
-      <c r="K11" s="158"/>
-      <c r="M11" s="81" t="s">
-        <v>167</v>
       </c>
       <c r="N11" s="82"/>
     </row>
@@ -11613,22 +11642,22 @@
       <c r="D12" s="77"/>
       <c r="E12" s="78"/>
       <c r="G12" s="79" t="s">
+        <v>152</v>
+      </c>
+      <c r="H12" s="79" t="s">
         <v>153</v>
       </c>
-      <c r="H12" s="79" t="s">
+      <c r="I12" s="79" t="s">
+        <v>102</v>
+      </c>
+      <c r="J12" s="80" t="s">
         <v>154</v>
       </c>
-      <c r="I12" s="79" t="s">
-        <v>103</v>
-      </c>
-      <c r="J12" s="80" t="s">
+      <c r="K12" s="80" t="s">
         <v>155</v>
       </c>
-      <c r="K12" s="80" t="s">
-        <v>156</v>
-      </c>
       <c r="M12" s="81" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="N12" s="82"/>
     </row>
@@ -11638,7 +11667,7 @@
       <c r="D13" s="77"/>
       <c r="E13" s="78"/>
       <c r="G13" s="79" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H13" s="77">
         <v>1</v>
@@ -11650,11 +11679,11 @@
         <v>3</v>
       </c>
       <c r="M13" s="81" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="N13" s="82"/>
       <c r="W13" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
@@ -11663,7 +11692,7 @@
       <c r="D14" s="77"/>
       <c r="E14" s="78"/>
       <c r="G14" s="79" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H14" s="77"/>
       <c r="I14" s="77"/>
@@ -11673,7 +11702,7 @@
         <v>0</v>
       </c>
       <c r="M14" s="81" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="N14" s="82"/>
     </row>
@@ -11683,7 +11712,7 @@
       <c r="D15" s="77"/>
       <c r="E15" s="78"/>
       <c r="G15" s="79" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H15" s="77">
         <v>1</v>
@@ -11695,7 +11724,7 @@
         <v>3</v>
       </c>
       <c r="M15" s="81" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="N15" s="82"/>
     </row>
@@ -11704,18 +11733,18 @@
       <c r="B16" s="78"/>
       <c r="D16" s="77"/>
       <c r="E16" s="78"/>
-      <c r="G16" s="159" t="s">
-        <v>176</v>
-      </c>
-      <c r="H16" s="159"/>
-      <c r="I16" s="159"/>
-      <c r="J16" s="159"/>
+      <c r="G16" s="162" t="s">
+        <v>175</v>
+      </c>
+      <c r="H16" s="162"/>
+      <c r="I16" s="162"/>
+      <c r="J16" s="162"/>
       <c r="K16" s="83">
         <f>SUM(K9,K10,K13,K14,K15)</f>
         <v>14</v>
       </c>
       <c r="M16" s="81" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="N16" s="82"/>
     </row>
@@ -11725,7 +11754,7 @@
       <c r="D17" s="77"/>
       <c r="E17" s="78"/>
       <c r="M17" s="81" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="N17" s="82"/>
     </row>
@@ -11735,7 +11764,7 @@
       <c r="D18" s="77"/>
       <c r="E18" s="78"/>
       <c r="M18" s="81" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="N18" s="82"/>
     </row>
@@ -11745,7 +11774,7 @@
       <c r="D19" s="77"/>
       <c r="E19" s="78"/>
       <c r="M19" s="81" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="N19" s="82"/>
     </row>
@@ -11755,25 +11784,25 @@
       <c r="D20" s="77"/>
       <c r="E20" s="78"/>
       <c r="M20" s="81" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="N20" s="82"/>
     </row>
     <row r="21" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M21" s="81" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="N21" s="82"/>
     </row>
     <row r="22" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M22" s="81" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="N22" s="82"/>
     </row>
     <row r="23" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
       <c r="M23" s="84" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="N23" s="85">
         <f>SUM(N9:N22)</f>
@@ -11782,7 +11811,7 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M24" s="84" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N24" s="83">
         <f>(N23*0.01)+0.65</f>
@@ -11791,7 +11820,7 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M25" s="84" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N25" s="86">
         <f>K16*N24</f>
@@ -11800,7 +11829,7 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M26" s="84" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="N26" s="87">
         <v>19</v>
@@ -11808,7 +11837,7 @@
     </row>
     <row r="27" spans="1:14" ht="21" x14ac:dyDescent="0.3">
       <c r="M27" s="88" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N27" s="89">
         <f>N25*N26</f>
@@ -11869,118 +11898,118 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="160" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="160"/>
-      <c r="J1" s="160"/>
-      <c r="K1" s="160"/>
-      <c r="L1" s="160"/>
-      <c r="M1" s="160"/>
-      <c r="N1" s="160"/>
+      <c r="A1" s="163" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="163"/>
+      <c r="C1" s="163"/>
+      <c r="D1" s="163"/>
+      <c r="E1" s="163"/>
+      <c r="F1" s="163"/>
+      <c r="G1" s="163"/>
+      <c r="H1" s="163"/>
+      <c r="I1" s="163"/>
+      <c r="J1" s="163"/>
+      <c r="K1" s="163"/>
+      <c r="L1" s="163"/>
+      <c r="M1" s="163"/>
+      <c r="N1" s="163"/>
     </row>
     <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="166" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="166"/>
-      <c r="C3" s="166"/>
-      <c r="E3" s="166" t="s">
-        <v>189</v>
-      </c>
-      <c r="F3" s="166"/>
-      <c r="G3" s="166"/>
-      <c r="H3" s="166"/>
-      <c r="I3" s="166"/>
-      <c r="J3" s="166"/>
-      <c r="K3" s="166"/>
-      <c r="L3" s="166"/>
-      <c r="M3" s="166"/>
-      <c r="N3" s="166"/>
+      <c r="A3" s="169" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="169"/>
+      <c r="C3" s="169"/>
+      <c r="E3" s="169" t="s">
+        <v>188</v>
+      </c>
+      <c r="F3" s="169"/>
+      <c r="G3" s="169"/>
+      <c r="H3" s="169"/>
+      <c r="I3" s="169"/>
+      <c r="J3" s="169"/>
+      <c r="K3" s="169"/>
+      <c r="L3" s="169"/>
+      <c r="M3" s="169"/>
+      <c r="N3" s="169"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="90" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B4" s="91">
         <f>'#Estimativa-APF#'!$N$27</f>
         <v>172.9</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="E4" s="167" t="s">
-        <v>191</v>
-      </c>
-      <c r="F4" s="165" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="170" t="s">
+        <v>190</v>
+      </c>
+      <c r="F4" s="168" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="165"/>
-      <c r="H4" s="165" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" s="165"/>
-      <c r="J4" s="165" t="s">
+      <c r="G4" s="168"/>
+      <c r="H4" s="168" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="168"/>
+      <c r="J4" s="168" t="s">
+        <v>39</v>
+      </c>
+      <c r="K4" s="168"/>
+      <c r="L4" s="168" t="s">
         <v>40</v>
       </c>
-      <c r="K4" s="165"/>
-      <c r="L4" s="165" t="s">
-        <v>41</v>
-      </c>
-      <c r="M4" s="165"/>
+      <c r="M4" s="168"/>
       <c r="N4" s="92"/>
     </row>
     <row r="5" spans="1:14" ht="18" x14ac:dyDescent="0.35">
       <c r="A5" s="24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B5" s="25">
         <v>0</v>
       </c>
       <c r="C5" s="34" t="s">
+        <v>191</v>
+      </c>
+      <c r="E5" s="170"/>
+      <c r="F5" s="168" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="168"/>
+      <c r="H5" s="168" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="168"/>
+      <c r="J5" s="168" t="s">
+        <v>17</v>
+      </c>
+      <c r="K5" s="168"/>
+      <c r="L5" s="168" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="168"/>
+      <c r="N5" s="37" t="s">
         <v>192</v>
-      </c>
-      <c r="E5" s="167"/>
-      <c r="F5" s="165" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="165"/>
-      <c r="H5" s="165" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="165"/>
-      <c r="J5" s="165" t="s">
-        <v>17</v>
-      </c>
-      <c r="K5" s="165"/>
-      <c r="L5" s="165" t="s">
-        <v>17</v>
-      </c>
-      <c r="M5" s="165"/>
-      <c r="N5" s="37" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="93" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B6" s="94">
         <f>B4+(B4*B5)</f>
         <v>172.9</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>52</v>
-      </c>
-      <c r="E6" s="167"/>
+        <v>51</v>
+      </c>
+      <c r="E6" s="170"/>
       <c r="F6" s="95">
         <f>B6*G6</f>
         <v>8.6450000000000014</v>
@@ -12013,14 +12042,14 @@
     </row>
     <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="26" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B7" s="27">
         <v>1</v>
       </c>
       <c r="C7" s="26"/>
       <c r="E7" s="97" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F7" s="95">
         <f>F6*G7</f>
@@ -12057,16 +12086,16 @@
     </row>
     <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="26" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B8" s="27">
         <v>40</v>
       </c>
       <c r="C8" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="E8" s="97" t="s">
         <v>198</v>
-      </c>
-      <c r="E8" s="97" t="s">
-        <v>199</v>
       </c>
       <c r="F8" s="95">
         <f>F6*G8</f>
@@ -12103,16 +12132,16 @@
     </row>
     <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="26" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B9" s="27">
         <v>2</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E9" s="97" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F9" s="95">
         <f>F6*G9</f>
@@ -12149,17 +12178,17 @@
     </row>
     <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="99" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B10" s="100">
         <f>(B7*B8)*B9</f>
         <v>80</v>
       </c>
       <c r="C10" s="99" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E10" s="97" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F10" s="95">
         <f>F6*G10</f>
@@ -12196,17 +12225,17 @@
     </row>
     <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="90" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B11" s="101">
         <f>B6/B10*2</f>
         <v>4.3224999999999998</v>
       </c>
       <c r="C11" s="90" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E11" s="97" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F11" s="95">
         <f>F6*G11</f>
@@ -12243,17 +12272,17 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="90" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B12" s="101">
         <f>B11/4</f>
         <v>1.0806249999999999</v>
       </c>
       <c r="C12" s="90" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E12" s="102" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F12" s="103">
         <f t="shared" ref="F12:M12" si="0">SUM(F7:F11)</f>
@@ -12291,17 +12320,17 @@
     </row>
     <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="99" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B13" s="105">
         <f>B11/B9</f>
         <v>2.1612499999999999</v>
       </c>
       <c r="C13" s="99" t="s">
+        <v>208</v>
+      </c>
+      <c r="E13" s="97" t="s">
         <v>209</v>
-      </c>
-      <c r="E13" s="97" t="s">
-        <v>210</v>
       </c>
       <c r="F13" s="95">
         <f>F6*G13</f>
@@ -12338,7 +12367,7 @@
     </row>
     <row r="14" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="E14" s="97" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F14" s="95">
         <f>F6*G14</f>
@@ -12375,7 +12404,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E15" s="102" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F15" s="103">
         <f t="shared" ref="F15:M15" si="1">SUM(F13:F14)</f>
@@ -12412,13 +12441,13 @@
       <c r="N15" s="102"/>
     </row>
     <row r="16" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A16" s="166" t="s">
-        <v>66</v>
-      </c>
-      <c r="B16" s="166"/>
-      <c r="C16" s="166"/>
+      <c r="A16" s="169" t="s">
+        <v>65</v>
+      </c>
+      <c r="B16" s="169"/>
+      <c r="C16" s="169"/>
       <c r="E16" s="37" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F16" s="106">
         <f t="shared" ref="F16:M16" si="2">F12+F15</f>
@@ -12459,7 +12488,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B17" s="109">
         <v>20</v>
@@ -12469,7 +12498,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B18" s="35">
         <f>B6*B17</f>
@@ -12481,7 +12510,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B19" s="25">
         <v>0</v>
@@ -12491,7 +12520,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B20" s="36">
         <f>B18*B19</f>
@@ -12503,7 +12532,7 @@
     </row>
     <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B21" s="110">
         <f>B18+B20</f>
@@ -12514,7 +12543,7 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B22" s="25">
         <v>0.2</v>
@@ -12524,7 +12553,7 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B23" s="39">
         <f>B21*B22</f>
@@ -12534,7 +12563,7 @@
     </row>
     <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B24" s="110">
         <f>B21+B23</f>

</xml_diff>

<commit_message>
Diversas alterações após checklist
Foram feitos os refinamentos finais para os artefatos analisados no checklist de fase de elaboração do spinoff.
</commit_message>
<xml_diff>
--- a/6.Gerenciamento de Projeto/INST360 - Planejamento e Controle do Projeto.xlsx
+++ b/6.Gerenciamento de Projeto/INST360 - Planejamento e Controle do Projeto.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eacddf4c3ed15e81/Documentos/GitHub/INST360/6.Gerenciamento de Projeto/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Desktop\IFSP\Instituto-360\6.Gerenciamento de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="67" documentId="13_ncr:1_{A967EC93-9336-4C19-87ED-FCD4293988F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9B217F6-1FF9-4FD7-83F0-91118253A4C5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{938A6981-0024-4C8B-A706-B8B4E375CE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{31237A52-FFD1-4E1D-B5BB-391D11929C61}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipe" sheetId="1" r:id="rId1"/>
@@ -4738,7 +4738,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="286">
   <si>
     <t>Equipe</t>
   </si>
@@ -5533,36 +5533,12 @@
     <t>Modelar, Implementar e Testar o UC "Validar cadastro"</t>
   </si>
   <si>
-    <t>Modelar o UC "Enviar postagem"</t>
-  </si>
-  <si>
-    <t>Modelar, Implementar e Testar o UC "Enviar postagem"</t>
-  </si>
-  <si>
-    <t>Modelar o UC "Visualizar postagens"</t>
-  </si>
-  <si>
-    <t>Modelar, Implementar e Testar o UC "Visualizar postagens"</t>
-  </si>
-  <si>
-    <t>Modelar o UC "Comentar postagem"</t>
-  </si>
-  <si>
-    <t>Modelar, Implementar e Testar o UC "Comentar postagem"</t>
-  </si>
-  <si>
     <t>Modelar o UC "Realizar login"</t>
   </si>
   <si>
     <t>Modelar, Implementar e Testar o UC "Realizar login"</t>
   </si>
   <si>
-    <t>Modelar o UC "Logar administrador"</t>
-  </si>
-  <si>
-    <t>Modelar, Implementar e Testar o UC "Logar administrador"</t>
-  </si>
-  <si>
     <t>Modelar o UC "Manter postagem"</t>
   </si>
   <si>
@@ -5575,42 +5551,21 @@
     <t>Modelar, Implementar e Testar o UC "Alterar status postagem"</t>
   </si>
   <si>
-    <t>Modelar o UC "Visualizar postagens privadas"</t>
-  </si>
-  <si>
-    <t>Modelar, Implementar e Testar o UC "Visualizar postagens privadas"</t>
-  </si>
-  <si>
     <t>Modelar o UC "Restringir usuário"</t>
   </si>
   <si>
     <t>Modelar, Implementar e Testar o UC "Restringir usuário"</t>
   </si>
   <si>
-    <t>Enviar postagem</t>
-  </si>
-  <si>
-    <t>Visualizar postagens</t>
-  </si>
-  <si>
-    <t>Comentar postagem</t>
-  </si>
-  <si>
     <t>Realizar login</t>
   </si>
   <si>
-    <t>Logar administrador</t>
-  </si>
-  <si>
     <t>Manter postagem</t>
   </si>
   <si>
     <t>Alterar status postagem</t>
   </si>
   <si>
-    <t>Visualizar postagens privadas</t>
-  </si>
-  <si>
     <t>Restringir usuário</t>
   </si>
   <si>
@@ -5713,22 +5668,22 @@
     <t>1 a 9</t>
   </si>
   <si>
-    <t>45 a 48</t>
-  </si>
-  <si>
-    <t>49 a 53</t>
-  </si>
-  <si>
-    <t>33 a 42</t>
-  </si>
-  <si>
-    <t>25 a 32</t>
-  </si>
-  <si>
-    <t>16 a 24</t>
-  </si>
-  <si>
     <t>Em execução</t>
+  </si>
+  <si>
+    <t>16 a 22</t>
+  </si>
+  <si>
+    <t>23 a 26</t>
+  </si>
+  <si>
+    <t>27 a 32</t>
+  </si>
+  <si>
+    <t>33 a 36</t>
+  </si>
+  <si>
+    <t>37 a 41</t>
   </si>
 </sst>
 </file>
@@ -6699,17 +6654,50 @@
     </xf>
     <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="10" applyFont="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="42" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="26" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="23" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="27" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="15" borderId="1" xfId="17" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="15" borderId="9" xfId="17" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="42" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="13" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6718,66 +6706,23 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="6" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="13" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="2" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="21" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="21" fillId="5" borderId="7" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="30" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="26" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="5" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="27" fillId="9" borderId="1" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="31" fillId="5" borderId="3" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -6787,9 +6732,36 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="30" fillId="13" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="30" fillId="13" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="4" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="9" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="30" fillId="9" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="3" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="12" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="17" fillId="11" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -6819,23 +6791,6 @@
     </xf>
     <xf numFmtId="164" fontId="28" fillId="6" borderId="1" xfId="10" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="42" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="15" borderId="1" xfId="17" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="15" borderId="9" xfId="17" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="42" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="18">
@@ -6932,7 +6887,7 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>750960</xdr:colOff>
-      <xdr:row>16</xdr:row>
+      <xdr:row>11</xdr:row>
       <xdr:rowOff>67318</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3725997" cy="1047957"/>
@@ -8713,30 +8668,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6D9A491-4C31-4A24-BC3E-B9501FBB562C}">
   <dimension ref="A1:AMJ17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.59765625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="44.69921875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="21.625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="44.75" style="1" customWidth="1"/>
     <col min="3" max="3" width="29.5" style="1" customWidth="1"/>
-    <col min="4" max="1024" width="8.09765625" style="1" customWidth="1"/>
+    <col min="4" max="1024" width="8.125" style="1" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A1" s="134" t="s">
+    <row r="1" spans="1:3" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="145" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="134"/>
-      <c r="C1" s="134"/>
-    </row>
-    <row r="2" spans="1:3" ht="24.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="135" t="s">
+      <c r="B1" s="145"/>
+      <c r="C1" s="145"/>
+    </row>
+    <row r="2" spans="1:3" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="146" t="s">
         <v>228</v>
       </c>
-      <c r="B2" s="135"/>
-      <c r="C2" s="135"/>
-    </row>
-    <row r="3" spans="1:3" ht="15" x14ac:dyDescent="0.3">
+      <c r="B2" s="146"/>
+      <c r="C2" s="146"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -8747,7 +8702,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -8758,7 +8713,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
@@ -8767,7 +8722,7 @@
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
@@ -8778,7 +8733,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -8789,7 +8744,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -8800,7 +8755,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
@@ -8811,42 +8766,42 @@
         <v>227</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -8872,58 +8827,58 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F6C5642-BF97-4AFF-B370-04CC3D024494}">
-  <dimension ref="A1:AMJ60"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AMJ50"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.19921875" style="19" customWidth="1"/>
-    <col min="2" max="2" width="11.59765625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="64.19921875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="8.69921875" style="17" customWidth="1"/>
-    <col min="5" max="5" width="1.59765625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="4.19921875" style="4" customWidth="1"/>
-    <col min="7" max="7" width="18.8984375" style="4" customWidth="1"/>
+    <col min="1" max="1" width="10.25" style="19" customWidth="1"/>
+    <col min="2" max="2" width="11.625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="64.25" style="4" customWidth="1"/>
+    <col min="4" max="4" width="8.75" style="17" customWidth="1"/>
+    <col min="5" max="5" width="1.625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="4.25" style="4" customWidth="1"/>
+    <col min="7" max="7" width="18.875" style="4" customWidth="1"/>
     <col min="8" max="9" width="8.5" style="4" customWidth="1"/>
-    <col min="10" max="10" width="10.69921875" style="4" customWidth="1"/>
-    <col min="11" max="11" width="11.8984375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="10.75" style="4" customWidth="1"/>
+    <col min="11" max="11" width="11.875" style="4" customWidth="1"/>
     <col min="12" max="1024" width="8.5" style="4" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="144" t="s">
+    <row r="1" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="140" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="144"/>
-      <c r="C1" s="144"/>
-      <c r="D1" s="144"/>
-      <c r="F1" s="136" t="s">
+      <c r="B1" s="140"/>
+      <c r="C1" s="140"/>
+      <c r="D1" s="140"/>
+      <c r="F1" s="141" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="136"/>
-      <c r="H1" s="136"/>
-      <c r="I1" s="136"/>
-      <c r="J1" s="136"/>
-      <c r="K1" s="136"/>
-      <c r="L1" s="136"/>
-    </row>
-    <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="137" t="s">
+      <c r="G1" s="141"/>
+      <c r="H1" s="141"/>
+      <c r="I1" s="141"/>
+      <c r="J1" s="141"/>
+      <c r="K1" s="141"/>
+      <c r="L1" s="141"/>
+    </row>
+    <row r="2" spans="1:12" ht="42" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="142" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="137"/>
-      <c r="C2" s="137"/>
-      <c r="D2" s="137"/>
-      <c r="F2" s="138" t="s">
+      <c r="B2" s="142"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="F2" s="143" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="138"/>
-      <c r="H2" s="138"/>
-      <c r="I2" s="138"/>
-      <c r="J2" s="138"/>
-      <c r="K2" s="138"/>
-      <c r="L2" s="138"/>
-    </row>
-    <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="143"/>
+      <c r="H2" s="143"/>
+      <c r="I2" s="143"/>
+      <c r="J2" s="143"/>
+      <c r="K2" s="143"/>
+      <c r="L2" s="143"/>
+    </row>
+    <row r="3" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>11</v>
       </c>
@@ -8942,20 +8897,20 @@
       <c r="G3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="139" t="s">
+      <c r="H3" s="144" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="139"/>
-      <c r="J3" s="139"/>
-      <c r="K3" s="139"/>
-      <c r="L3" s="139"/>
-    </row>
-    <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="140" t="s">
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
+    </row>
+    <row r="4" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="136" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="140"/>
-      <c r="C4" s="140"/>
+      <c r="B4" s="136"/>
+      <c r="C4" s="136"/>
       <c r="D4" s="8" t="s">
         <v>17</v>
       </c>
@@ -8981,7 +8936,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="10">
         <v>1</v>
       </c>
@@ -8998,7 +8953,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="123" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="H5" s="124">
         <v>8</v>
@@ -9017,7 +8972,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="10">
         <v>2</v>
       </c>
@@ -9034,7 +8989,7 @@
         <v>2</v>
       </c>
       <c r="G6" s="123" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="H6" s="124">
         <v>7</v>
@@ -9053,7 +9008,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="10">
         <v>3</v>
       </c>
@@ -9070,7 +9025,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="123" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="H7" s="124">
         <v>9</v>
@@ -9089,7 +9044,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="10">
         <v>4</v>
       </c>
@@ -9106,26 +9061,26 @@
         <v>4</v>
       </c>
       <c r="G8" s="123" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="H8" s="124">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I8" s="124">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="124">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K8" s="124">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L8" s="15">
-        <f t="shared" ref="L8:L16" si="0">SUM(H8:K8)</f>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+        <f t="shared" ref="L8:L11" si="0">SUM(H8:K8)</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="10">
         <v>5</v>
       </c>
@@ -9142,26 +9097,26 @@
         <v>5</v>
       </c>
       <c r="G9" s="123" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="H9" s="124">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I9" s="124">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="124">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K9" s="124">
         <v>4</v>
       </c>
       <c r="L9" s="15">
         <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.2">
       <c r="A10" s="10">
         <v>6</v>
       </c>
@@ -9178,31 +9133,31 @@
         <v>6</v>
       </c>
       <c r="G10" s="123" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="H10" s="124">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I10" s="124">
         <v>2</v>
       </c>
       <c r="J10" s="124">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K10" s="124">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L10" s="15">
         <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="140" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="136" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="140"/>
-      <c r="C11" s="140"/>
+      <c r="B11" s="136"/>
+      <c r="C11" s="136"/>
       <c r="D11" s="8">
         <f>SUM(D5:D10)</f>
         <v>62</v>
@@ -9211,26 +9166,26 @@
         <v>7</v>
       </c>
       <c r="G11" s="123" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="H11" s="124">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="I11" s="124">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J11" s="124">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K11" s="124">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L11" s="15">
         <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="10">
         <v>7</v>
       </c>
@@ -9243,30 +9198,13 @@
       <c r="D12" s="13">
         <v>2</v>
       </c>
-      <c r="F12" s="14">
-        <v>8</v>
-      </c>
-      <c r="G12" s="123" t="s">
-        <v>257</v>
-      </c>
-      <c r="H12" s="124">
-        <v>8</v>
-      </c>
-      <c r="I12" s="124">
-        <v>1</v>
-      </c>
-      <c r="J12" s="124">
-        <v>8</v>
-      </c>
-      <c r="K12" s="124">
-        <v>3</v>
-      </c>
-      <c r="L12" s="15">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+      <c r="L12" s="17"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="10">
         <v>8</v>
       </c>
@@ -9279,30 +9217,13 @@
       <c r="D13" s="13">
         <v>20</v>
       </c>
-      <c r="F13" s="14">
-        <v>9</v>
-      </c>
-      <c r="G13" s="123" t="s">
-        <v>258</v>
-      </c>
-      <c r="H13" s="124">
-        <v>9</v>
-      </c>
-      <c r="I13" s="124">
-        <v>2</v>
-      </c>
-      <c r="J13" s="124">
-        <v>7</v>
-      </c>
-      <c r="K13" s="124">
-        <v>4</v>
-      </c>
-      <c r="L13" s="15">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+      <c r="L13" s="17"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="10">
         <v>9</v>
       </c>
@@ -9315,30 +9236,13 @@
       <c r="D14" s="13">
         <v>3</v>
       </c>
-      <c r="F14" s="14">
-        <v>10</v>
-      </c>
-      <c r="G14" s="123" t="s">
-        <v>259</v>
-      </c>
-      <c r="H14" s="124">
-        <v>8</v>
-      </c>
-      <c r="I14" s="124">
-        <v>2</v>
-      </c>
-      <c r="J14" s="124">
-        <v>8</v>
-      </c>
-      <c r="K14" s="124">
-        <v>4</v>
-      </c>
-      <c r="L14" s="15">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="28.8" x14ac:dyDescent="0.25">
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="L14" s="17"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="10">
         <v>10</v>
       </c>
@@ -9351,30 +9255,13 @@
       <c r="D15" s="13">
         <v>7</v>
       </c>
-      <c r="F15" s="14">
-        <v>11</v>
-      </c>
-      <c r="G15" s="123" t="s">
-        <v>260</v>
-      </c>
-      <c r="H15" s="124">
-        <v>8</v>
-      </c>
-      <c r="I15" s="124">
-        <v>2</v>
-      </c>
-      <c r="J15" s="124">
-        <v>6</v>
-      </c>
-      <c r="K15" s="124">
-        <v>4</v>
-      </c>
-      <c r="L15" s="15">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+    </row>
+    <row r="16" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="10">
         <v>11</v>
       </c>
@@ -9387,30 +9274,8 @@
       <c r="D16" s="13">
         <v>20</v>
       </c>
-      <c r="F16" s="14">
-        <v>12</v>
-      </c>
-      <c r="G16" s="123" t="s">
-        <v>261</v>
-      </c>
-      <c r="H16" s="124">
-        <v>6</v>
-      </c>
-      <c r="I16" s="124">
-        <v>3</v>
-      </c>
-      <c r="J16" s="124">
-        <v>4</v>
-      </c>
-      <c r="K16" s="124">
-        <v>4</v>
-      </c>
-      <c r="L16" s="15">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="10">
         <v>12</v>
       </c>
@@ -9423,13 +9288,8 @@
       <c r="D17" s="13">
         <v>7</v>
       </c>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="10">
         <v>13</v>
       </c>
@@ -9442,13 +9302,8 @@
       <c r="D18" s="13">
         <v>22</v>
       </c>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="10">
         <v>14</v>
       </c>
@@ -9461,13 +9316,8 @@
       <c r="D19" s="13">
         <v>4</v>
       </c>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="10">
         <v>15</v>
       </c>
@@ -9480,24 +9330,19 @@
       <c r="D20" s="13">
         <v>7</v>
       </c>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-    </row>
-    <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="140" t="s">
+    </row>
+    <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="136" t="s">
         <v>39</v>
       </c>
-      <c r="B21" s="140"/>
-      <c r="C21" s="141"/>
+      <c r="B21" s="136"/>
+      <c r="C21" s="137"/>
       <c r="D21" s="113">
         <f>SUM(D12:D20)</f>
         <v>92</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="10">
         <v>16</v>
       </c>
@@ -9508,10 +9353,10 @@
         <v>31</v>
       </c>
       <c r="D22" s="116">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A23" s="10">
         <v>17</v>
       </c>
@@ -9522,10 +9367,10 @@
         <v>229</v>
       </c>
       <c r="D23" s="116">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A24" s="10">
         <v>18</v>
       </c>
@@ -9536,10 +9381,10 @@
         <v>230</v>
       </c>
       <c r="D24" s="116">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="10">
         <v>19</v>
       </c>
@@ -9550,10 +9395,10 @@
         <v>231</v>
       </c>
       <c r="D25" s="116">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="10">
         <v>20</v>
       </c>
@@ -9564,10 +9409,10 @@
         <v>232</v>
       </c>
       <c r="D26" s="116">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A27" s="10">
         <v>21</v>
       </c>
@@ -9578,10 +9423,10 @@
         <v>233</v>
       </c>
       <c r="D27" s="116">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A28" s="10">
         <v>22</v>
       </c>
@@ -9592,10 +9437,10 @@
         <v>234</v>
       </c>
       <c r="D28" s="116">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A29" s="10">
         <v>23</v>
       </c>
@@ -9606,13 +9451,10 @@
         <v>235</v>
       </c>
       <c r="D29" s="116">
-        <v>4</v>
-      </c>
-      <c r="H29" s="4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A30" s="10">
         <v>24</v>
       </c>
@@ -9623,10 +9465,10 @@
         <v>236</v>
       </c>
       <c r="D30" s="116">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A31" s="10">
         <v>25</v>
       </c>
@@ -9637,10 +9479,10 @@
         <v>237</v>
       </c>
       <c r="D31" s="116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A32" s="10">
         <v>26</v>
       </c>
@@ -9651,10 +9493,10 @@
         <v>238</v>
       </c>
       <c r="D32" s="116">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A33" s="10">
         <v>27</v>
       </c>
@@ -9665,10 +9507,10 @@
         <v>239</v>
       </c>
       <c r="D33" s="116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A34" s="10">
         <v>28</v>
       </c>
@@ -9679,10 +9521,10 @@
         <v>240</v>
       </c>
       <c r="D34" s="116">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A35" s="10">
         <v>29</v>
       </c>
@@ -9693,10 +9535,10 @@
         <v>241</v>
       </c>
       <c r="D35" s="116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A36" s="10">
         <v>30</v>
       </c>
@@ -9707,10 +9549,10 @@
         <v>242</v>
       </c>
       <c r="D36" s="116">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A37" s="10">
         <v>31</v>
       </c>
@@ -9718,13 +9560,13 @@
         <v>39</v>
       </c>
       <c r="C37" s="115" t="s">
-        <v>243</v>
+        <v>37</v>
       </c>
       <c r="D37" s="116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A38" s="10">
         <v>32</v>
       </c>
@@ -9732,316 +9574,176 @@
         <v>39</v>
       </c>
       <c r="C38" s="115" t="s">
-        <v>244</v>
+        <v>38</v>
       </c>
       <c r="D38" s="116">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A39" s="10">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="136" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="136"/>
+      <c r="C39" s="138"/>
+      <c r="D39" s="121">
+        <f>SUM(D22:D38)</f>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A40" s="10">
         <v>33</v>
       </c>
-      <c r="B39" s="112" t="s">
+      <c r="B40" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C40" s="119" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" s="122">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A41" s="10">
+        <v>34</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C41" s="120" t="s">
+        <v>41</v>
+      </c>
+      <c r="D41" s="122">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A42" s="10">
+        <v>35</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C42" s="120" t="s">
+        <v>42</v>
+      </c>
+      <c r="D42" s="122">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A43" s="10">
+        <v>36</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C43" s="120" t="s">
+        <v>43</v>
+      </c>
+      <c r="D43" s="122">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A44" s="10">
+        <v>37</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C44" s="119" t="s">
+        <v>44</v>
+      </c>
+      <c r="D44" s="122">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A45" s="10">
+        <v>38</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C45" s="119" t="s">
+        <v>45</v>
+      </c>
+      <c r="D45" s="122">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A46" s="10">
         <v>39</v>
       </c>
-      <c r="C39" s="115" t="s">
-        <v>245</v>
-      </c>
-      <c r="D39" s="116">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A40" s="10">
-        <v>34</v>
-      </c>
-      <c r="B40" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C40" s="115" t="s">
-        <v>246</v>
-      </c>
-      <c r="D40" s="116">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A41" s="10">
-        <v>35</v>
-      </c>
-      <c r="B41" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C41" s="115" t="s">
-        <v>247</v>
-      </c>
-      <c r="D41" s="116">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A42" s="10">
-        <v>36</v>
-      </c>
-      <c r="B42" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C42" s="115" t="s">
-        <v>248</v>
-      </c>
-      <c r="D42" s="116">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A43" s="10">
+      <c r="B46" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C46" s="119" t="s">
+        <v>46</v>
+      </c>
+      <c r="D46" s="122">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A47" s="10">
+        <v>40</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C47" s="119" t="s">
+        <v>47</v>
+      </c>
+      <c r="D47" s="122">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A48" s="10">
+        <v>41</v>
+      </c>
+      <c r="B48" s="18" t="s">
+        <v>40</v>
+      </c>
+      <c r="C48" s="120" t="s">
         <v>37</v>
       </c>
-      <c r="B43" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C43" s="115" t="s">
-        <v>249</v>
-      </c>
-      <c r="D43" s="116">
+      <c r="D48" s="122">
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A44" s="10">
-        <v>38</v>
-      </c>
-      <c r="B44" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C44" s="115" t="s">
-        <v>250</v>
-      </c>
-      <c r="D44" s="116">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A45" s="10">
-        <v>39</v>
-      </c>
-      <c r="B45" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C45" s="115" t="s">
-        <v>251</v>
-      </c>
-      <c r="D45" s="116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A46" s="10">
-        <v>40</v>
-      </c>
-      <c r="B46" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C46" s="115" t="s">
-        <v>252</v>
-      </c>
-      <c r="D46" s="116">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A47" s="10">
-        <v>41</v>
-      </c>
-      <c r="B47" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C47" s="115" t="s">
-        <v>37</v>
-      </c>
-      <c r="D47" s="116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A48" s="10">
-        <v>42</v>
-      </c>
-      <c r="B48" s="112" t="s">
-        <v>39</v>
-      </c>
-      <c r="C48" s="115" t="s">
-        <v>38</v>
-      </c>
-      <c r="D48" s="116">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="140" t="s">
-        <v>40</v>
-      </c>
-      <c r="B49" s="140"/>
-      <c r="C49" s="142"/>
-      <c r="D49" s="121">
-        <f>SUM(D22:D48)</f>
-        <v>164</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A50" s="10">
-        <v>45</v>
-      </c>
-      <c r="B50" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C50" s="119" t="s">
-        <v>31</v>
-      </c>
-      <c r="D50" s="122">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A51" s="10">
-        <v>46</v>
-      </c>
-      <c r="B51" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C51" s="120" t="s">
-        <v>41</v>
-      </c>
-      <c r="D51" s="122">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A52" s="10">
-        <v>47</v>
-      </c>
-      <c r="B52" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C52" s="120" t="s">
-        <v>42</v>
-      </c>
-      <c r="D52" s="122">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A53" s="10">
-        <v>48</v>
-      </c>
-      <c r="B53" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C53" s="120" t="s">
-        <v>43</v>
-      </c>
-      <c r="D53" s="122">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A54" s="10">
-        <v>49</v>
-      </c>
-      <c r="B54" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C54" s="119" t="s">
-        <v>44</v>
-      </c>
-      <c r="D54" s="122">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A55" s="10">
-        <v>50</v>
-      </c>
-      <c r="B55" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C55" s="119" t="s">
-        <v>45</v>
-      </c>
-      <c r="D55" s="122">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A56" s="10">
-        <v>51</v>
-      </c>
-      <c r="B56" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C56" s="119" t="s">
-        <v>46</v>
-      </c>
-      <c r="D56" s="122">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A57" s="10">
-        <v>52</v>
-      </c>
-      <c r="B57" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C57" s="119" t="s">
-        <v>47</v>
-      </c>
-      <c r="D57" s="122">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A58" s="10">
-        <v>53</v>
-      </c>
-      <c r="B58" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C58" s="120" t="s">
-        <v>37</v>
-      </c>
-      <c r="D58" s="122">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="143"/>
-      <c r="B59" s="143"/>
-      <c r="C59" s="143"/>
-      <c r="D59" s="114">
-        <f>SUM(D50:D58)</f>
+    <row r="49" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="139"/>
+      <c r="B49" s="139"/>
+      <c r="C49" s="139"/>
+      <c r="D49" s="114">
+        <f>SUM(D40:D48)</f>
         <v>54</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="D60" s="20">
-        <f>SUM(D11,D21,D49,D59)</f>
-        <v>372</v>
+    <row r="50" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="D50" s="20">
+        <f>SUM(D11,D21,D39,D49)</f>
+        <v>371</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A1:D1"/>
     <mergeCell ref="F1:L1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="F2:L2"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <phoneticPr fontId="41" type="noConversion"/>
   <pageMargins left="0.70000000000000007" right="0.70000000000000007" top="1.1437007874015752" bottom="1.1437007874015752" header="0.75000000000000011" footer="0.75000000000000011"/>
@@ -10055,43 +9757,43 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12CD3DDD-A46C-49EB-857E-53C854C2AEB1}">
   <dimension ref="A1:AMJ22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.19921875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="48.25" style="1" customWidth="1"/>
     <col min="2" max="2" width="15.5" style="21" customWidth="1"/>
-    <col min="3" max="3" width="20.69921875" style="1" customWidth="1"/>
-    <col min="4" max="1024" width="8.09765625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.75" style="1" customWidth="1"/>
+    <col min="4" max="1024" width="8.125" style="1" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="145" t="s">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="147" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="145"/>
-      <c r="C1" s="145"/>
-    </row>
-    <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="146" t="s">
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+    </row>
+    <row r="2" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="148" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="146"/>
-      <c r="C3" s="146"/>
-    </row>
-    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B3" s="148"/>
+      <c r="C3" s="148"/>
+    </row>
+    <row r="4" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
         <v>50</v>
       </c>
       <c r="B4" s="23">
-        <f>Backlog_Produto!$D$60</f>
-        <v>372</v>
+        <f>Backlog_Produto!$D$50</f>
+        <v>371</v>
       </c>
       <c r="C4" s="22" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
         <v>52</v>
       </c>
@@ -10105,7 +9807,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
         <v>55</v>
       </c>
@@ -10114,7 +9816,7 @@
       </c>
       <c r="C6" s="26"/>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>56</v>
       </c>
@@ -10125,7 +9827,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>57</v>
       </c>
@@ -10137,62 +9839,62 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="19.8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:5" ht="19.5" x14ac:dyDescent="0.3">
       <c r="A9" s="29" t="s">
         <v>58</v>
       </c>
       <c r="B9" s="30">
         <f>B11/2</f>
-        <v>6.9749999999999996</v>
+        <v>6.9562499999999998</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="19.8" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:5" ht="19.5" x14ac:dyDescent="0.3">
       <c r="A10" s="31" t="s">
         <v>60</v>
       </c>
       <c r="B10" s="30">
         <f>B4+(B4*B5)</f>
-        <v>558</v>
+        <v>556.5</v>
       </c>
       <c r="C10" s="31" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
         <v>61</v>
       </c>
       <c r="B11" s="28">
         <f>B10/B8*2</f>
-        <v>13.95</v>
+        <v>13.9125</v>
       </c>
       <c r="C11" s="26" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
         <v>63</v>
       </c>
       <c r="B12" s="32">
         <f>B11/4</f>
-        <v>3.4874999999999998</v>
+        <v>3.4781249999999999</v>
       </c>
       <c r="C12" s="22" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="146" t="s">
+    <row r="14" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="148" t="s">
         <v>65</v>
       </c>
-      <c r="B14" s="146"/>
-      <c r="C14" s="146"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B14" s="148"/>
+      <c r="C14" s="148"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
         <v>66</v>
       </c>
@@ -10201,17 +9903,17 @@
       </c>
       <c r="C15" s="34"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
         <v>67</v>
       </c>
       <c r="B16" s="35">
         <f>B10*B15</f>
-        <v>5580</v>
+        <v>5565</v>
       </c>
       <c r="C16" s="34"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
         <v>68</v>
       </c>
@@ -10220,27 +9922,27 @@
       </c>
       <c r="C17" s="34"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
         <v>69</v>
       </c>
       <c r="B18" s="36">
         <f>B16*B17</f>
-        <v>1116</v>
+        <v>1113</v>
       </c>
       <c r="C18" s="34"/>
     </row>
-    <row r="19" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A19" s="37" t="s">
         <v>70</v>
       </c>
       <c r="B19" s="38">
         <f>B16+B18</f>
-        <v>6696</v>
+        <v>6678</v>
       </c>
       <c r="C19" s="34"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
         <v>71</v>
       </c>
@@ -10249,23 +9951,23 @@
       </c>
       <c r="C20" s="34"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="26" t="s">
         <v>72</v>
       </c>
       <c r="B21" s="39">
         <f>B19*B20</f>
-        <v>669.6</v>
+        <v>667.80000000000007</v>
       </c>
       <c r="C21" s="34"/>
     </row>
-    <row r="22" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A22" s="37" t="s">
         <v>73</v>
       </c>
       <c r="B22" s="38">
         <f>B19+B21</f>
-        <v>7365.6</v>
+        <v>7345.8</v>
       </c>
       <c r="C22" s="34"/>
     </row>
@@ -10285,72 +9987,72 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9939D1DA-E220-439A-8C7F-F35A70866D36}">
   <dimension ref="A1:AMJ13"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6.09765625" style="55" customWidth="1"/>
-    <col min="2" max="2" width="45.19921875" style="4" customWidth="1"/>
-    <col min="3" max="3" width="13.8984375" style="55" customWidth="1"/>
-    <col min="4" max="6" width="13.09765625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="6.125" style="55" customWidth="1"/>
+    <col min="2" max="2" width="45.25" style="4" customWidth="1"/>
+    <col min="3" max="3" width="13.875" style="55" customWidth="1"/>
+    <col min="4" max="6" width="13.125" style="4" customWidth="1"/>
     <col min="7" max="9" width="13" style="4" customWidth="1"/>
     <col min="10" max="10" width="13" style="19" customWidth="1"/>
-    <col min="11" max="11" width="14.69921875" style="4" customWidth="1"/>
+    <col min="11" max="11" width="14.75" style="4" customWidth="1"/>
     <col min="12" max="1024" width="8.5" style="4" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="130" t="s">
+    <row r="1" spans="1:11" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="A1" s="149" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
-      <c r="F1" s="130"/>
-      <c r="G1" s="130"/>
-      <c r="H1" s="130"/>
-      <c r="I1" s="130"/>
-      <c r="J1" s="130"/>
-      <c r="K1" s="130"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="131" t="s">
+      <c r="B1" s="149"/>
+      <c r="C1" s="149"/>
+      <c r="D1" s="149"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="150" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="131"/>
-      <c r="C2" s="131"/>
-      <c r="D2" s="131"/>
+      <c r="B2" s="150"/>
+      <c r="C2" s="150"/>
+      <c r="D2" s="150"/>
       <c r="E2" s="40">
         <f>Planejamento!$B$10</f>
-        <v>558</v>
+        <v>556.5</v>
       </c>
       <c r="F2" s="41"/>
-      <c r="G2" s="131" t="s">
+      <c r="G2" s="150" t="s">
         <v>75</v>
       </c>
-      <c r="H2" s="131"/>
-      <c r="I2" s="131"/>
-      <c r="J2" s="131"/>
+      <c r="H2" s="150"/>
+      <c r="I2" s="150"/>
+      <c r="J2" s="150"/>
       <c r="K2" s="40"/>
     </row>
-    <row r="3" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="42"/>
       <c r="B3" s="43"/>
-      <c r="C3" s="132" t="s">
+      <c r="C3" s="151" t="s">
         <v>76</v>
       </c>
-      <c r="D3" s="132"/>
-      <c r="E3" s="132"/>
+      <c r="D3" s="151"/>
+      <c r="E3" s="151"/>
       <c r="F3" s="44"/>
-      <c r="G3" s="133" t="s">
+      <c r="G3" s="152" t="s">
         <v>77</v>
       </c>
-      <c r="H3" s="133"/>
-      <c r="I3" s="133"/>
+      <c r="H3" s="152"/>
+      <c r="I3" s="152"/>
       <c r="J3" s="46"/>
       <c r="K3" s="47"/>
     </row>
-    <row r="4" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="45" t="s">
         <v>78</v>
       </c>
@@ -10385,18 +10087,18 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="125">
         <v>1</v>
       </c>
       <c r="B5" s="129" t="s">
-        <v>294</v>
+        <v>279</v>
       </c>
       <c r="C5" s="126" t="s">
-        <v>265</v>
+        <v>250</v>
       </c>
       <c r="D5" s="124" t="s">
-        <v>266</v>
+        <v>251</v>
       </c>
       <c r="E5" s="124">
         <v>87</v>
@@ -10405,63 +10107,69 @@
         <v>86</v>
       </c>
       <c r="G5" s="124" t="s">
-        <v>265</v>
-      </c>
-      <c r="H5" s="174">
+        <v>250</v>
+      </c>
+      <c r="H5" s="133">
         <v>46120</v>
       </c>
       <c r="I5" s="124">
         <v>87</v>
       </c>
       <c r="J5" s="124" t="s">
-        <v>267</v>
+        <v>252</v>
       </c>
       <c r="K5" s="124" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="125">
         <v>2</v>
       </c>
       <c r="B6" s="129" t="s">
-        <v>293</v>
-      </c>
-      <c r="C6" s="175">
+        <v>278</v>
+      </c>
+      <c r="C6" s="134">
         <v>46121</v>
       </c>
-      <c r="D6" s="174">
+      <c r="D6" s="133">
         <v>46127</v>
       </c>
       <c r="E6" s="124">
         <v>67</v>
       </c>
       <c r="F6" s="124" t="s">
-        <v>300</v>
-      </c>
-      <c r="G6" s="124"/>
-      <c r="H6" s="124"/>
-      <c r="I6" s="124"/>
+        <v>280</v>
+      </c>
+      <c r="G6" s="133">
+        <v>46121</v>
+      </c>
+      <c r="H6" s="133">
+        <v>46153</v>
+      </c>
+      <c r="I6" s="124">
+        <v>67</v>
+      </c>
       <c r="J6" s="124"/>
       <c r="K6" s="124" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="125">
         <v>3</v>
       </c>
       <c r="B7" s="129" t="s">
-        <v>299</v>
-      </c>
-      <c r="C7" s="175">
+        <v>281</v>
+      </c>
+      <c r="C7" s="134">
         <v>46128</v>
       </c>
-      <c r="D7" s="174">
+      <c r="D7" s="133">
         <v>46141</v>
       </c>
       <c r="E7" s="124">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F7" s="124" t="s">
         <v>87</v>
@@ -10471,24 +10179,24 @@
       <c r="I7" s="124"/>
       <c r="J7" s="124"/>
       <c r="K7" s="124" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="125">
         <v>4</v>
       </c>
       <c r="B8" s="129" t="s">
-        <v>298</v>
-      </c>
-      <c r="C8" s="175">
+        <v>282</v>
+      </c>
+      <c r="C8" s="134">
         <v>46142</v>
       </c>
-      <c r="D8" s="174">
+      <c r="D8" s="133">
         <v>46155</v>
       </c>
       <c r="E8" s="124">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>87</v>
@@ -10498,24 +10206,24 @@
       <c r="I8" s="124"/>
       <c r="J8" s="124"/>
       <c r="K8" s="124" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="125">
         <v>5</v>
       </c>
       <c r="B9" s="129" t="s">
-        <v>297</v>
-      </c>
-      <c r="C9" s="175">
+        <v>283</v>
+      </c>
+      <c r="C9" s="134">
         <v>46156</v>
       </c>
-      <c r="D9" s="174">
+      <c r="D9" s="133">
         <v>46169</v>
       </c>
       <c r="E9" s="124">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F9" s="124" t="s">
         <v>87</v>
@@ -10525,20 +10233,20 @@
       <c r="I9" s="124"/>
       <c r="J9" s="124"/>
       <c r="K9" s="124" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="125">
         <v>6</v>
       </c>
       <c r="B10" s="129" t="s">
-        <v>295</v>
-      </c>
-      <c r="C10" s="175">
+        <v>284</v>
+      </c>
+      <c r="C10" s="134">
         <v>46170</v>
       </c>
-      <c r="D10" s="174">
+      <c r="D10" s="133">
         <v>46183</v>
       </c>
       <c r="E10" s="124">
@@ -10552,51 +10260,51 @@
       <c r="I10" s="124"/>
       <c r="J10" s="124"/>
       <c r="K10" s="124" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="171">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="A11" s="130">
         <v>7</v>
       </c>
-      <c r="B11" s="172" t="s">
-        <v>296</v>
-      </c>
-      <c r="C11" s="176">
+      <c r="B11" s="131" t="s">
+        <v>285</v>
+      </c>
+      <c r="C11" s="135">
         <v>46184</v>
       </c>
-      <c r="D11" s="176">
+      <c r="D11" s="135">
         <v>46197</v>
       </c>
-      <c r="E11" s="173">
+      <c r="E11" s="132">
         <v>25</v>
       </c>
-      <c r="F11" s="173" t="s">
+      <c r="F11" s="132" t="s">
         <v>87</v>
       </c>
-      <c r="G11" s="173"/>
-      <c r="H11" s="173"/>
-      <c r="I11" s="173"/>
-      <c r="J11" s="173"/>
-      <c r="K11" s="173" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="G11" s="132"/>
+      <c r="H11" s="132"/>
+      <c r="I11" s="132"/>
+      <c r="J11" s="132"/>
+      <c r="K11" s="132" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="49"/>
       <c r="B12" s="128"/>
       <c r="C12" s="51"/>
       <c r="D12" s="50"/>
       <c r="E12" s="52">
         <f>SUM(E5:E11)</f>
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="F12" s="50"/>
       <c r="G12" s="53"/>
       <c r="H12" s="53"/>
       <c r="I12" s="52">
         <f>SUM(I5:I10)</f>
-        <v>87</v>
+        <v>154</v>
       </c>
       <c r="J12" s="54">
         <f>SUM(J5:J10)</f>
@@ -10604,7 +10312,7 @@
       </c>
       <c r="K12" s="53"/>
     </row>
-    <row r="13" spans="1:11" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="J13" s="19"/>
     </row>
   </sheetData>
@@ -10648,237 +10356,237 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{000B64FE-1B63-401C-B573-13BE1BFD24E2}">
   <dimension ref="A1:AMJ60"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.59765625" style="57" customWidth="1"/>
-    <col min="2" max="2" width="35.59765625" style="57" customWidth="1"/>
+    <col min="1" max="1" width="5.625" style="57" customWidth="1"/>
+    <col min="2" max="2" width="35.625" style="57" customWidth="1"/>
     <col min="3" max="3" width="6.5" style="57" customWidth="1"/>
-    <col min="4" max="4" width="13.19921875" style="57" customWidth="1"/>
-    <col min="5" max="5" width="8.8984375" style="57" customWidth="1"/>
+    <col min="4" max="4" width="13.25" style="57" customWidth="1"/>
+    <col min="5" max="5" width="8.875" style="57" customWidth="1"/>
     <col min="6" max="6" width="12.5" style="57" customWidth="1"/>
-    <col min="7" max="7" width="9.09765625" style="57" customWidth="1"/>
-    <col min="8" max="8" width="12.19921875" style="57" customWidth="1"/>
-    <col min="9" max="9" width="15.8984375" style="57" customWidth="1"/>
-    <col min="10" max="10" width="24.19921875" style="57" customWidth="1"/>
-    <col min="11" max="11" width="27.8984375" style="57" customWidth="1"/>
+    <col min="7" max="7" width="9.125" style="57" customWidth="1"/>
+    <col min="8" max="8" width="12.25" style="57" customWidth="1"/>
+    <col min="9" max="9" width="15.875" style="57" customWidth="1"/>
+    <col min="10" max="10" width="24.25" style="57" customWidth="1"/>
+    <col min="11" max="11" width="27.875" style="57" customWidth="1"/>
     <col min="12" max="12" width="8.5" style="57" customWidth="1"/>
     <col min="13" max="14" width="20.5" style="57" customWidth="1"/>
     <col min="15" max="256" width="8.5" style="57" customWidth="1"/>
     <col min="257" max="258" width="6.5" style="57" customWidth="1"/>
-    <col min="259" max="259" width="13.8984375" style="57" customWidth="1"/>
+    <col min="259" max="259" width="13.875" style="57" customWidth="1"/>
     <col min="260" max="260" width="9" style="57" customWidth="1"/>
     <col min="261" max="261" width="13.5" style="57" customWidth="1"/>
     <col min="262" max="262" width="10" style="57" customWidth="1"/>
-    <col min="263" max="263" width="12.19921875" style="57" customWidth="1"/>
-    <col min="264" max="264" width="5.8984375" style="57" customWidth="1"/>
-    <col min="265" max="265" width="24.19921875" style="57" customWidth="1"/>
+    <col min="263" max="263" width="12.25" style="57" customWidth="1"/>
+    <col min="264" max="264" width="5.875" style="57" customWidth="1"/>
+    <col min="265" max="265" width="24.25" style="57" customWidth="1"/>
     <col min="266" max="266" width="32.5" style="57" customWidth="1"/>
-    <col min="267" max="267" width="17.59765625" style="57" customWidth="1"/>
+    <col min="267" max="267" width="17.625" style="57" customWidth="1"/>
     <col min="268" max="268" width="8.5" style="57" customWidth="1"/>
     <col min="269" max="270" width="20.5" style="57" customWidth="1"/>
     <col min="271" max="512" width="8.5" style="57" customWidth="1"/>
     <col min="513" max="514" width="6.5" style="57" customWidth="1"/>
-    <col min="515" max="515" width="13.8984375" style="57" customWidth="1"/>
+    <col min="515" max="515" width="13.875" style="57" customWidth="1"/>
     <col min="516" max="516" width="9" style="57" customWidth="1"/>
     <col min="517" max="517" width="13.5" style="57" customWidth="1"/>
     <col min="518" max="518" width="10" style="57" customWidth="1"/>
-    <col min="519" max="519" width="12.19921875" style="57" customWidth="1"/>
-    <col min="520" max="520" width="5.8984375" style="57" customWidth="1"/>
-    <col min="521" max="521" width="24.19921875" style="57" customWidth="1"/>
+    <col min="519" max="519" width="12.25" style="57" customWidth="1"/>
+    <col min="520" max="520" width="5.875" style="57" customWidth="1"/>
+    <col min="521" max="521" width="24.25" style="57" customWidth="1"/>
     <col min="522" max="522" width="32.5" style="57" customWidth="1"/>
-    <col min="523" max="523" width="17.59765625" style="57" customWidth="1"/>
+    <col min="523" max="523" width="17.625" style="57" customWidth="1"/>
     <col min="524" max="524" width="8.5" style="57" customWidth="1"/>
     <col min="525" max="526" width="20.5" style="57" customWidth="1"/>
     <col min="527" max="768" width="8.5" style="57" customWidth="1"/>
     <col min="769" max="770" width="6.5" style="57" customWidth="1"/>
-    <col min="771" max="771" width="13.8984375" style="57" customWidth="1"/>
+    <col min="771" max="771" width="13.875" style="57" customWidth="1"/>
     <col min="772" max="772" width="9" style="57" customWidth="1"/>
     <col min="773" max="773" width="13.5" style="57" customWidth="1"/>
     <col min="774" max="774" width="10" style="57" customWidth="1"/>
-    <col min="775" max="775" width="12.19921875" style="57" customWidth="1"/>
-    <col min="776" max="776" width="5.8984375" style="57" customWidth="1"/>
-    <col min="777" max="777" width="24.19921875" style="57" customWidth="1"/>
+    <col min="775" max="775" width="12.25" style="57" customWidth="1"/>
+    <col min="776" max="776" width="5.875" style="57" customWidth="1"/>
+    <col min="777" max="777" width="24.25" style="57" customWidth="1"/>
     <col min="778" max="778" width="32.5" style="57" customWidth="1"/>
-    <col min="779" max="779" width="17.59765625" style="57" customWidth="1"/>
+    <col min="779" max="779" width="17.625" style="57" customWidth="1"/>
     <col min="780" max="780" width="8.5" style="57" customWidth="1"/>
     <col min="781" max="782" width="20.5" style="57" customWidth="1"/>
     <col min="783" max="1024" width="8.5" style="57" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="130" t="s">
+    <row r="1" spans="1:11" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="149" t="s">
         <v>88</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
-      <c r="F1" s="130"/>
-      <c r="G1" s="130"/>
-      <c r="H1" s="130"/>
-      <c r="I1" s="130"/>
-      <c r="J1" s="130"/>
-      <c r="K1" s="130"/>
-    </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="149"/>
+      <c r="C1" s="149"/>
+      <c r="D1" s="149"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+    </row>
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D3" s="58" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D4" s="59" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D5" s="59" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D6" s="59" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D7" s="59" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D8" s="59" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D9" s="59" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D10" s="59" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D11" s="59" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D12" s="59" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D13" s="59" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D14" s="58" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D15" s="59" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D16" s="59" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="17" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D17" s="59" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="18" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D18" s="58" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="19" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D19" s="59" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="20" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D20" s="59" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D21" s="59" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D22" s="58" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D23" s="59" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D24" s="59" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="25" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D25" s="59" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="26" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D26" s="59" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="27" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D27" s="58" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="28" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D28" s="59" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="29" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D29" s="59" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="30" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D30" s="59" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="31" spans="4:4" s="60" customFormat="1" ht="10.199999999999999" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="4:4" s="60" customFormat="1" ht="11.25" hidden="1" x14ac:dyDescent="0.2">
       <c r="D31" s="61" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="32" spans="4:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="4:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="D32" s="62" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="150" t="s">
+    <row r="33" spans="1:11" ht="22.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D33" s="162" t="s">
         <v>119</v>
       </c>
-      <c r="E33" s="150"/>
-    </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+      <c r="E33" s="162"/>
+    </row>
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D34" s="59">
         <v>4290</v>
       </c>
@@ -10886,7 +10594,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D35" s="59">
         <v>5082</v>
       </c>
@@ -10894,7 +10602,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D36" s="59">
         <v>4356</v>
       </c>
@@ -10902,7 +10610,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="22.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="D37" s="59">
         <v>5929</v>
       </c>
@@ -10910,7 +10618,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D38" s="59">
         <v>5005</v>
       </c>
@@ -10918,7 +10626,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.2">
       <c r="D39" s="59">
         <v>4225</v>
       </c>
@@ -10926,139 +10634,139 @@
         <v>125</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="151" t="s">
+    <row r="40" spans="1:11" ht="8.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="163" t="s">
         <v>126</v>
       </c>
-      <c r="B41" s="151"/>
-      <c r="C41" s="151"/>
-      <c r="D41" s="151"/>
-      <c r="E41" s="151"/>
-      <c r="F41" s="151"/>
-      <c r="G41" s="151"/>
-      <c r="H41" s="151"/>
-      <c r="I41" s="151"/>
-      <c r="J41" s="151"/>
-      <c r="K41" s="151"/>
-    </row>
-    <row r="42" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="152" t="s">
+      <c r="B41" s="163"/>
+      <c r="C41" s="163"/>
+      <c r="D41" s="163"/>
+      <c r="E41" s="163"/>
+      <c r="F41" s="163"/>
+      <c r="G41" s="163"/>
+      <c r="H41" s="163"/>
+      <c r="I41" s="163"/>
+      <c r="J41" s="163"/>
+      <c r="K41" s="163"/>
+    </row>
+    <row r="42" spans="1:11" s="56" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="164" t="s">
         <v>127</v>
       </c>
-      <c r="B42" s="152"/>
-      <c r="C42" s="152"/>
-      <c r="D42" s="152"/>
-      <c r="E42" s="152"/>
-      <c r="F42" s="152"/>
-      <c r="G42" s="152"/>
-      <c r="H42" s="152"/>
-      <c r="I42" s="152"/>
-      <c r="J42" s="152"/>
-      <c r="K42" s="152"/>
-    </row>
-    <row r="43" spans="1:11" s="56" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="153" t="s">
+      <c r="B42" s="164"/>
+      <c r="C42" s="164"/>
+      <c r="D42" s="164"/>
+      <c r="E42" s="164"/>
+      <c r="F42" s="164"/>
+      <c r="G42" s="164"/>
+      <c r="H42" s="164"/>
+      <c r="I42" s="164"/>
+      <c r="J42" s="164"/>
+      <c r="K42" s="164"/>
+    </row>
+    <row r="43" spans="1:11" s="56" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="165" t="s">
         <v>128</v>
       </c>
-      <c r="B43" s="153"/>
-      <c r="C43" s="153"/>
-      <c r="D43" s="153"/>
-      <c r="E43" s="153"/>
-      <c r="F43" s="153"/>
-      <c r="G43" s="153"/>
-      <c r="H43" s="153"/>
-      <c r="I43" s="153"/>
-      <c r="J43" s="153"/>
-      <c r="K43" s="153"/>
-    </row>
-    <row r="44" spans="1:11" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="149" t="s">
+      <c r="B43" s="165"/>
+      <c r="C43" s="165"/>
+      <c r="D43" s="165"/>
+      <c r="E43" s="165"/>
+      <c r="F43" s="165"/>
+      <c r="G43" s="165"/>
+      <c r="H43" s="165"/>
+      <c r="I43" s="165"/>
+      <c r="J43" s="165"/>
+      <c r="K43" s="165"/>
+    </row>
+    <row r="44" spans="1:11" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="161" t="s">
         <v>129</v>
       </c>
-      <c r="B44" s="149"/>
-      <c r="C44" s="149"/>
-      <c r="D44" s="149"/>
-      <c r="E44" s="149"/>
-      <c r="F44" s="149"/>
-      <c r="G44" s="149"/>
-      <c r="H44" s="149"/>
-      <c r="I44" s="149"/>
-      <c r="J44" s="149"/>
-      <c r="K44" s="149"/>
-    </row>
-    <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46" s="157" t="s">
+      <c r="B44" s="161"/>
+      <c r="C44" s="161"/>
+      <c r="D44" s="161"/>
+      <c r="E44" s="161"/>
+      <c r="F44" s="161"/>
+      <c r="G44" s="161"/>
+      <c r="H44" s="161"/>
+      <c r="I44" s="161"/>
+      <c r="J44" s="161"/>
+      <c r="K44" s="161"/>
+    </row>
+    <row r="45" spans="1:11" ht="9" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:11" ht="15" x14ac:dyDescent="0.25">
+      <c r="A46" s="154" t="s">
         <v>130</v>
       </c>
-      <c r="B46" s="157"/>
-      <c r="C46" s="157"/>
-      <c r="D46" s="157"/>
-      <c r="E46" s="157"/>
-      <c r="F46" s="157"/>
-      <c r="G46" s="157"/>
-      <c r="H46" s="157"/>
-      <c r="I46" s="157"/>
-      <c r="J46" s="157"/>
-      <c r="K46" s="157"/>
-    </row>
-    <row r="47" spans="1:11" s="65" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="154"/>
+      <c r="C46" s="154"/>
+      <c r="D46" s="154"/>
+      <c r="E46" s="154"/>
+      <c r="F46" s="154"/>
+      <c r="G46" s="154"/>
+      <c r="H46" s="154"/>
+      <c r="I46" s="154"/>
+      <c r="J46" s="154"/>
+      <c r="K46" s="154"/>
+    </row>
+    <row r="47" spans="1:11" s="65" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="63" t="s">
         <v>131</v>
       </c>
       <c r="B47" s="64"/>
-      <c r="C47" s="158" t="s">
+      <c r="C47" s="155" t="s">
         <v>132</v>
       </c>
-      <c r="D47" s="158"/>
-      <c r="E47" s="158"/>
-      <c r="F47" s="158"/>
-      <c r="G47" s="158"/>
-      <c r="H47" s="158"/>
-      <c r="I47" s="158"/>
-      <c r="J47" s="158"/>
-      <c r="K47" s="158"/>
-    </row>
-    <row r="48" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="159"/>
-      <c r="B48" s="154" t="s">
+      <c r="D47" s="155"/>
+      <c r="E47" s="155"/>
+      <c r="F47" s="155"/>
+      <c r="G47" s="155"/>
+      <c r="H47" s="155"/>
+      <c r="I47" s="155"/>
+      <c r="J47" s="155"/>
+      <c r="K47" s="155"/>
+    </row>
+    <row r="48" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="156"/>
+      <c r="B48" s="157" t="s">
         <v>133</v>
       </c>
-      <c r="C48" s="154" t="s">
+      <c r="C48" s="157" t="s">
         <v>134</v>
       </c>
-      <c r="D48" s="154" t="s">
+      <c r="D48" s="157" t="s">
         <v>135</v>
       </c>
-      <c r="E48" s="154" t="s">
+      <c r="E48" s="157" t="s">
         <v>104</v>
       </c>
-      <c r="F48" s="154" t="s">
+      <c r="F48" s="157" t="s">
         <v>136</v>
       </c>
-      <c r="G48" s="154" t="s">
+      <c r="G48" s="157" t="s">
         <v>108</v>
       </c>
-      <c r="H48" s="160" t="s">
+      <c r="H48" s="158" t="s">
         <v>137</v>
       </c>
-      <c r="I48" s="160"/>
-      <c r="J48" s="160"/>
-      <c r="K48" s="160"/>
-    </row>
-    <row r="49" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="159"/>
-      <c r="B49" s="154"/>
-      <c r="C49" s="154"/>
-      <c r="D49" s="154"/>
-      <c r="E49" s="154"/>
-      <c r="F49" s="154"/>
-      <c r="G49" s="154"/>
-      <c r="H49" s="154" t="s">
+      <c r="I48" s="158"/>
+      <c r="J48" s="158"/>
+      <c r="K48" s="158"/>
+    </row>
+    <row r="49" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="156"/>
+      <c r="B49" s="157"/>
+      <c r="C49" s="157"/>
+      <c r="D49" s="157"/>
+      <c r="E49" s="157"/>
+      <c r="F49" s="157"/>
+      <c r="G49" s="157"/>
+      <c r="H49" s="157" t="s">
         <v>138</v>
       </c>
-      <c r="I49" s="154"/>
+      <c r="I49" s="157"/>
       <c r="J49" s="66" t="s">
         <v>139</v>
       </c>
@@ -11071,7 +10779,7 @@
         <v>1</v>
       </c>
       <c r="B50" s="69" t="s">
-        <v>273</v>
+        <v>258</v>
       </c>
       <c r="C50" s="70">
         <v>46117</v>
@@ -11089,23 +10797,23 @@
       <c r="G50" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="H50" s="155" t="s">
-        <v>274</v>
-      </c>
-      <c r="I50" s="155"/>
+      <c r="H50" s="166" t="s">
+        <v>259</v>
+      </c>
+      <c r="I50" s="166"/>
       <c r="J50" s="73" t="s">
-        <v>275</v>
+        <v>260</v>
       </c>
       <c r="K50" s="73" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" s="67" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.25">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" s="67" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A51" s="68">
         <v>2</v>
       </c>
       <c r="B51" s="69" t="s">
-        <v>277</v>
+        <v>262</v>
       </c>
       <c r="C51" s="70">
         <v>46117</v>
@@ -11123,23 +10831,23 @@
       <c r="G51" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="H51" s="147" t="s">
-        <v>278</v>
-      </c>
-      <c r="I51" s="148"/>
+      <c r="H51" s="159" t="s">
+        <v>263</v>
+      </c>
+      <c r="I51" s="160"/>
       <c r="J51" s="73" t="s">
-        <v>279</v>
+        <v>264</v>
       </c>
       <c r="K51" s="73" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" s="67" customFormat="1" ht="40.799999999999997" x14ac:dyDescent="0.25">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" s="67" customFormat="1" ht="45" x14ac:dyDescent="0.2">
       <c r="A52" s="68">
         <v>3</v>
       </c>
       <c r="B52" s="69" t="s">
-        <v>281</v>
+        <v>266</v>
       </c>
       <c r="C52" s="70">
         <v>46117</v>
@@ -11157,23 +10865,23 @@
       <c r="G52" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="H52" s="147" t="s">
-        <v>282</v>
-      </c>
-      <c r="I52" s="148"/>
+      <c r="H52" s="159" t="s">
+        <v>267</v>
+      </c>
+      <c r="I52" s="160"/>
       <c r="J52" s="73" t="s">
-        <v>283</v>
+        <v>268</v>
       </c>
       <c r="K52" s="73" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" s="67" customFormat="1" ht="30.6" x14ac:dyDescent="0.25">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" s="67" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A53" s="68">
         <v>4</v>
       </c>
       <c r="B53" s="69" t="s">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="C53" s="70">
         <v>46117</v>
@@ -11191,23 +10899,23 @@
       <c r="G53" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="H53" s="147" t="s">
-        <v>286</v>
-      </c>
-      <c r="I53" s="148"/>
+      <c r="H53" s="159" t="s">
+        <v>271</v>
+      </c>
+      <c r="I53" s="160"/>
       <c r="J53" s="73" t="s">
-        <v>287</v>
+        <v>272</v>
       </c>
       <c r="K53" s="73" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" s="67" customFormat="1" ht="30.6" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" s="67" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
       <c r="A54" s="68">
         <v>5</v>
       </c>
       <c r="B54" s="69" t="s">
-        <v>289</v>
+        <v>274</v>
       </c>
       <c r="C54" s="70">
         <v>46117</v>
@@ -11225,18 +10933,18 @@
       <c r="G54" s="71" t="s">
         <v>109</v>
       </c>
-      <c r="H54" s="147" t="s">
-        <v>290</v>
-      </c>
-      <c r="I54" s="148"/>
+      <c r="H54" s="159" t="s">
+        <v>275</v>
+      </c>
+      <c r="I54" s="160"/>
       <c r="J54" s="73" t="s">
-        <v>291</v>
+        <v>276</v>
       </c>
       <c r="K54" s="73" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="68"/>
       <c r="B55" s="69"/>
       <c r="C55" s="70"/>
@@ -11252,7 +10960,7 @@
       <c r="J55" s="73"/>
       <c r="K55" s="73"/>
     </row>
-    <row r="56" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="68"/>
       <c r="B56" s="69"/>
       <c r="C56" s="70"/>
@@ -11268,7 +10976,7 @@
       <c r="J56" s="73"/>
       <c r="K56" s="73"/>
     </row>
-    <row r="57" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="68"/>
       <c r="B57" s="69"/>
       <c r="C57" s="70"/>
@@ -11284,7 +10992,7 @@
       <c r="J57" s="73"/>
       <c r="K57" s="73"/>
     </row>
-    <row r="58" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="68"/>
       <c r="B58" s="69"/>
       <c r="C58" s="70"/>
@@ -11300,7 +11008,7 @@
       <c r="J58" s="73"/>
       <c r="K58" s="73"/>
     </row>
-    <row r="59" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="68"/>
       <c r="B59" s="69"/>
       <c r="C59" s="70"/>
@@ -11311,12 +11019,12 @@
         <v>#VALUE!</v>
       </c>
       <c r="G59" s="71"/>
-      <c r="H59" s="156"/>
-      <c r="I59" s="156"/>
+      <c r="H59" s="153"/>
+      <c r="I59" s="153"/>
       <c r="J59" s="73"/>
       <c r="K59" s="73"/>
     </row>
-    <row r="60" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" s="67" customFormat="1" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="68"/>
       <c r="B60" s="69"/>
       <c r="C60" s="70"/>
@@ -11327,13 +11035,21 @@
         <v>#VALUE!</v>
       </c>
       <c r="G60" s="71"/>
-      <c r="H60" s="156"/>
-      <c r="I60" s="156"/>
+      <c r="H60" s="153"/>
+      <c r="I60" s="153"/>
       <c r="J60" s="73"/>
       <c r="K60" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="H49:I49"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
+    <mergeCell ref="A43:K43"/>
     <mergeCell ref="H59:I59"/>
     <mergeCell ref="H60:I60"/>
     <mergeCell ref="A46:K46"/>
@@ -11350,14 +11066,6 @@
     <mergeCell ref="H52:I52"/>
     <mergeCell ref="H53:I53"/>
     <mergeCell ref="H54:I54"/>
-    <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
-    <mergeCell ref="A43:K43"/>
-    <mergeCell ref="H49:I49"/>
-    <mergeCell ref="H50:I50"/>
   </mergeCells>
   <conditionalFormatting sqref="F50:F60">
     <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="equal">
@@ -11394,139 +11102,139 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFDDF7CC-49D1-41E6-88FF-D333F1DE112D}">
   <dimension ref="A1:AMJ27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.09765625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.69921875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="0.8984375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.09765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.69921875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="1.09765625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.3984375" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.75" style="1" customWidth="1"/>
+    <col min="3" max="3" width="0.875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28.125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.75" style="1" customWidth="1"/>
+    <col min="6" max="6" width="1.125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.375" style="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="1" customWidth="1"/>
     <col min="9" max="9" width="5.5" style="1" customWidth="1"/>
     <col min="10" max="10" width="8.5" style="1" customWidth="1"/>
     <col min="11" max="11" width="10.5" style="1" customWidth="1"/>
-    <col min="12" max="12" width="1.3984375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="37.3984375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="1.375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="37.375" style="1" customWidth="1"/>
     <col min="14" max="14" width="10" style="1" customWidth="1"/>
-    <col min="15" max="1024" width="8.09765625" style="1" customWidth="1"/>
+    <col min="15" max="1024" width="8.125" style="1" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="163" t="s">
+    <row r="1" spans="1:23" s="56" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="169" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="163"/>
-      <c r="C1" s="163"/>
-      <c r="D1" s="163"/>
-      <c r="E1" s="163"/>
-      <c r="F1" s="163"/>
-      <c r="G1" s="163"/>
-      <c r="H1" s="163"/>
-      <c r="I1" s="163"/>
-      <c r="J1" s="163"/>
-      <c r="K1" s="163"/>
-      <c r="L1" s="163"/>
-      <c r="M1" s="163"/>
-      <c r="N1" s="163"/>
-    </row>
-    <row r="2" spans="1:23" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="164" t="s">
+      <c r="B1" s="169"/>
+      <c r="C1" s="169"/>
+      <c r="D1" s="169"/>
+      <c r="E1" s="169"/>
+      <c r="F1" s="169"/>
+      <c r="G1" s="169"/>
+      <c r="H1" s="169"/>
+      <c r="I1" s="169"/>
+      <c r="J1" s="169"/>
+      <c r="K1" s="169"/>
+      <c r="L1" s="169"/>
+      <c r="M1" s="169"/>
+      <c r="N1" s="169"/>
+    </row>
+    <row r="2" spans="1:23" s="76" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="170" t="s">
         <v>126</v>
       </c>
-      <c r="B2" s="164"/>
-      <c r="C2" s="164"/>
-      <c r="D2" s="164"/>
-      <c r="E2" s="164"/>
-      <c r="F2" s="164"/>
-      <c r="G2" s="164"/>
-      <c r="H2" s="164"/>
-      <c r="I2" s="164"/>
-      <c r="J2" s="164"/>
-      <c r="K2" s="164"/>
-      <c r="L2" s="164"/>
-      <c r="M2" s="164"/>
-      <c r="N2" s="164"/>
-    </row>
-    <row r="3" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="165" t="s">
+      <c r="B2" s="170"/>
+      <c r="C2" s="170"/>
+      <c r="D2" s="170"/>
+      <c r="E2" s="170"/>
+      <c r="F2" s="170"/>
+      <c r="G2" s="170"/>
+      <c r="H2" s="170"/>
+      <c r="I2" s="170"/>
+      <c r="J2" s="170"/>
+      <c r="K2" s="170"/>
+      <c r="L2" s="170"/>
+      <c r="M2" s="170"/>
+      <c r="N2" s="170"/>
+    </row>
+    <row r="3" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="171" t="s">
         <v>142</v>
       </c>
-      <c r="B3" s="165"/>
-      <c r="C3" s="165"/>
-      <c r="D3" s="165"/>
-      <c r="E3" s="165"/>
-      <c r="F3" s="165"/>
-      <c r="G3" s="165"/>
-      <c r="H3" s="165"/>
-      <c r="I3" s="165"/>
-      <c r="J3" s="165"/>
-      <c r="K3" s="165"/>
-      <c r="L3" s="165"/>
-      <c r="M3" s="165"/>
-      <c r="N3" s="165"/>
-    </row>
-    <row r="4" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="166" t="s">
+      <c r="B3" s="171"/>
+      <c r="C3" s="171"/>
+      <c r="D3" s="171"/>
+      <c r="E3" s="171"/>
+      <c r="F3" s="171"/>
+      <c r="G3" s="171"/>
+      <c r="H3" s="171"/>
+      <c r="I3" s="171"/>
+      <c r="J3" s="171"/>
+      <c r="K3" s="171"/>
+      <c r="L3" s="171"/>
+      <c r="M3" s="171"/>
+      <c r="N3" s="171"/>
+    </row>
+    <row r="4" spans="1:23" s="76" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="172" t="s">
         <v>143</v>
       </c>
-      <c r="B4" s="166"/>
-      <c r="C4" s="166"/>
-      <c r="D4" s="166"/>
-      <c r="E4" s="166"/>
-      <c r="F4" s="166"/>
-      <c r="G4" s="166"/>
-      <c r="H4" s="166"/>
-      <c r="I4" s="166"/>
-      <c r="J4" s="166"/>
-      <c r="K4" s="166"/>
-      <c r="L4" s="166"/>
-      <c r="M4" s="166"/>
-      <c r="N4" s="166"/>
-    </row>
-    <row r="5" spans="1:23" s="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="167" t="s">
+      <c r="B4" s="172"/>
+      <c r="C4" s="172"/>
+      <c r="D4" s="172"/>
+      <c r="E4" s="172"/>
+      <c r="F4" s="172"/>
+      <c r="G4" s="172"/>
+      <c r="H4" s="172"/>
+      <c r="I4" s="172"/>
+      <c r="J4" s="172"/>
+      <c r="K4" s="172"/>
+      <c r="L4" s="172"/>
+      <c r="M4" s="172"/>
+      <c r="N4" s="172"/>
+    </row>
+    <row r="5" spans="1:23" s="76" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="173" t="s">
         <v>144</v>
       </c>
-      <c r="B5" s="167"/>
-      <c r="C5" s="167"/>
-      <c r="D5" s="167"/>
-      <c r="E5" s="167"/>
-      <c r="F5" s="167"/>
-      <c r="G5" s="167"/>
-      <c r="H5" s="167"/>
-      <c r="I5" s="167"/>
-      <c r="J5" s="167"/>
-      <c r="K5" s="167"/>
-      <c r="L5" s="167"/>
-      <c r="M5" s="167"/>
-      <c r="N5" s="167"/>
-    </row>
-    <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="161" t="s">
+      <c r="B5" s="173"/>
+      <c r="C5" s="173"/>
+      <c r="D5" s="173"/>
+      <c r="E5" s="173"/>
+      <c r="F5" s="173"/>
+      <c r="G5" s="173"/>
+      <c r="H5" s="173"/>
+      <c r="I5" s="173"/>
+      <c r="J5" s="173"/>
+      <c r="K5" s="173"/>
+      <c r="L5" s="173"/>
+      <c r="M5" s="173"/>
+      <c r="N5" s="173"/>
+    </row>
+    <row r="6" spans="1:23" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="7" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="167" t="s">
         <v>145</v>
       </c>
-      <c r="B7" s="161"/>
-      <c r="D7" s="161" t="s">
+      <c r="B7" s="167"/>
+      <c r="D7" s="167" t="s">
         <v>146</v>
       </c>
-      <c r="E7" s="161"/>
-      <c r="G7" s="161" t="s">
+      <c r="E7" s="167"/>
+      <c r="G7" s="167" t="s">
         <v>147</v>
       </c>
-      <c r="H7" s="161"/>
-      <c r="I7" s="161"/>
-      <c r="J7" s="161"/>
-      <c r="K7" s="161"/>
-      <c r="M7" s="161" t="s">
+      <c r="H7" s="167"/>
+      <c r="I7" s="167"/>
+      <c r="J7" s="167"/>
+      <c r="K7" s="167"/>
+      <c r="M7" s="167" t="s">
         <v>148</v>
       </c>
-      <c r="N7" s="161"/>
-    </row>
-    <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N7" s="167"/>
+    </row>
+    <row r="8" spans="1:23" s="4" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="79" t="s">
         <v>149</v>
       </c>
@@ -11561,7 +11269,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="9" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A9" s="77" t="s">
         <v>158</v>
       </c>
@@ -11595,7 +11303,7 @@
       </c>
       <c r="N9" s="82"/>
     </row>
-    <row r="10" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A10" s="77" t="s">
         <v>162</v>
       </c>
@@ -11619,24 +11327,24 @@
       </c>
       <c r="N10" s="82"/>
     </row>
-    <row r="11" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="77"/>
       <c r="B11" s="78"/>
       <c r="D11" s="77"/>
       <c r="E11" s="78"/>
-      <c r="G11" s="161" t="s">
+      <c r="G11" s="167" t="s">
         <v>165</v>
       </c>
-      <c r="H11" s="161"/>
-      <c r="I11" s="161"/>
-      <c r="J11" s="161"/>
-      <c r="K11" s="161"/>
+      <c r="H11" s="167"/>
+      <c r="I11" s="167"/>
+      <c r="J11" s="167"/>
+      <c r="K11" s="167"/>
       <c r="M11" s="81" t="s">
         <v>166</v>
       </c>
       <c r="N11" s="82"/>
     </row>
-    <row r="12" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A12" s="77"/>
       <c r="B12" s="78"/>
       <c r="D12" s="77"/>
@@ -11661,7 +11369,7 @@
       </c>
       <c r="N12" s="82"/>
     </row>
-    <row r="13" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A13" s="77"/>
       <c r="B13" s="78"/>
       <c r="D13" s="77"/>
@@ -11686,7 +11394,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A14" s="77"/>
       <c r="B14" s="78"/>
       <c r="D14" s="77"/>
@@ -11706,7 +11414,7 @@
       </c>
       <c r="N14" s="82"/>
     </row>
-    <row r="15" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A15" s="77"/>
       <c r="B15" s="78"/>
       <c r="D15" s="77"/>
@@ -11728,17 +11436,17 @@
       </c>
       <c r="N15" s="82"/>
     </row>
-    <row r="16" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:23" s="4" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="77"/>
       <c r="B16" s="78"/>
       <c r="D16" s="77"/>
       <c r="E16" s="78"/>
-      <c r="G16" s="162" t="s">
+      <c r="G16" s="168" t="s">
         <v>175</v>
       </c>
-      <c r="H16" s="162"/>
-      <c r="I16" s="162"/>
-      <c r="J16" s="162"/>
+      <c r="H16" s="168"/>
+      <c r="I16" s="168"/>
+      <c r="J16" s="168"/>
       <c r="K16" s="83">
         <f>SUM(K9,K10,K13,K14,K15)</f>
         <v>14</v>
@@ -11748,7 +11456,7 @@
       </c>
       <c r="N16" s="82"/>
     </row>
-    <row r="17" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A17" s="77"/>
       <c r="B17" s="78"/>
       <c r="D17" s="77"/>
@@ -11758,7 +11466,7 @@
       </c>
       <c r="N17" s="82"/>
     </row>
-    <row r="18" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A18" s="77"/>
       <c r="B18" s="78"/>
       <c r="D18" s="77"/>
@@ -11768,7 +11476,7 @@
       </c>
       <c r="N18" s="82"/>
     </row>
-    <row r="19" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A19" s="77"/>
       <c r="B19" s="78"/>
       <c r="D19" s="77"/>
@@ -11778,7 +11486,7 @@
       </c>
       <c r="N19" s="82"/>
     </row>
-    <row r="20" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="A20" s="77"/>
       <c r="B20" s="78"/>
       <c r="D20" s="77"/>
@@ -11788,19 +11496,19 @@
       </c>
       <c r="N20" s="82"/>
     </row>
-    <row r="21" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="M21" s="81" t="s">
         <v>181</v>
       </c>
       <c r="N21" s="82"/>
     </row>
-    <row r="22" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="M22" s="81" t="s">
         <v>182</v>
       </c>
       <c r="N22" s="82"/>
     </row>
-    <row r="23" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" s="4" customFormat="1" ht="12" x14ac:dyDescent="0.2">
       <c r="M23" s="84" t="s">
         <v>183</v>
       </c>
@@ -11809,7 +11517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="M24" s="84" t="s">
         <v>184</v>
       </c>
@@ -11818,7 +11526,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="M25" s="84" t="s">
         <v>185</v>
       </c>
@@ -11827,7 +11535,7 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="M26" s="84" t="s">
         <v>186</v>
       </c>
@@ -11835,7 +11543,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" ht="21" x14ac:dyDescent="0.25">
       <c r="M27" s="88" t="s">
         <v>187</v>
       </c>
@@ -11877,65 +11585,65 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{389CB43A-5794-4661-ACA8-D26510321904}">
   <dimension ref="A1:AMJ29"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="45.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.59765625" style="21" customWidth="1"/>
-    <col min="3" max="3" width="12.69921875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="1.09765625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.8984375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="6.69921875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.625" style="21" customWidth="1"/>
+    <col min="3" max="3" width="12.75" style="1" customWidth="1"/>
+    <col min="4" max="4" width="1.125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="24.875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="6.75" style="1" customWidth="1"/>
     <col min="7" max="7" width="7" style="1" customWidth="1"/>
     <col min="8" max="8" width="6.5" style="1" customWidth="1"/>
     <col min="9" max="9" width="7" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10.09765625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="10.125" style="1" customWidth="1"/>
     <col min="11" max="11" width="7" style="1" customWidth="1"/>
-    <col min="12" max="12" width="7.59765625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="7.625" style="1" customWidth="1"/>
     <col min="13" max="13" width="7" style="1" customWidth="1"/>
-    <col min="14" max="14" width="19.09765625" style="1" customWidth="1"/>
-    <col min="15" max="1024" width="8.09765625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="19.125" style="1" customWidth="1"/>
+    <col min="15" max="1024" width="8.125" style="1" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="163" t="s">
+    <row r="1" spans="1:14" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="169" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="163"/>
-      <c r="C1" s="163"/>
-      <c r="D1" s="163"/>
-      <c r="E1" s="163"/>
-      <c r="F1" s="163"/>
-      <c r="G1" s="163"/>
-      <c r="H1" s="163"/>
-      <c r="I1" s="163"/>
-      <c r="J1" s="163"/>
-      <c r="K1" s="163"/>
-      <c r="L1" s="163"/>
-      <c r="M1" s="163"/>
-      <c r="N1" s="163"/>
-    </row>
-    <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="169" t="s">
+      <c r="B1" s="169"/>
+      <c r="C1" s="169"/>
+      <c r="D1" s="169"/>
+      <c r="E1" s="169"/>
+      <c r="F1" s="169"/>
+      <c r="G1" s="169"/>
+      <c r="H1" s="169"/>
+      <c r="I1" s="169"/>
+      <c r="J1" s="169"/>
+      <c r="K1" s="169"/>
+      <c r="L1" s="169"/>
+      <c r="M1" s="169"/>
+      <c r="N1" s="169"/>
+    </row>
+    <row r="2" spans="1:14" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="175" t="s">
         <v>49</v>
       </c>
-      <c r="B3" s="169"/>
-      <c r="C3" s="169"/>
-      <c r="E3" s="169" t="s">
+      <c r="B3" s="175"/>
+      <c r="C3" s="175"/>
+      <c r="E3" s="175" t="s">
         <v>188</v>
       </c>
-      <c r="F3" s="169"/>
-      <c r="G3" s="169"/>
-      <c r="H3" s="169"/>
-      <c r="I3" s="169"/>
-      <c r="J3" s="169"/>
-      <c r="K3" s="169"/>
-      <c r="L3" s="169"/>
-      <c r="M3" s="169"/>
-      <c r="N3" s="169"/>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="F3" s="175"/>
+      <c r="G3" s="175"/>
+      <c r="H3" s="175"/>
+      <c r="I3" s="175"/>
+      <c r="J3" s="175"/>
+      <c r="K3" s="175"/>
+      <c r="L3" s="175"/>
+      <c r="M3" s="175"/>
+      <c r="N3" s="175"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="90" t="s">
         <v>189</v>
       </c>
@@ -11946,28 +11654,28 @@
       <c r="C4" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="170" t="s">
+      <c r="E4" s="176" t="s">
         <v>190</v>
       </c>
-      <c r="F4" s="168" t="s">
+      <c r="F4" s="174" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="168"/>
-      <c r="H4" s="168" t="s">
+      <c r="G4" s="174"/>
+      <c r="H4" s="174" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="168"/>
-      <c r="J4" s="168" t="s">
+      <c r="I4" s="174"/>
+      <c r="J4" s="174" t="s">
         <v>39</v>
       </c>
-      <c r="K4" s="168"/>
-      <c r="L4" s="168" t="s">
+      <c r="K4" s="174"/>
+      <c r="L4" s="174" t="s">
         <v>40</v>
       </c>
-      <c r="M4" s="168"/>
+      <c r="M4" s="174"/>
       <c r="N4" s="92"/>
     </row>
-    <row r="5" spans="1:14" ht="18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
         <v>52</v>
       </c>
@@ -11977,28 +11685,28 @@
       <c r="C5" s="34" t="s">
         <v>191</v>
       </c>
-      <c r="E5" s="170"/>
-      <c r="F5" s="168" t="s">
+      <c r="E5" s="176"/>
+      <c r="F5" s="174" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="168"/>
-      <c r="H5" s="168" t="s">
+      <c r="G5" s="174"/>
+      <c r="H5" s="174" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="168"/>
-      <c r="J5" s="168" t="s">
+      <c r="I5" s="174"/>
+      <c r="J5" s="174" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="168"/>
-      <c r="L5" s="168" t="s">
+      <c r="K5" s="174"/>
+      <c r="L5" s="174" t="s">
         <v>17</v>
       </c>
-      <c r="M5" s="168"/>
+      <c r="M5" s="174"/>
       <c r="N5" s="37" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="93" t="s">
         <v>193</v>
       </c>
@@ -12009,7 +11717,7 @@
       <c r="C6" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="170"/>
+      <c r="E6" s="176"/>
       <c r="F6" s="95">
         <f>B6*G6</f>
         <v>8.6450000000000014</v>
@@ -12040,7 +11748,7 @@
       </c>
       <c r="N6" s="95"/>
     </row>
-    <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>194</v>
       </c>
@@ -12084,7 +11792,7 @@
         <v>29.47945</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
         <v>196</v>
       </c>
@@ -12130,7 +11838,7 @@
         <v>20.315750000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
         <v>199</v>
       </c>
@@ -12176,7 +11884,7 @@
         <v>54.636400000000009</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="99" t="s">
         <v>201</v>
       </c>
@@ -12223,7 +11931,7 @@
         <v>16.166150000000002</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="90" t="s">
         <v>203</v>
       </c>
@@ -12270,7 +11978,7 @@
         <v>8.0398500000000013</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="90" t="s">
         <v>205</v>
       </c>
@@ -12318,7 +12026,7 @@
       </c>
       <c r="N12" s="102"/>
     </row>
-    <row r="13" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="99" t="s">
         <v>207</v>
       </c>
@@ -12365,7 +12073,7 @@
         <v>22.822800000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="E14" s="97" t="s">
         <v>210</v>
       </c>
@@ -12402,7 +12110,7 @@
         <v>21.439600000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E15" s="102" t="s">
         <v>211</v>
       </c>
@@ -12440,12 +12148,12 @@
       </c>
       <c r="N15" s="102"/>
     </row>
-    <row r="16" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A16" s="169" t="s">
+    <row r="16" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A16" s="175" t="s">
         <v>65</v>
       </c>
-      <c r="B16" s="169"/>
-      <c r="C16" s="169"/>
+      <c r="B16" s="175"/>
+      <c r="C16" s="175"/>
       <c r="E16" s="37" t="s">
         <v>212</v>
       </c>
@@ -12486,7 +12194,7 @@
         <v>172.90000000000003</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
         <v>66</v>
       </c>
@@ -12496,7 +12204,7 @@
       <c r="C17" s="34"/>
       <c r="N17" s="53"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
         <v>67</v>
       </c>
@@ -12508,7 +12216,7 @@
       <c r="L18" s="53"/>
       <c r="N18" s="53"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
         <v>68</v>
       </c>
@@ -12518,7 +12226,7 @@
       <c r="C19" s="34"/>
       <c r="N19" s="53"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
         <v>69</v>
       </c>
@@ -12530,7 +12238,7 @@
       <c r="L20" s="53"/>
       <c r="N20" s="53"/>
     </row>
-    <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
         <v>213</v>
       </c>
@@ -12541,7 +12249,7 @@
       <c r="C21" s="34"/>
       <c r="N21" s="53"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="26" t="s">
         <v>71</v>
       </c>
@@ -12551,7 +12259,7 @@
       <c r="C22" s="34"/>
       <c r="J22" s="53"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="26" t="s">
         <v>72</v>
       </c>
@@ -12561,7 +12269,7 @@
       </c>
       <c r="C23" s="34"/>
     </row>
-    <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="22" t="s">
         <v>214</v>
       </c>
@@ -12571,16 +12279,16 @@
       </c>
       <c r="C24" s="34"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J26" s="53"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J27" s="53"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N28" s="53"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N29" s="53"/>
     </row>
   </sheetData>

</xml_diff>